<commit_message>
Add temporary file for individual annotations of Oscar Andres Rincon Cardeño
</commit_message>
<xml_diff>
--- a/main/04_data_extraction/Individual AnnotationsORC.xlsx
+++ b/main/04_data_extraction/Individual AnnotationsORC.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\orincon\scoping-ml-wave-seismology\main\04_data_extraction\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4ABAF4DA-C250-4EA8-9E9E-06457612B994}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{85D38A46-7185-47F3-8BEC-678E23D57EEC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{115BB8D9-8B86-4726-97F8-E06477FD353D}"/>
   </bookViews>
@@ -1723,15 +1723,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1758,16 +1755,16 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -2114,52 +2111,52 @@
   <dimension ref="A1:P46"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.09765625" defaultRowHeight="13.2"/>
   <cols>
-    <col min="1" max="1" width="36.59765625" style="6" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="39.296875" style="6" customWidth="1"/>
-    <col min="3" max="3" width="36.59765625" style="6" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="24.8984375" style="6" customWidth="1"/>
-    <col min="5" max="8" width="36.59765625" style="6" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="35.69921875" style="6" bestFit="1" customWidth="1"/>
-    <col min="10" max="15" width="36.59765625" style="6" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="32.296875" style="6" bestFit="1" customWidth="1"/>
-    <col min="17" max="16384" width="9.09765625" style="6"/>
+    <col min="1" max="1" width="36.59765625" style="5" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="39.296875" style="5" customWidth="1"/>
+    <col min="3" max="3" width="36.59765625" style="5" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="24.8984375" style="5" customWidth="1"/>
+    <col min="5" max="8" width="36.59765625" style="5" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="35.69921875" style="5" bestFit="1" customWidth="1"/>
+    <col min="10" max="15" width="36.59765625" style="5" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="32.296875" style="5" bestFit="1" customWidth="1"/>
+    <col min="17" max="16384" width="9.09765625" style="5"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:16" ht="15" customHeight="1">
       <c r="A1" s="1"/>
-      <c r="B1" s="13" t="s">
+      <c r="B1" s="14" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="13" t="s">
+      <c r="C1" s="14" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="13"/>
-      <c r="E1" s="13"/>
-      <c r="F1" s="13" t="s">
+      <c r="D1" s="14"/>
+      <c r="E1" s="14"/>
+      <c r="F1" s="14" t="s">
         <v>2</v>
       </c>
-      <c r="G1" s="13"/>
+      <c r="G1" s="14"/>
       <c r="H1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="I1" s="13" t="s">
+      <c r="I1" s="14" t="s">
         <v>4</v>
       </c>
-      <c r="J1" s="13"/>
-      <c r="K1" s="13" t="s">
+      <c r="J1" s="14"/>
+      <c r="K1" s="14" t="s">
         <v>5</v>
       </c>
-      <c r="L1" s="13"/>
-      <c r="M1" s="13" t="s">
+      <c r="L1" s="14"/>
+      <c r="M1" s="14" t="s">
         <v>6</v>
       </c>
-      <c r="N1" s="13" t="s">
+      <c r="N1" s="14" t="s">
         <v>7</v>
       </c>
-      <c r="O1" s="13" t="s">
+      <c r="O1" s="14" t="s">
         <v>8</v>
       </c>
-      <c r="P1" s="12" t="s">
+      <c r="P1" s="13" t="s">
         <v>390</v>
       </c>
     </row>
@@ -2167,7 +2164,7 @@
       <c r="A2" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="B2" s="13"/>
+      <c r="B2" s="14"/>
       <c r="C2" s="2" t="s">
         <v>10</v>
       </c>
@@ -2198,192 +2195,192 @@
       <c r="L2" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="M2" s="13"/>
-      <c r="N2" s="13"/>
-      <c r="O2" s="13"/>
-      <c r="P2" s="12"/>
+      <c r="M2" s="14"/>
+      <c r="N2" s="14"/>
+      <c r="O2" s="14"/>
+      <c r="P2" s="13"/>
     </row>
-    <row r="3" spans="1:16" ht="250.8">
-      <c r="A3" s="1" t="s">
+    <row r="3" spans="1:16" s="4" customFormat="1" ht="250.8">
+      <c r="A3" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="B3" s="1" t="s">
+      <c r="B3" s="3" t="s">
         <v>71</v>
       </c>
-      <c r="C3" s="1" t="s">
+      <c r="C3" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="D3" s="1" t="s">
+      <c r="D3" s="3" t="s">
         <v>73</v>
       </c>
-      <c r="E3" s="1" t="s">
+      <c r="E3" s="3" t="s">
         <v>63</v>
       </c>
-      <c r="F3" s="1" t="s">
+      <c r="F3" s="3" t="s">
         <v>74</v>
       </c>
-      <c r="G3" s="1" t="s">
+      <c r="G3" s="3" t="s">
         <v>75</v>
       </c>
-      <c r="H3" s="1" t="s">
+      <c r="H3" s="3" t="s">
         <v>64</v>
       </c>
-      <c r="I3" s="1" t="s">
+      <c r="I3" s="3" t="s">
         <v>68</v>
       </c>
-      <c r="J3" s="1" t="s">
+      <c r="J3" s="3" t="s">
         <v>76</v>
       </c>
-      <c r="K3" s="1" t="s">
+      <c r="K3" s="3" t="s">
         <v>77</v>
       </c>
-      <c r="L3" s="1" t="s">
+      <c r="L3" s="3" t="s">
         <v>78</v>
       </c>
-      <c r="M3" s="1" t="s">
+      <c r="M3" s="3" t="s">
         <v>79</v>
       </c>
-      <c r="N3" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="O3" s="1" t="s">
+      <c r="N3" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="O3" s="3" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="4" spans="1:16" ht="171.6">
-      <c r="A4" s="1" t="s">
+    <row r="4" spans="1:16" s="4" customFormat="1" ht="171.6">
+      <c r="A4" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="B4" s="1" t="s">
+      <c r="B4" s="3" t="s">
         <v>81</v>
       </c>
-      <c r="C4" s="1" t="s">
+      <c r="C4" s="3" t="s">
         <v>82</v>
       </c>
-      <c r="D4" s="1" t="s">
+      <c r="D4" s="3" t="s">
         <v>83</v>
       </c>
-      <c r="E4" s="1" t="s">
+      <c r="E4" s="3" t="s">
         <v>84</v>
       </c>
-      <c r="F4" s="1" t="s">
+      <c r="F4" s="3" t="s">
         <v>85</v>
       </c>
-      <c r="G4" s="1" t="s">
+      <c r="G4" s="3" t="s">
         <v>78</v>
       </c>
-      <c r="H4" s="1" t="s">
+      <c r="H4" s="3" t="s">
         <v>86</v>
       </c>
-      <c r="I4" s="1" t="s">
+      <c r="I4" s="3" t="s">
         <v>68</v>
       </c>
-      <c r="J4" s="1" t="s">
+      <c r="J4" s="3" t="s">
         <v>87</v>
       </c>
-      <c r="K4" s="1" t="s">
+      <c r="K4" s="3" t="s">
         <v>88</v>
       </c>
-      <c r="L4" s="1" t="s">
+      <c r="L4" s="3" t="s">
         <v>89</v>
       </c>
-      <c r="M4" s="1"/>
-      <c r="N4" s="1"/>
-      <c r="O4" s="1" t="s">
+      <c r="M4" s="3"/>
+      <c r="N4" s="3"/>
+      <c r="O4" s="3" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="5" spans="1:16" ht="184.8">
-      <c r="A5" s="1" t="s">
+    <row r="5" spans="1:16" s="4" customFormat="1" ht="201" customHeight="1">
+      <c r="A5" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="B5" s="1" t="s">
+      <c r="B5" s="3" t="s">
         <v>91</v>
       </c>
-      <c r="C5" s="1" t="s">
+      <c r="C5" s="3" t="s">
         <v>65</v>
       </c>
       <c r="D5" s="3" t="s">
         <v>92</v>
       </c>
-      <c r="E5" s="1" t="s">
+      <c r="E5" s="3" t="s">
         <v>93</v>
       </c>
-      <c r="F5" s="1" t="s">
+      <c r="F5" s="3" t="s">
         <v>85</v>
       </c>
-      <c r="G5" s="1" t="s">
+      <c r="G5" s="3" t="s">
         <v>78</v>
       </c>
-      <c r="H5" s="1" t="s">
+      <c r="H5" s="3" t="s">
         <v>94</v>
       </c>
-      <c r="I5" s="1" t="s">
+      <c r="I5" s="3" t="s">
         <v>68</v>
       </c>
-      <c r="J5" s="1" t="s">
+      <c r="J5" s="3" t="s">
         <v>78</v>
       </c>
-      <c r="K5" s="1" t="s">
+      <c r="K5" s="3" t="s">
         <v>70</v>
       </c>
-      <c r="L5" s="1" t="s">
+      <c r="L5" s="3" t="s">
         <v>78</v>
       </c>
-      <c r="M5" s="1" t="s">
+      <c r="M5" s="3" t="s">
         <v>95</v>
       </c>
-      <c r="N5" s="1" t="s">
+      <c r="N5" s="3" t="s">
         <v>96</v>
       </c>
-      <c r="O5" s="1" t="s">
+      <c r="O5" s="3" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="6" spans="1:16" ht="198">
-      <c r="A6" s="1" t="s">
+    <row r="6" spans="1:16" s="4" customFormat="1" ht="210" customHeight="1">
+      <c r="A6" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="B6" s="1" t="s">
+      <c r="B6" s="3" t="s">
         <v>98</v>
       </c>
-      <c r="C6" s="1" t="s">
+      <c r="C6" s="3" t="s">
         <v>99</v>
       </c>
-      <c r="D6" s="1" t="s">
+      <c r="D6" s="3" t="s">
         <v>100</v>
       </c>
-      <c r="E6" s="1" t="s">
+      <c r="E6" s="3" t="s">
         <v>78</v>
       </c>
-      <c r="F6" s="1" t="s">
+      <c r="F6" s="3" t="s">
         <v>85</v>
       </c>
-      <c r="G6" s="1" t="s">
+      <c r="G6" s="3" t="s">
         <v>78</v>
       </c>
-      <c r="H6" s="1" t="s">
+      <c r="H6" s="3" t="s">
         <v>101</v>
       </c>
-      <c r="I6" s="1" t="s">
+      <c r="I6" s="3" t="s">
         <v>68</v>
       </c>
-      <c r="J6" s="1" t="s">
+      <c r="J6" s="3" t="s">
         <v>78</v>
       </c>
-      <c r="K6" s="1" t="s">
+      <c r="K6" s="3" t="s">
         <v>88</v>
       </c>
-      <c r="L6" s="1" t="s">
+      <c r="L6" s="3" t="s">
         <v>78</v>
       </c>
-      <c r="M6" s="1" t="s">
+      <c r="M6" s="3" t="s">
         <v>102</v>
       </c>
-      <c r="N6" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="O6" s="1" t="s">
+      <c r="N6" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="O6" s="3" t="s">
         <v>103</v>
       </c>
     </row>
@@ -2810,100 +2807,100 @@
         <v>174</v>
       </c>
     </row>
-    <row r="16" spans="1:16" s="5" customFormat="1" ht="290.39999999999998">
-      <c r="A16" s="4" t="s">
+    <row r="16" spans="1:16" s="4" customFormat="1" ht="290.39999999999998">
+      <c r="A16" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="B16" s="4" t="s">
+      <c r="B16" s="3" t="s">
         <v>175</v>
       </c>
-      <c r="C16" s="4" t="s">
+      <c r="C16" s="3" t="s">
         <v>330</v>
       </c>
-      <c r="D16" s="4" t="s">
+      <c r="D16" s="3" t="s">
         <v>176</v>
       </c>
-      <c r="E16" s="4" t="s">
+      <c r="E16" s="3" t="s">
         <v>135</v>
       </c>
-      <c r="F16" s="4" t="s">
+      <c r="F16" s="3" t="s">
         <v>331</v>
       </c>
-      <c r="G16" s="4" t="s">
+      <c r="G16" s="3" t="s">
         <v>332</v>
       </c>
-      <c r="H16" s="4" t="s">
+      <c r="H16" s="3" t="s">
         <v>333</v>
       </c>
-      <c r="I16" s="4" t="s">
+      <c r="I16" s="3" t="s">
         <v>68</v>
       </c>
-      <c r="J16" s="4" t="s">
+      <c r="J16" s="3" t="s">
         <v>334</v>
       </c>
-      <c r="K16" s="4" t="s">
+      <c r="K16" s="3" t="s">
         <v>69</v>
       </c>
-      <c r="L16" s="4" t="s">
+      <c r="L16" s="3" t="s">
         <v>335</v>
       </c>
-      <c r="M16" s="4" t="s">
+      <c r="M16" s="3" t="s">
         <v>336</v>
       </c>
-      <c r="N16" s="4" t="s">
+      <c r="N16" s="3" t="s">
         <v>177</v>
       </c>
-      <c r="O16" s="4" t="s">
+      <c r="O16" s="3" t="s">
         <v>178</v>
       </c>
     </row>
-    <row r="17" spans="1:16" s="5" customFormat="1" ht="132">
-      <c r="A17" s="4" t="s">
+    <row r="17" spans="1:16" s="4" customFormat="1" ht="132">
+      <c r="A17" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="B17" s="4" t="s">
+      <c r="B17" s="3" t="s">
         <v>301</v>
       </c>
-      <c r="C17" s="4" t="s">
+      <c r="C17" s="3" t="s">
         <v>289</v>
       </c>
-      <c r="D17" s="4" t="s">
+      <c r="D17" s="3" t="s">
         <v>290</v>
       </c>
-      <c r="E17" s="4" t="s">
+      <c r="E17" s="3" t="s">
         <v>291</v>
       </c>
-      <c r="F17" s="4" t="s">
+      <c r="F17" s="3" t="s">
         <v>292</v>
       </c>
-      <c r="G17" s="4" t="s">
+      <c r="G17" s="3" t="s">
         <v>293</v>
       </c>
-      <c r="H17" s="4" t="s">
+      <c r="H17" s="3" t="s">
         <v>294</v>
       </c>
-      <c r="I17" s="4" t="s">
+      <c r="I17" s="3" t="s">
         <v>295</v>
       </c>
-      <c r="J17" s="4" t="s">
+      <c r="J17" s="3" t="s">
         <v>296</v>
       </c>
-      <c r="K17" s="4" t="s">
+      <c r="K17" s="3" t="s">
         <v>69</v>
       </c>
-      <c r="L17" s="4" t="s">
+      <c r="L17" s="3" t="s">
         <v>297</v>
       </c>
-      <c r="M17" s="4" t="s">
+      <c r="M17" s="3" t="s">
         <v>298</v>
       </c>
-      <c r="N17" s="4" t="s">
+      <c r="N17" s="3" t="s">
         <v>300</v>
       </c>
-      <c r="O17" s="4" t="s">
+      <c r="O17" s="3" t="s">
         <v>391</v>
       </c>
-      <c r="P17" s="4" t="s">
+      <c r="P17" s="3" t="s">
         <v>299</v>
       </c>
     </row>
@@ -2954,53 +2951,53 @@
         <v>66</v>
       </c>
     </row>
-    <row r="19" spans="1:16" s="5" customFormat="1" ht="61.5" customHeight="1">
-      <c r="A19" s="4" t="s">
+    <row r="19" spans="1:16" s="4" customFormat="1" ht="61.5" customHeight="1">
+      <c r="A19" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="B19" s="4" t="s">
+      <c r="B19" s="3" t="s">
         <v>191</v>
       </c>
-      <c r="C19" s="4" t="s">
+      <c r="C19" s="3" t="s">
         <v>192</v>
       </c>
-      <c r="D19" s="4" t="s">
+      <c r="D19" s="3" t="s">
         <v>193</v>
       </c>
-      <c r="E19" s="4" t="s">
+      <c r="E19" s="3" t="s">
         <v>194</v>
       </c>
-      <c r="F19" s="4" t="s">
+      <c r="F19" s="3" t="s">
         <v>195</v>
       </c>
-      <c r="G19" s="4" t="s">
+      <c r="G19" s="3" t="s">
         <v>194</v>
       </c>
-      <c r="H19" s="4" t="s">
+      <c r="H19" s="3" t="s">
         <v>196</v>
       </c>
-      <c r="I19" s="4" t="s">
+      <c r="I19" s="3" t="s">
         <v>197</v>
       </c>
-      <c r="J19" s="4" t="s">
+      <c r="J19" s="3" t="s">
         <v>198</v>
       </c>
-      <c r="K19" s="4" t="s">
+      <c r="K19" s="3" t="s">
         <v>199</v>
       </c>
-      <c r="L19" s="4" t="s">
+      <c r="L19" s="3" t="s">
         <v>200</v>
       </c>
-      <c r="M19" s="4" t="s">
+      <c r="M19" s="3" t="s">
         <v>201</v>
       </c>
-      <c r="N19" s="4" t="s">
+      <c r="N19" s="3" t="s">
         <v>202</v>
       </c>
-      <c r="O19" s="4" t="s">
+      <c r="O19" s="3" t="s">
         <v>194</v>
       </c>
-      <c r="P19" s="5" t="s">
+      <c r="P19" s="4" t="s">
         <v>203</v>
       </c>
     </row>
@@ -3051,103 +3048,103 @@
         <v>208</v>
       </c>
     </row>
-    <row r="21" spans="1:16" s="5" customFormat="1" ht="132">
-      <c r="A21" s="4" t="s">
+    <row r="21" spans="1:16" s="4" customFormat="1" ht="132">
+      <c r="A21" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="B21" s="4" t="s">
+      <c r="B21" s="3" t="s">
         <v>302</v>
       </c>
-      <c r="C21" s="4" t="s">
+      <c r="C21" s="3" t="s">
         <v>303</v>
       </c>
-      <c r="D21" s="4" t="s">
+      <c r="D21" s="3" t="s">
         <v>304</v>
       </c>
-      <c r="E21" s="4" t="s">
+      <c r="E21" s="3" t="s">
         <v>305</v>
       </c>
-      <c r="F21" s="4" t="s">
+      <c r="F21" s="3" t="s">
         <v>306</v>
       </c>
-      <c r="G21" s="4" t="s">
+      <c r="G21" s="3" t="s">
         <v>267</v>
       </c>
-      <c r="H21" s="4" t="s">
+      <c r="H21" s="3" t="s">
         <v>307</v>
       </c>
-      <c r="I21" s="4" t="s">
+      <c r="I21" s="3" t="s">
         <v>308</v>
       </c>
-      <c r="J21" s="4" t="s">
+      <c r="J21" s="3" t="s">
         <v>309</v>
       </c>
-      <c r="K21" s="4" t="s">
+      <c r="K21" s="3" t="s">
         <v>311</v>
       </c>
-      <c r="L21" s="4" t="s">
+      <c r="L21" s="3" t="s">
         <v>310</v>
       </c>
-      <c r="M21" s="4" t="s">
+      <c r="M21" s="3" t="s">
         <v>312</v>
       </c>
-      <c r="N21" s="4" t="s">
+      <c r="N21" s="3" t="s">
         <v>315</v>
       </c>
-      <c r="O21" s="4" t="s">
+      <c r="O21" s="3" t="s">
         <v>313</v>
       </c>
-      <c r="P21" s="5" t="s">
+      <c r="P21" s="4" t="s">
         <v>314</v>
       </c>
     </row>
-    <row r="22" spans="1:16" s="5" customFormat="1" ht="158.4">
-      <c r="A22" s="4" t="s">
+    <row r="22" spans="1:16" s="4" customFormat="1" ht="158.4">
+      <c r="A22" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="B22" s="4" t="s">
+      <c r="B22" s="3" t="s">
         <v>316</v>
       </c>
-      <c r="C22" s="4" t="s">
+      <c r="C22" s="3" t="s">
         <v>317</v>
       </c>
-      <c r="D22" s="4" t="s">
+      <c r="D22" s="3" t="s">
         <v>319</v>
       </c>
-      <c r="E22" s="4" t="s">
+      <c r="E22" s="3" t="s">
         <v>318</v>
       </c>
-      <c r="F22" s="4" t="s">
+      <c r="F22" s="3" t="s">
         <v>321</v>
       </c>
-      <c r="G22" s="4" t="s">
+      <c r="G22" s="3" t="s">
         <v>320</v>
       </c>
-      <c r="H22" s="4" t="s">
+      <c r="H22" s="3" t="s">
         <v>322</v>
       </c>
-      <c r="I22" s="4" t="s">
+      <c r="I22" s="3" t="s">
         <v>68</v>
       </c>
-      <c r="J22" s="4" t="s">
+      <c r="J22" s="3" t="s">
         <v>269</v>
       </c>
-      <c r="K22" s="4" t="s">
+      <c r="K22" s="3" t="s">
         <v>323</v>
       </c>
-      <c r="L22" s="4" t="s">
+      <c r="L22" s="3" t="s">
         <v>324</v>
       </c>
-      <c r="M22" s="4" t="s">
+      <c r="M22" s="3" t="s">
         <v>325</v>
       </c>
-      <c r="N22" s="4" t="s">
+      <c r="N22" s="3" t="s">
         <v>326</v>
       </c>
-      <c r="O22" s="4" t="s">
+      <c r="O22" s="3" t="s">
         <v>327</v>
       </c>
-      <c r="P22" s="5" t="s">
+      <c r="P22" s="4" t="s">
         <v>328</v>
       </c>
     </row>
@@ -3199,103 +3196,103 @@
         <v>217</v>
       </c>
     </row>
-    <row r="24" spans="1:16" s="5" customFormat="1" ht="145.19999999999999">
-      <c r="A24" s="4" t="s">
+    <row r="24" spans="1:16" s="4" customFormat="1" ht="145.19999999999999">
+      <c r="A24" s="3" t="s">
         <v>337</v>
       </c>
-      <c r="B24" s="4" t="s">
+      <c r="B24" s="3" t="s">
         <v>338</v>
       </c>
-      <c r="C24" s="4" t="s">
+      <c r="C24" s="3" t="s">
         <v>339</v>
       </c>
-      <c r="D24" s="4" t="s">
+      <c r="D24" s="3" t="s">
         <v>340</v>
       </c>
-      <c r="E24" s="4" t="s">
+      <c r="E24" s="3" t="s">
         <v>341</v>
       </c>
-      <c r="F24" s="4" t="s">
+      <c r="F24" s="3" t="s">
         <v>343</v>
       </c>
-      <c r="G24" s="4" t="s">
+      <c r="G24" s="3" t="s">
         <v>342</v>
       </c>
-      <c r="H24" s="4" t="s">
+      <c r="H24" s="3" t="s">
         <v>344</v>
       </c>
-      <c r="I24" s="4" t="s">
+      <c r="I24" s="3" t="s">
         <v>345</v>
       </c>
-      <c r="J24" s="4" t="s">
+      <c r="J24" s="3" t="s">
         <v>346</v>
       </c>
-      <c r="K24" s="4" t="s">
+      <c r="K24" s="3" t="s">
         <v>347</v>
       </c>
-      <c r="L24" s="4" t="s">
+      <c r="L24" s="3" t="s">
         <v>348</v>
       </c>
-      <c r="M24" s="4" t="s">
+      <c r="M24" s="3" t="s">
         <v>352</v>
       </c>
-      <c r="N24" s="4" t="s">
+      <c r="N24" s="3" t="s">
         <v>351</v>
       </c>
-      <c r="O24" s="4" t="s">
+      <c r="O24" s="3" t="s">
         <v>349</v>
       </c>
-      <c r="P24" s="5" t="s">
+      <c r="P24" s="4" t="s">
         <v>350</v>
       </c>
     </row>
-    <row r="25" spans="1:16" s="5" customFormat="1" ht="118.8">
-      <c r="A25" s="4" t="s">
+    <row r="25" spans="1:16" s="4" customFormat="1" ht="118.8">
+      <c r="A25" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="B25" s="4" t="s">
+      <c r="B25" s="3" t="s">
         <v>353</v>
       </c>
-      <c r="C25" s="4" t="s">
+      <c r="C25" s="3" t="s">
         <v>363</v>
       </c>
-      <c r="D25" s="4" t="s">
+      <c r="D25" s="3" t="s">
         <v>354</v>
       </c>
-      <c r="E25" s="5" t="s">
+      <c r="E25" s="4" t="s">
         <v>318</v>
       </c>
-      <c r="F25" s="4" t="s">
+      <c r="F25" s="3" t="s">
         <v>331</v>
       </c>
-      <c r="G25" s="4" t="s">
+      <c r="G25" s="3" t="s">
         <v>355</v>
       </c>
-      <c r="H25" s="4" t="s">
+      <c r="H25" s="3" t="s">
         <v>356</v>
       </c>
-      <c r="I25" s="4" t="s">
+      <c r="I25" s="3" t="s">
         <v>257</v>
       </c>
-      <c r="J25" s="4" t="s">
+      <c r="J25" s="3" t="s">
         <v>269</v>
       </c>
-      <c r="K25" s="4" t="s">
+      <c r="K25" s="3" t="s">
         <v>357</v>
       </c>
-      <c r="L25" s="4" t="s">
+      <c r="L25" s="3" t="s">
         <v>358</v>
       </c>
-      <c r="M25" s="4" t="s">
+      <c r="M25" s="3" t="s">
         <v>359</v>
       </c>
-      <c r="N25" s="4" t="s">
+      <c r="N25" s="3" t="s">
         <v>360</v>
       </c>
-      <c r="O25" s="4" t="s">
+      <c r="O25" s="3" t="s">
         <v>361</v>
       </c>
-      <c r="P25" s="5" t="s">
+      <c r="P25" s="4" t="s">
         <v>362</v>
       </c>
     </row>
@@ -3344,53 +3341,53 @@
         <v>222</v>
       </c>
     </row>
-    <row r="27" spans="1:16" s="10" customFormat="1" ht="132">
-      <c r="A27" s="9" t="s">
+    <row r="27" spans="1:16" s="9" customFormat="1" ht="132">
+      <c r="A27" s="8" t="s">
         <v>43</v>
       </c>
-      <c r="B27" s="9" t="s">
+      <c r="B27" s="8" t="s">
         <v>380</v>
       </c>
-      <c r="C27" s="9" t="s">
+      <c r="C27" s="8" t="s">
         <v>381</v>
       </c>
-      <c r="D27" s="9" t="s">
+      <c r="D27" s="8" t="s">
         <v>382</v>
       </c>
-      <c r="E27" s="9" t="s">
+      <c r="E27" s="8" t="s">
         <v>383</v>
       </c>
-      <c r="F27" s="9" t="s">
+      <c r="F27" s="8" t="s">
         <v>384</v>
       </c>
-      <c r="G27" s="9" t="s">
+      <c r="G27" s="8" t="s">
         <v>212</v>
       </c>
-      <c r="H27" s="9" t="s">
+      <c r="H27" s="8" t="s">
         <v>385</v>
       </c>
-      <c r="I27" s="9" t="s">
+      <c r="I27" s="8" t="s">
         <v>257</v>
       </c>
-      <c r="J27" s="9" t="s">
+      <c r="J27" s="8" t="s">
         <v>78</v>
       </c>
-      <c r="K27" s="9" t="s">
+      <c r="K27" s="8" t="s">
         <v>386</v>
       </c>
-      <c r="L27" s="9" t="s">
+      <c r="L27" s="8" t="s">
         <v>387</v>
       </c>
-      <c r="M27" s="9" t="s">
+      <c r="M27" s="8" t="s">
         <v>388</v>
       </c>
-      <c r="N27" s="9" t="s">
+      <c r="N27" s="8" t="s">
         <v>393</v>
       </c>
-      <c r="O27" s="9" t="s">
+      <c r="O27" s="8" t="s">
         <v>389</v>
       </c>
-      <c r="P27" s="10" t="s">
+      <c r="P27" s="9" t="s">
         <v>392</v>
       </c>
     </row>
@@ -3441,153 +3438,153 @@
         <v>236</v>
       </c>
     </row>
-    <row r="29" spans="1:16" s="5" customFormat="1" ht="409.6">
-      <c r="A29" s="4" t="s">
+    <row r="29" spans="1:16" s="4" customFormat="1" ht="409.6">
+      <c r="A29" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="B29" s="4" t="s">
+      <c r="B29" s="3" t="s">
         <v>237</v>
       </c>
-      <c r="C29" s="4" t="s">
+      <c r="C29" s="3" t="s">
         <v>238</v>
       </c>
-      <c r="D29" s="4" t="s">
+      <c r="D29" s="3" t="s">
         <v>239</v>
       </c>
-      <c r="E29" s="4" t="s">
+      <c r="E29" s="3" t="s">
         <v>240</v>
       </c>
-      <c r="F29" s="4" t="s">
+      <c r="F29" s="3" t="s">
         <v>241</v>
       </c>
-      <c r="G29" s="4" t="s">
+      <c r="G29" s="3" t="s">
         <v>242</v>
       </c>
-      <c r="H29" s="4" t="s">
+      <c r="H29" s="3" t="s">
         <v>243</v>
       </c>
-      <c r="I29" s="4" t="s">
+      <c r="I29" s="3" t="s">
         <v>244</v>
       </c>
-      <c r="J29" s="4" t="s">
+      <c r="J29" s="3" t="s">
         <v>245</v>
       </c>
-      <c r="K29" s="4" t="s">
+      <c r="K29" s="3" t="s">
         <v>246</v>
       </c>
-      <c r="L29" s="4" t="s">
+      <c r="L29" s="3" t="s">
         <v>247</v>
       </c>
-      <c r="M29" s="4" t="s">
+      <c r="M29" s="3" t="s">
         <v>248</v>
       </c>
-      <c r="N29" s="4" t="s">
+      <c r="N29" s="3" t="s">
         <v>249</v>
       </c>
-      <c r="O29" s="4" t="s">
+      <c r="O29" s="3" t="s">
         <v>250</v>
       </c>
-      <c r="P29" s="5" t="s">
+      <c r="P29" s="4" t="s">
         <v>251</v>
       </c>
     </row>
-    <row r="30" spans="1:16" s="5" customFormat="1" ht="250.8">
-      <c r="A30" s="4" t="s">
+    <row r="30" spans="1:16" s="4" customFormat="1" ht="250.8">
+      <c r="A30" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="B30" s="4" t="s">
+      <c r="B30" s="3" t="s">
         <v>262</v>
       </c>
-      <c r="C30" s="4" t="s">
+      <c r="C30" s="3" t="s">
         <v>263</v>
       </c>
-      <c r="D30" s="4" t="s">
+      <c r="D30" s="3" t="s">
         <v>264</v>
       </c>
-      <c r="E30" s="4" t="s">
+      <c r="E30" s="3" t="s">
         <v>265</v>
       </c>
-      <c r="F30" s="4" t="s">
+      <c r="F30" s="3" t="s">
         <v>266</v>
       </c>
-      <c r="G30" s="4" t="s">
+      <c r="G30" s="3" t="s">
         <v>267</v>
       </c>
-      <c r="H30" s="4" t="s">
+      <c r="H30" s="3" t="s">
         <v>275</v>
       </c>
-      <c r="I30" s="4" t="s">
+      <c r="I30" s="3" t="s">
         <v>268</v>
       </c>
-      <c r="J30" s="4" t="s">
+      <c r="J30" s="3" t="s">
         <v>269</v>
       </c>
-      <c r="K30" s="4" t="s">
+      <c r="K30" s="3" t="s">
         <v>270</v>
       </c>
-      <c r="L30" s="4" t="s">
+      <c r="L30" s="3" t="s">
         <v>271</v>
       </c>
-      <c r="M30" s="7" t="s">
+      <c r="M30" s="6" t="s">
         <v>364</v>
       </c>
-      <c r="N30" s="4" t="s">
+      <c r="N30" s="3" t="s">
         <v>272</v>
       </c>
-      <c r="O30" s="4" t="s">
+      <c r="O30" s="3" t="s">
         <v>274</v>
       </c>
-      <c r="P30" s="5" t="s">
+      <c r="P30" s="4" t="s">
         <v>273</v>
       </c>
     </row>
-    <row r="31" spans="1:16" s="5" customFormat="1" ht="132">
-      <c r="A31" s="4" t="s">
+    <row r="31" spans="1:16" s="4" customFormat="1" ht="132">
+      <c r="A31" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="B31" s="4" t="s">
+      <c r="B31" s="3" t="s">
         <v>276</v>
       </c>
-      <c r="C31" s="4" t="s">
+      <c r="C31" s="3" t="s">
         <v>277</v>
       </c>
-      <c r="D31" s="4" t="s">
+      <c r="D31" s="3" t="s">
         <v>278</v>
       </c>
-      <c r="E31" s="8" t="s">
+      <c r="E31" s="7" t="s">
         <v>365</v>
       </c>
-      <c r="F31" s="4" t="s">
+      <c r="F31" s="3" t="s">
         <v>279</v>
       </c>
-      <c r="G31" s="4" t="s">
+      <c r="G31" s="3" t="s">
         <v>280</v>
       </c>
-      <c r="H31" s="4" t="s">
+      <c r="H31" s="3" t="s">
         <v>281</v>
       </c>
-      <c r="I31" s="4" t="s">
+      <c r="I31" s="3" t="s">
         <v>282</v>
       </c>
-      <c r="J31" s="4" t="s">
+      <c r="J31" s="3" t="s">
         <v>269</v>
       </c>
-      <c r="K31" s="4" t="s">
+      <c r="K31" s="3" t="s">
         <v>283</v>
       </c>
-      <c r="L31" s="4" t="s">
+      <c r="L31" s="3" t="s">
         <v>284</v>
       </c>
-      <c r="M31" s="4" t="s">
+      <c r="M31" s="3" t="s">
         <v>285</v>
       </c>
-      <c r="N31" s="4" t="s">
+      <c r="N31" s="3" t="s">
         <v>286</v>
       </c>
-      <c r="O31" s="4" t="s">
+      <c r="O31" s="3" t="s">
         <v>288</v>
       </c>
-      <c r="P31" s="4" t="s">
+      <c r="P31" s="3" t="s">
         <v>287</v>
       </c>
     </row>
@@ -3637,7 +3634,7 @@
       <c r="O32" s="1" t="s">
         <v>378</v>
       </c>
-      <c r="P32" s="6" t="s">
+      <c r="P32" s="5" t="s">
         <v>379</v>
       </c>
     </row>
@@ -3732,7 +3729,7 @@
       <c r="O34" s="1" t="s">
         <v>406</v>
       </c>
-      <c r="P34" s="6" t="s">
+      <c r="P34" s="5" t="s">
         <v>407</v>
       </c>
     </row>
@@ -3749,7 +3746,7 @@
       <c r="D35" s="1" t="s">
         <v>410</v>
       </c>
-      <c r="E35" s="11" t="s">
+      <c r="E35" s="10" t="s">
         <v>318</v>
       </c>
       <c r="F35" s="1" t="s">
@@ -3782,7 +3779,7 @@
       <c r="O35" s="1" t="s">
         <v>417</v>
       </c>
-      <c r="P35" s="6" t="s">
+      <c r="P35" s="5" t="s">
         <v>418</v>
       </c>
     </row>
@@ -3832,7 +3829,7 @@
       <c r="O36" s="1" t="s">
         <v>428</v>
       </c>
-      <c r="P36" s="6" t="s">
+      <c r="P36" s="5" t="s">
         <v>429</v>
       </c>
     </row>
@@ -3882,52 +3879,52 @@
       <c r="O37" s="1" t="s">
         <v>441</v>
       </c>
-      <c r="P37" s="6" t="s">
+      <c r="P37" s="5" t="s">
         <v>442</v>
       </c>
     </row>
-    <row r="38" spans="1:16" s="15" customFormat="1">
-      <c r="A38" s="14" t="s">
+    <row r="38" spans="1:16" s="12" customFormat="1">
+      <c r="A38" s="11" t="s">
         <v>54</v>
       </c>
-      <c r="B38" s="14" t="s">
-        <v>66</v>
-      </c>
-      <c r="C38" s="14" t="s">
-        <v>66</v>
-      </c>
-      <c r="D38" s="14" t="s">
-        <v>66</v>
-      </c>
-      <c r="E38" s="14" t="s">
-        <v>66</v>
-      </c>
-      <c r="F38" s="14" t="s">
-        <v>66</v>
-      </c>
-      <c r="G38" s="14" t="s">
-        <v>66</v>
-      </c>
-      <c r="H38" s="14" t="s">
-        <v>66</v>
-      </c>
-      <c r="I38" s="14" t="s">
-        <v>66</v>
-      </c>
-      <c r="J38" s="14" t="s">
-        <v>66</v>
-      </c>
-      <c r="K38" s="14" t="s">
-        <v>66</v>
-      </c>
-      <c r="L38" s="14" t="s">
-        <v>66</v>
-      </c>
-      <c r="M38" s="14" t="s">
-        <v>66</v>
-      </c>
-      <c r="N38" s="14"/>
-      <c r="O38" s="14" t="s">
+      <c r="B38" s="11" t="s">
+        <v>66</v>
+      </c>
+      <c r="C38" s="11" t="s">
+        <v>66</v>
+      </c>
+      <c r="D38" s="11" t="s">
+        <v>66</v>
+      </c>
+      <c r="E38" s="11" t="s">
+        <v>66</v>
+      </c>
+      <c r="F38" s="11" t="s">
+        <v>66</v>
+      </c>
+      <c r="G38" s="11" t="s">
+        <v>66</v>
+      </c>
+      <c r="H38" s="11" t="s">
+        <v>66</v>
+      </c>
+      <c r="I38" s="11" t="s">
+        <v>66</v>
+      </c>
+      <c r="J38" s="11" t="s">
+        <v>66</v>
+      </c>
+      <c r="K38" s="11" t="s">
+        <v>66</v>
+      </c>
+      <c r="L38" s="11" t="s">
+        <v>66</v>
+      </c>
+      <c r="M38" s="11" t="s">
+        <v>66</v>
+      </c>
+      <c r="N38" s="11"/>
+      <c r="O38" s="11" t="s">
         <v>66</v>
       </c>
     </row>
@@ -4315,12 +4312,9 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -4468,15 +4462,19 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{24F2579D-323E-48EA-8FED-D372AFFF0A04}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1160EB8C-E200-4916-A3B3-9BF8115D37F8}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -4500,10 +4498,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1160EB8C-E200-4916-A3B3-9BF8115D37F8}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{24F2579D-323E-48EA-8FED-D372AFFF0A04}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Add initial version of Individual AnnotationsORC.xlsx with Oscar Andres Rincon Cardeño data
</commit_message>
<xml_diff>
--- a/main/04_data_extraction/Individual AnnotationsORC.xlsx
+++ b/main/04_data_extraction/Individual AnnotationsORC.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\orincon\scoping-ml-wave-seismology\main\04_data_extraction\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB662C5E-E0C0-44CB-81B7-70F2198F677D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{74B956C0-3662-49FF-8CA7-1CEC509FEC4D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{115BB8D9-8B86-4726-97F8-E06477FD353D}"/>
   </bookViews>
@@ -2384,379 +2384,379 @@
         <v>103</v>
       </c>
     </row>
-    <row r="7" spans="1:16" ht="250.8">
-      <c r="A7" s="1" t="s">
+    <row r="7" spans="1:16" s="4" customFormat="1" ht="250.8">
+      <c r="A7" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="B7" s="1" t="s">
+      <c r="B7" s="3" t="s">
         <v>104</v>
       </c>
-      <c r="C7" s="1" t="s">
+      <c r="C7" s="3" t="s">
         <v>105</v>
       </c>
-      <c r="D7" s="1" t="s">
+      <c r="D7" s="3" t="s">
         <v>106</v>
       </c>
-      <c r="E7" s="1" t="s">
+      <c r="E7" s="3" t="s">
         <v>107</v>
       </c>
-      <c r="F7" s="1" t="s">
+      <c r="F7" s="3" t="s">
         <v>108</v>
       </c>
-      <c r="G7" s="1" t="s">
+      <c r="G7" s="3" t="s">
         <v>109</v>
       </c>
-      <c r="H7" s="1" t="s">
+      <c r="H7" s="3" t="s">
         <v>110</v>
       </c>
-      <c r="I7" s="1" t="s">
+      <c r="I7" s="3" t="s">
         <v>67</v>
       </c>
-      <c r="J7" s="1" t="s">
+      <c r="J7" s="3" t="s">
         <v>111</v>
       </c>
-      <c r="K7" s="1" t="s">
+      <c r="K7" s="3" t="s">
         <v>70</v>
       </c>
-      <c r="L7" s="1" t="s">
+      <c r="L7" s="3" t="s">
         <v>78</v>
       </c>
-      <c r="M7" s="1" t="s">
+      <c r="M7" s="3" t="s">
         <v>112</v>
       </c>
-      <c r="N7" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="O7" s="1" t="s">
+      <c r="N7" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="O7" s="3" t="s">
         <v>113</v>
       </c>
     </row>
-    <row r="8" spans="1:16" ht="250.8">
-      <c r="A8" s="1" t="s">
+    <row r="8" spans="1:16" s="4" customFormat="1" ht="250.8">
+      <c r="A8" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="B8" s="1" t="s">
+      <c r="B8" s="3" t="s">
         <v>114</v>
       </c>
-      <c r="C8" s="1" t="s">
+      <c r="C8" s="3" t="s">
         <v>115</v>
       </c>
-      <c r="D8" s="1" t="s">
+      <c r="D8" s="3" t="s">
         <v>116</v>
       </c>
-      <c r="E8" s="1" t="s">
+      <c r="E8" s="3" t="s">
         <v>117</v>
       </c>
-      <c r="F8" s="1" t="s">
+      <c r="F8" s="3" t="s">
         <v>85</v>
       </c>
-      <c r="G8" s="1" t="s">
+      <c r="G8" s="3" t="s">
         <v>78</v>
       </c>
-      <c r="H8" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="I8" s="1" t="s">
+      <c r="H8" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="I8" s="3" t="s">
         <v>67</v>
       </c>
-      <c r="J8" s="1" t="s">
+      <c r="J8" s="3" t="s">
         <v>118</v>
       </c>
-      <c r="K8" s="1" t="s">
+      <c r="K8" s="3" t="s">
         <v>119</v>
       </c>
-      <c r="L8" s="1" t="s">
+      <c r="L8" s="3" t="s">
         <v>120</v>
       </c>
-      <c r="M8" s="1" t="s">
+      <c r="M8" s="3" t="s">
         <v>121</v>
       </c>
-      <c r="N8" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="O8" s="1" t="s">
+      <c r="N8" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="O8" s="3" t="s">
         <v>122</v>
       </c>
     </row>
-    <row r="9" spans="1:16" ht="184.8">
-      <c r="A9" s="1" t="s">
+    <row r="9" spans="1:16" s="4" customFormat="1" ht="184.8">
+      <c r="A9" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="B9" s="1" t="s">
+      <c r="B9" s="3" t="s">
         <v>123</v>
       </c>
-      <c r="C9" s="1" t="s">
+      <c r="C9" s="3" t="s">
         <v>124</v>
       </c>
-      <c r="D9" s="1" t="s">
+      <c r="D9" s="3" t="s">
         <v>125</v>
       </c>
-      <c r="E9" s="1" t="s">
+      <c r="E9" s="3" t="s">
         <v>126</v>
       </c>
-      <c r="F9" s="1" t="s">
+      <c r="F9" s="3" t="s">
         <v>85</v>
       </c>
-      <c r="G9" s="1" t="s">
+      <c r="G9" s="3" t="s">
         <v>127</v>
       </c>
-      <c r="H9" s="1" t="s">
+      <c r="H9" s="3" t="s">
         <v>128</v>
       </c>
-      <c r="I9" s="1" t="s">
+      <c r="I9" s="3" t="s">
         <v>329</v>
       </c>
-      <c r="J9" s="1" t="s">
+      <c r="J9" s="3" t="s">
         <v>129</v>
       </c>
-      <c r="K9" s="1" t="s">
+      <c r="K9" s="3" t="s">
         <v>77</v>
       </c>
-      <c r="L9" s="1" t="s">
+      <c r="L9" s="3" t="s">
         <v>78</v>
       </c>
-      <c r="M9" s="1" t="s">
+      <c r="M9" s="3" t="s">
         <v>130</v>
       </c>
-      <c r="N9" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="O9" s="1" t="s">
+      <c r="N9" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="O9" s="3" t="s">
         <v>131</v>
       </c>
     </row>
-    <row r="10" spans="1:16" ht="290.39999999999998">
-      <c r="A10" s="1" t="s">
+    <row r="10" spans="1:16" s="4" customFormat="1" ht="290.39999999999998">
+      <c r="A10" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="B10" s="1" t="s">
+      <c r="B10" s="3" t="s">
         <v>132</v>
       </c>
-      <c r="C10" s="1" t="s">
+      <c r="C10" s="3" t="s">
         <v>133</v>
       </c>
-      <c r="D10" s="1" t="s">
+      <c r="D10" s="3" t="s">
         <v>134</v>
       </c>
-      <c r="E10" s="1" t="s">
+      <c r="E10" s="3" t="s">
         <v>135</v>
       </c>
-      <c r="F10" s="1" t="s">
+      <c r="F10" s="3" t="s">
         <v>85</v>
       </c>
-      <c r="G10" s="1" t="s">
+      <c r="G10" s="3" t="s">
         <v>78</v>
       </c>
-      <c r="H10" s="1" t="s">
+      <c r="H10" s="3" t="s">
         <v>136</v>
       </c>
-      <c r="I10" s="1" t="s">
+      <c r="I10" s="3" t="s">
         <v>329</v>
       </c>
-      <c r="J10" s="1" t="s">
+      <c r="J10" s="3" t="s">
         <v>78</v>
       </c>
-      <c r="K10" s="1" t="s">
+      <c r="K10" s="3" t="s">
         <v>137</v>
       </c>
-      <c r="L10" s="1" t="s">
+      <c r="L10" s="3" t="s">
         <v>138</v>
       </c>
-      <c r="M10" s="1" t="s">
+      <c r="M10" s="3" t="s">
         <v>139</v>
       </c>
-      <c r="N10" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="O10" s="1" t="s">
+      <c r="N10" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="O10" s="3" t="s">
         <v>140</v>
       </c>
     </row>
-    <row r="11" spans="1:16" ht="211.2">
-      <c r="A11" s="1" t="s">
+    <row r="11" spans="1:16" s="4" customFormat="1" ht="211.2">
+      <c r="A11" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="B11" s="1" t="s">
+      <c r="B11" s="3" t="s">
         <v>141</v>
       </c>
-      <c r="C11" s="1" t="s">
+      <c r="C11" s="3" t="s">
         <v>142</v>
       </c>
-      <c r="D11" s="1" t="s">
+      <c r="D11" s="3" t="s">
         <v>143</v>
       </c>
-      <c r="E11" s="1" t="s">
+      <c r="E11" s="3" t="s">
         <v>78</v>
       </c>
-      <c r="F11" s="1" t="s">
+      <c r="F11" s="3" t="s">
         <v>85</v>
       </c>
-      <c r="G11" s="1" t="s">
+      <c r="G11" s="3" t="s">
         <v>78</v>
       </c>
-      <c r="H11" s="1" t="s">
+      <c r="H11" s="3" t="s">
         <v>144</v>
       </c>
-      <c r="I11" s="1" t="s">
+      <c r="I11" s="3" t="s">
         <v>68</v>
       </c>
-      <c r="J11" s="1" t="s">
+      <c r="J11" s="3" t="s">
         <v>78</v>
       </c>
-      <c r="K11" s="1" t="s">
+      <c r="K11" s="3" t="s">
         <v>69</v>
       </c>
-      <c r="L11" s="1" t="s">
+      <c r="L11" s="3" t="s">
         <v>78</v>
       </c>
-      <c r="M11" s="1" t="s">
+      <c r="M11" s="3" t="s">
         <v>145</v>
       </c>
-      <c r="N11" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="O11" s="1" t="s">
+      <c r="N11" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="O11" s="3" t="s">
         <v>146</v>
       </c>
     </row>
-    <row r="12" spans="1:16" ht="198">
-      <c r="A12" s="1" t="s">
+    <row r="12" spans="1:16" s="4" customFormat="1" ht="198">
+      <c r="A12" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="B12" s="1" t="s">
+      <c r="B12" s="3" t="s">
         <v>147</v>
       </c>
-      <c r="C12" s="1" t="s">
+      <c r="C12" s="3" t="s">
         <v>148</v>
       </c>
-      <c r="D12" s="1" t="s">
+      <c r="D12" s="3" t="s">
         <v>149</v>
       </c>
-      <c r="E12" s="1" t="s">
+      <c r="E12" s="3" t="s">
         <v>78</v>
       </c>
-      <c r="F12" s="1" t="s">
+      <c r="F12" s="3" t="s">
         <v>150</v>
       </c>
-      <c r="G12" s="1" t="s">
+      <c r="G12" s="3" t="s">
         <v>151</v>
       </c>
-      <c r="H12" s="1" t="s">
+      <c r="H12" s="3" t="s">
         <v>152</v>
       </c>
-      <c r="I12" s="1" t="s">
+      <c r="I12" s="3" t="s">
         <v>67</v>
       </c>
-      <c r="J12" s="1" t="s">
+      <c r="J12" s="3" t="s">
         <v>78</v>
       </c>
-      <c r="K12" s="1" t="s">
+      <c r="K12" s="3" t="s">
         <v>70</v>
       </c>
-      <c r="L12" s="1" t="s">
+      <c r="L12" s="3" t="s">
         <v>78</v>
       </c>
-      <c r="M12" s="1" t="s">
+      <c r="M12" s="3" t="s">
         <v>153</v>
       </c>
-      <c r="N12" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="O12" s="1" t="s">
+      <c r="N12" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="O12" s="3" t="s">
         <v>154</v>
       </c>
     </row>
-    <row r="13" spans="1:16" ht="264">
-      <c r="A13" s="1" t="s">
+    <row r="13" spans="1:16" s="4" customFormat="1" ht="264">
+      <c r="A13" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="B13" s="1" t="s">
+      <c r="B13" s="3" t="s">
         <v>155</v>
       </c>
-      <c r="C13" s="1" t="s">
+      <c r="C13" s="3" t="s">
         <v>156</v>
       </c>
-      <c r="D13" s="1" t="s">
+      <c r="D13" s="3" t="s">
         <v>157</v>
       </c>
-      <c r="E13" s="1" t="s">
+      <c r="E13" s="3" t="s">
         <v>78</v>
       </c>
-      <c r="F13" s="1" t="s">
+      <c r="F13" s="3" t="s">
         <v>85</v>
       </c>
-      <c r="G13" s="1" t="s">
+      <c r="G13" s="3" t="s">
         <v>158</v>
       </c>
-      <c r="H13" s="1" t="s">
+      <c r="H13" s="3" t="s">
         <v>144</v>
       </c>
-      <c r="I13" s="1" t="s">
+      <c r="I13" s="3" t="s">
         <v>68</v>
       </c>
-      <c r="J13" s="1" t="s">
+      <c r="J13" s="3" t="s">
         <v>159</v>
       </c>
-      <c r="K13" s="1" t="s">
+      <c r="K13" s="3" t="s">
         <v>69</v>
       </c>
-      <c r="L13" s="1" t="s">
+      <c r="L13" s="3" t="s">
         <v>78</v>
       </c>
-      <c r="M13" s="1" t="s">
+      <c r="M13" s="3" t="s">
         <v>160</v>
       </c>
-      <c r="N13" s="1" t="s">
+      <c r="N13" s="3" t="s">
         <v>161</v>
       </c>
-      <c r="O13" s="1" t="s">
+      <c r="O13" s="3" t="s">
         <v>162</v>
       </c>
     </row>
-    <row r="14" spans="1:16" ht="290.39999999999998">
-      <c r="A14" s="1" t="s">
+    <row r="14" spans="1:16" s="4" customFormat="1" ht="290.39999999999998">
+      <c r="A14" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="B14" s="1" t="s">
+      <c r="B14" s="3" t="s">
         <v>163</v>
       </c>
-      <c r="C14" s="1" t="s">
+      <c r="C14" s="3" t="s">
         <v>164</v>
       </c>
-      <c r="D14" s="1" t="s">
+      <c r="D14" s="3" t="s">
         <v>165</v>
       </c>
-      <c r="E14" s="1" t="s">
+      <c r="E14" s="3" t="s">
         <v>78</v>
       </c>
-      <c r="F14" s="1" t="s">
+      <c r="F14" s="3" t="s">
         <v>166</v>
       </c>
-      <c r="G14" s="1" t="s">
+      <c r="G14" s="3" t="s">
         <v>78</v>
       </c>
-      <c r="H14" s="1" t="s">
+      <c r="H14" s="3" t="s">
         <v>167</v>
       </c>
-      <c r="I14" s="1" t="s">
+      <c r="I14" s="3" t="s">
         <v>329</v>
       </c>
-      <c r="J14" s="1" t="s">
+      <c r="J14" s="3" t="s">
         <v>168</v>
       </c>
-      <c r="K14" s="1" t="s">
+      <c r="K14" s="3" t="s">
         <v>69</v>
       </c>
-      <c r="L14" s="1" t="s">
+      <c r="L14" s="3" t="s">
         <v>78</v>
       </c>
-      <c r="M14" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="N14" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="O14" s="1" t="s">
+      <c r="M14" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="N14" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="O14" s="3" t="s">
         <v>169</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update figures and data extraction files
- Modified the universal approximation demo SVG and PDF files to adjust dimensions and improve rendering.
- Updated the Individual AnnotationsORC.xlsx file with new data.
- Removed temporary file ~\$Individual AnnotationsORC.xlsx.
</commit_message>
<xml_diff>
--- a/main/04_data_extraction/Individual AnnotationsORC.xlsx
+++ b/main/04_data_extraction/Individual AnnotationsORC.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\orincon\scoping-ml-wave-seismology\main\04_data_extraction\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D81D38E5-8546-4A2C-96DC-1BA9017EB71E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8DBC3A76-1326-489B-9828-D39BBF03E9F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{115BB8D9-8B86-4726-97F8-E06477FD353D}"/>
   </bookViews>
@@ -2904,50 +2904,50 @@
         <v>299</v>
       </c>
     </row>
-    <row r="18" spans="1:16" ht="379.5" customHeight="1">
-      <c r="A18" s="1" t="s">
+    <row r="18" spans="1:16" s="4" customFormat="1" ht="379.5" customHeight="1">
+      <c r="A18" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="B18" s="1" t="s">
+      <c r="B18" s="3" t="s">
         <v>179</v>
       </c>
-      <c r="C18" s="1" t="s">
+      <c r="C18" s="3" t="s">
         <v>180</v>
       </c>
-      <c r="D18" s="1" t="s">
+      <c r="D18" s="3" t="s">
         <v>181</v>
       </c>
-      <c r="E18" s="1" t="s">
+      <c r="E18" s="3" t="s">
         <v>182</v>
       </c>
-      <c r="F18" s="1" t="s">
+      <c r="F18" s="3" t="s">
         <v>183</v>
       </c>
-      <c r="G18" s="1" t="s">
+      <c r="G18" s="3" t="s">
         <v>78</v>
       </c>
-      <c r="H18" s="1" t="s">
+      <c r="H18" s="3" t="s">
         <v>184</v>
       </c>
-      <c r="I18" s="1" t="s">
+      <c r="I18" s="3" t="s">
         <v>185</v>
       </c>
-      <c r="J18" s="1" t="s">
+      <c r="J18" s="3" t="s">
         <v>186</v>
       </c>
-      <c r="K18" s="1" t="s">
+      <c r="K18" s="3" t="s">
         <v>187</v>
       </c>
-      <c r="L18" s="1" t="s">
+      <c r="L18" s="3" t="s">
         <v>188</v>
       </c>
-      <c r="M18" s="1" t="s">
+      <c r="M18" s="3" t="s">
         <v>189</v>
       </c>
-      <c r="N18" s="1" t="s">
+      <c r="N18" s="3" t="s">
         <v>190</v>
       </c>
-      <c r="O18" s="1" t="s">
+      <c r="O18" s="3" t="s">
         <v>66</v>
       </c>
     </row>
@@ -3001,50 +3001,50 @@
         <v>203</v>
       </c>
     </row>
-    <row r="20" spans="1:16" ht="409.6">
-      <c r="A20" s="1" t="s">
+    <row r="20" spans="1:16" s="4" customFormat="1" ht="409.6">
+      <c r="A20" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="B20" s="1" t="s">
+      <c r="B20" s="3" t="s">
         <v>204</v>
       </c>
-      <c r="C20" s="1" t="s">
+      <c r="C20" s="3" t="s">
         <v>205</v>
       </c>
-      <c r="D20" s="1" t="s">
+      <c r="D20" s="3" t="s">
         <v>206</v>
       </c>
-      <c r="E20" s="1" t="s">
+      <c r="E20" s="3" t="s">
         <v>78</v>
       </c>
-      <c r="F20" s="1" t="s">
+      <c r="F20" s="3" t="s">
         <v>85</v>
       </c>
-      <c r="G20" s="1" t="s">
+      <c r="G20" s="3" t="s">
         <v>78</v>
       </c>
-      <c r="H20" s="1" t="s">
+      <c r="H20" s="3" t="s">
         <v>78</v>
       </c>
-      <c r="I20" s="1" t="s">
+      <c r="I20" s="3" t="s">
         <v>68</v>
       </c>
-      <c r="J20" s="1" t="s">
+      <c r="J20" s="3" t="s">
         <v>207</v>
       </c>
-      <c r="K20" s="1" t="s">
+      <c r="K20" s="3" t="s">
         <v>77</v>
       </c>
-      <c r="L20" s="1" t="s">
+      <c r="L20" s="3" t="s">
         <v>78</v>
       </c>
-      <c r="M20" s="1" t="s">
+      <c r="M20" s="3" t="s">
         <v>95</v>
       </c>
-      <c r="N20" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="O20" s="1" t="s">
+      <c r="N20" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="O20" s="3" t="s">
         <v>208</v>
       </c>
     </row>
@@ -3148,51 +3148,51 @@
         <v>328</v>
       </c>
     </row>
-    <row r="23" spans="1:16" ht="250.8">
-      <c r="A23" s="1" t="s">
+    <row r="23" spans="1:16" s="4" customFormat="1" ht="250.8">
+      <c r="A23" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="B23" s="1" t="s">
+      <c r="B23" s="3" t="s">
         <v>209</v>
       </c>
-      <c r="C23" s="1" t="s">
+      <c r="C23" s="3" t="s">
         <v>210</v>
       </c>
-      <c r="D23" s="1" t="s">
+      <c r="D23" s="3" t="s">
         <v>211</v>
       </c>
-      <c r="E23" s="1" t="s">
+      <c r="E23" s="3" t="s">
         <v>135</v>
       </c>
-      <c r="F23" s="1" t="s">
+      <c r="F23" s="3" t="s">
         <v>212</v>
       </c>
-      <c r="G23" s="1" t="s">
+      <c r="G23" s="3" t="s">
         <v>212</v>
       </c>
-      <c r="H23" s="1" t="s">
+      <c r="H23" s="3" t="s">
         <v>213</v>
       </c>
-      <c r="I23" s="1" t="s">
+      <c r="I23" s="3" t="s">
         <v>67</v>
       </c>
-      <c r="J23" s="1" t="s">
+      <c r="J23" s="3" t="s">
         <v>214</v>
       </c>
-      <c r="K23" s="1" t="s">
+      <c r="K23" s="3" t="s">
         <v>77</v>
       </c>
-      <c r="L23" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="M23" s="1" t="s">
+      <c r="L23" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="M23" s="3" t="s">
         <v>215</v>
       </c>
-      <c r="N23" s="1"/>
-      <c r="O23" s="1" t="s">
+      <c r="N23" s="3"/>
+      <c r="O23" s="3" t="s">
         <v>216</v>
       </c>
-      <c r="P23" s="1" t="s">
+      <c r="P23" s="3" t="s">
         <v>217</v>
       </c>
     </row>
@@ -4312,12 +4312,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x01010009048CEEA230F14796749F6DFD5F5263" ma:contentTypeVersion="4" ma:contentTypeDescription="Crear nuevo documento." ma:contentTypeScope="" ma:versionID="5105af4e7c1b0ed6cdb04338eaf51f7a">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="96457c7a-bdfc-427e-9d05-5faa5ab5244b" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="0baee1a300280ca08e7397f1756276d6" ns2:_="">
     <xsd:import namespace="96457c7a-bdfc-427e-9d05-5faa5ab5244b"/>
@@ -4461,6 +4455,12 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
@@ -4471,15 +4471,6 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1160EB8C-E200-4916-A3B3-9BF8115D37F8}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{75ADFBF6-8C74-4292-833E-68A026E87063}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -4497,6 +4488,15 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1160EB8C-E200-4916-A3B3-9BF8115D37F8}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{24F2579D-323E-48EA-8FED-D372AFFF0A04}">
   <ds:schemaRefs>

</xml_diff>

<commit_message>
Update Individual AnnotationsORC.xlsx with new data
</commit_message>
<xml_diff>
--- a/main/04_data_extraction/Individual AnnotationsORC.xlsx
+++ b/main/04_data_extraction/Individual AnnotationsORC.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\orincon\scoping-ml-wave-seismology\main\04_data_extraction\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8DBC3A76-1326-489B-9828-D39BBF03E9F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DDD15176-2129-4954-9E2A-153DB8BED907}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{115BB8D9-8B86-4726-97F8-E06477FD353D}"/>
   </bookViews>
@@ -1670,7 +1670,7 @@
       <family val="1"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1680,12 +1680,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFF00"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFC000"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1723,7 +1717,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1746,19 +1740,13 @@
     <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -2124,39 +2112,39 @@
   <sheetData>
     <row r="1" spans="1:16" ht="15" customHeight="1">
       <c r="A1" s="1"/>
-      <c r="B1" s="14" t="s">
+      <c r="B1" s="12" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="14" t="s">
+      <c r="C1" s="12" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="14"/>
-      <c r="E1" s="14"/>
-      <c r="F1" s="14" t="s">
+      <c r="D1" s="12"/>
+      <c r="E1" s="12"/>
+      <c r="F1" s="12" t="s">
         <v>2</v>
       </c>
-      <c r="G1" s="14"/>
+      <c r="G1" s="12"/>
       <c r="H1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="I1" s="14" t="s">
+      <c r="I1" s="12" t="s">
         <v>4</v>
       </c>
-      <c r="J1" s="14"/>
-      <c r="K1" s="14" t="s">
+      <c r="J1" s="12"/>
+      <c r="K1" s="12" t="s">
         <v>5</v>
       </c>
-      <c r="L1" s="14"/>
-      <c r="M1" s="14" t="s">
+      <c r="L1" s="12"/>
+      <c r="M1" s="12" t="s">
         <v>6</v>
       </c>
-      <c r="N1" s="14" t="s">
+      <c r="N1" s="12" t="s">
         <v>7</v>
       </c>
-      <c r="O1" s="14" t="s">
+      <c r="O1" s="12" t="s">
         <v>8</v>
       </c>
-      <c r="P1" s="13" t="s">
+      <c r="P1" s="11" t="s">
         <v>390</v>
       </c>
     </row>
@@ -2164,7 +2152,7 @@
       <c r="A2" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="B2" s="14"/>
+      <c r="B2" s="12"/>
       <c r="C2" s="2" t="s">
         <v>10</v>
       </c>
@@ -2195,10 +2183,10 @@
       <c r="L2" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="M2" s="14"/>
-      <c r="N2" s="14"/>
-      <c r="O2" s="14"/>
-      <c r="P2" s="13"/>
+      <c r="M2" s="12"/>
+      <c r="N2" s="12"/>
+      <c r="O2" s="12"/>
+      <c r="P2" s="11"/>
     </row>
     <row r="3" spans="1:16" s="4" customFormat="1" ht="250.8">
       <c r="A3" s="3" t="s">
@@ -3296,145 +3284,145 @@
         <v>362</v>
       </c>
     </row>
-    <row r="26" spans="1:16" ht="184.8">
-      <c r="A26" s="1" t="s">
+    <row r="26" spans="1:16" s="4" customFormat="1" ht="184.8">
+      <c r="A26" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="B26" s="1" t="s">
+      <c r="B26" s="3" t="s">
         <v>394</v>
       </c>
-      <c r="C26" s="1" t="s">
+      <c r="C26" s="3" t="s">
         <v>218</v>
       </c>
-      <c r="D26" s="1" t="s">
+      <c r="D26" s="3" t="s">
         <v>219</v>
       </c>
-      <c r="E26" s="1" t="s">
+      <c r="E26" s="3" t="s">
         <v>220</v>
       </c>
-      <c r="F26" s="1" t="s">
+      <c r="F26" s="3" t="s">
         <v>384</v>
       </c>
-      <c r="G26" s="1" t="s">
+      <c r="G26" s="3" t="s">
         <v>212</v>
       </c>
-      <c r="H26" s="1" t="s">
+      <c r="H26" s="3" t="s">
         <v>221</v>
       </c>
-      <c r="I26" s="1" t="s">
+      <c r="I26" s="3" t="s">
         <v>68</v>
       </c>
-      <c r="J26" s="1" t="s">
+      <c r="J26" s="3" t="s">
         <v>78</v>
       </c>
-      <c r="K26" s="1" t="s">
+      <c r="K26" s="3" t="s">
         <v>77</v>
       </c>
-      <c r="L26" s="1" t="s">
+      <c r="L26" s="3" t="s">
         <v>78</v>
       </c>
-      <c r="M26" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="N26" s="1"/>
-      <c r="O26" s="1" t="s">
+      <c r="M26" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="N26" s="3"/>
+      <c r="O26" s="3" t="s">
         <v>222</v>
       </c>
     </row>
-    <row r="27" spans="1:16" s="9" customFormat="1" ht="132">
-      <c r="A27" s="8" t="s">
+    <row r="27" spans="1:16" s="4" customFormat="1" ht="132">
+      <c r="A27" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="B27" s="8" t="s">
+      <c r="B27" s="3" t="s">
         <v>380</v>
       </c>
-      <c r="C27" s="8" t="s">
+      <c r="C27" s="3" t="s">
         <v>381</v>
       </c>
-      <c r="D27" s="8" t="s">
+      <c r="D27" s="3" t="s">
         <v>382</v>
       </c>
-      <c r="E27" s="8" t="s">
+      <c r="E27" s="3" t="s">
         <v>383</v>
       </c>
-      <c r="F27" s="8" t="s">
+      <c r="F27" s="3" t="s">
         <v>384</v>
       </c>
-      <c r="G27" s="8" t="s">
+      <c r="G27" s="3" t="s">
         <v>212</v>
       </c>
-      <c r="H27" s="8" t="s">
+      <c r="H27" s="3" t="s">
         <v>385</v>
       </c>
-      <c r="I27" s="8" t="s">
+      <c r="I27" s="3" t="s">
         <v>257</v>
       </c>
-      <c r="J27" s="8" t="s">
+      <c r="J27" s="3" t="s">
         <v>78</v>
       </c>
-      <c r="K27" s="8" t="s">
+      <c r="K27" s="3" t="s">
         <v>386</v>
       </c>
-      <c r="L27" s="8" t="s">
+      <c r="L27" s="3" t="s">
         <v>387</v>
       </c>
-      <c r="M27" s="8" t="s">
+      <c r="M27" s="3" t="s">
         <v>388</v>
       </c>
-      <c r="N27" s="8" t="s">
+      <c r="N27" s="3" t="s">
         <v>393</v>
       </c>
-      <c r="O27" s="8" t="s">
+      <c r="O27" s="3" t="s">
         <v>389</v>
       </c>
-      <c r="P27" s="9" t="s">
+      <c r="P27" s="4" t="s">
         <v>392</v>
       </c>
     </row>
-    <row r="28" spans="1:16" ht="224.4">
-      <c r="A28" s="1" t="s">
+    <row r="28" spans="1:16" s="4" customFormat="1" ht="224.4">
+      <c r="A28" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="B28" s="1" t="s">
+      <c r="B28" s="3" t="s">
         <v>223</v>
       </c>
-      <c r="C28" s="1" t="s">
+      <c r="C28" s="3" t="s">
         <v>224</v>
       </c>
-      <c r="D28" s="1" t="s">
+      <c r="D28" s="3" t="s">
         <v>225</v>
       </c>
-      <c r="E28" s="1" t="s">
+      <c r="E28" s="3" t="s">
         <v>226</v>
       </c>
-      <c r="F28" s="1" t="s">
+      <c r="F28" s="3" t="s">
         <v>227</v>
       </c>
-      <c r="G28" s="1" t="s">
+      <c r="G28" s="3" t="s">
         <v>228</v>
       </c>
-      <c r="H28" s="1" t="s">
+      <c r="H28" s="3" t="s">
         <v>229</v>
       </c>
-      <c r="I28" s="1" t="s">
+      <c r="I28" s="3" t="s">
         <v>230</v>
       </c>
-      <c r="J28" s="1" t="s">
+      <c r="J28" s="3" t="s">
         <v>231</v>
       </c>
-      <c r="K28" s="1" t="s">
+      <c r="K28" s="3" t="s">
         <v>232</v>
       </c>
-      <c r="L28" s="1" t="s">
+      <c r="L28" s="3" t="s">
         <v>233</v>
       </c>
-      <c r="M28" s="1" t="s">
+      <c r="M28" s="3" t="s">
         <v>234</v>
       </c>
-      <c r="N28" s="1" t="s">
+      <c r="N28" s="3" t="s">
         <v>235</v>
       </c>
-      <c r="O28" s="1" t="s">
+      <c r="O28" s="3" t="s">
         <v>236</v>
       </c>
     </row>
@@ -3588,53 +3576,53 @@
         <v>287</v>
       </c>
     </row>
-    <row r="32" spans="1:16" ht="105.6">
-      <c r="A32" s="1" t="s">
+    <row r="32" spans="1:16" s="4" customFormat="1" ht="105.6">
+      <c r="A32" s="3" t="s">
         <v>48</v>
       </c>
-      <c r="B32" s="1" t="s">
+      <c r="B32" s="3" t="s">
         <v>366</v>
       </c>
-      <c r="C32" s="1" t="s">
+      <c r="C32" s="3" t="s">
         <v>367</v>
       </c>
-      <c r="D32" s="1" t="s">
+      <c r="D32" s="3" t="s">
         <v>368</v>
       </c>
-      <c r="E32" s="1" t="s">
+      <c r="E32" s="3" t="s">
         <v>369</v>
       </c>
-      <c r="F32" s="1" t="s">
+      <c r="F32" s="3" t="s">
         <v>370</v>
       </c>
-      <c r="G32" s="1" t="s">
+      <c r="G32" s="3" t="s">
         <v>371</v>
       </c>
-      <c r="H32" s="1" t="s">
+      <c r="H32" s="3" t="s">
         <v>372</v>
       </c>
-      <c r="I32" s="1" t="s">
+      <c r="I32" s="3" t="s">
         <v>295</v>
       </c>
-      <c r="J32" s="1" t="s">
+      <c r="J32" s="3" t="s">
         <v>373</v>
       </c>
-      <c r="K32" s="1" t="s">
+      <c r="K32" s="3" t="s">
         <v>374</v>
       </c>
-      <c r="L32" s="1" t="s">
+      <c r="L32" s="3" t="s">
         <v>375</v>
       </c>
-      <c r="M32" s="1" t="s">
+      <c r="M32" s="3" t="s">
         <v>376</v>
       </c>
-      <c r="N32" s="1" t="s">
+      <c r="N32" s="3" t="s">
         <v>377</v>
       </c>
-      <c r="O32" s="1" t="s">
+      <c r="O32" s="3" t="s">
         <v>378</v>
       </c>
-      <c r="P32" s="5" t="s">
+      <c r="P32" s="4" t="s">
         <v>379</v>
       </c>
     </row>
@@ -3746,7 +3734,7 @@
       <c r="D35" s="1" t="s">
         <v>410</v>
       </c>
-      <c r="E35" s="10" t="s">
+      <c r="E35" s="8" t="s">
         <v>318</v>
       </c>
       <c r="F35" s="1" t="s">
@@ -3883,48 +3871,48 @@
         <v>442</v>
       </c>
     </row>
-    <row r="38" spans="1:16" s="12" customFormat="1">
-      <c r="A38" s="11" t="s">
+    <row r="38" spans="1:16" s="10" customFormat="1">
+      <c r="A38" s="9" t="s">
         <v>54</v>
       </c>
-      <c r="B38" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="C38" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="D38" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="E38" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="F38" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="G38" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="H38" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="I38" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="J38" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="K38" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="L38" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="M38" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="N38" s="11"/>
-      <c r="O38" s="11" t="s">
+      <c r="B38" s="9" t="s">
+        <v>66</v>
+      </c>
+      <c r="C38" s="9" t="s">
+        <v>66</v>
+      </c>
+      <c r="D38" s="9" t="s">
+        <v>66</v>
+      </c>
+      <c r="E38" s="9" t="s">
+        <v>66</v>
+      </c>
+      <c r="F38" s="9" t="s">
+        <v>66</v>
+      </c>
+      <c r="G38" s="9" t="s">
+        <v>66</v>
+      </c>
+      <c r="H38" s="9" t="s">
+        <v>66</v>
+      </c>
+      <c r="I38" s="9" t="s">
+        <v>66</v>
+      </c>
+      <c r="J38" s="9" t="s">
+        <v>66</v>
+      </c>
+      <c r="K38" s="9" t="s">
+        <v>66</v>
+      </c>
+      <c r="L38" s="9" t="s">
+        <v>66</v>
+      </c>
+      <c r="M38" s="9" t="s">
+        <v>66</v>
+      </c>
+      <c r="N38" s="9"/>
+      <c r="O38" s="9" t="s">
         <v>66</v>
       </c>
     </row>
@@ -4312,6 +4300,12 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x01010009048CEEA230F14796749F6DFD5F5263" ma:contentTypeVersion="4" ma:contentTypeDescription="Crear nuevo documento." ma:contentTypeScope="" ma:versionID="5105af4e7c1b0ed6cdb04338eaf51f7a">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="96457c7a-bdfc-427e-9d05-5faa5ab5244b" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="0baee1a300280ca08e7397f1756276d6" ns2:_="">
     <xsd:import namespace="96457c7a-bdfc-427e-9d05-5faa5ab5244b"/>
@@ -4455,12 +4449,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
@@ -4471,6 +4459,15 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1160EB8C-E200-4916-A3B3-9BF8115D37F8}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{75ADFBF6-8C74-4292-833E-68A026E87063}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -4488,15 +4485,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1160EB8C-E200-4916-A3B3-9BF8115D37F8}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{24F2579D-323E-48EA-8FED-D372AFFF0A04}">
   <ds:schemaRefs>

</xml_diff>

<commit_message>
Add temporary files for Campos et al. (2019) and Individual AnnotationsORC
</commit_message>
<xml_diff>
--- a/main/04_data_extraction/Individual AnnotationsORC.xlsx
+++ b/main/04_data_extraction/Individual AnnotationsORC.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\orincon\scoping-ml-wave-seismology\main\04_data_extraction\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DDD15176-2129-4954-9E2A-153DB8BED907}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B247EDC1-DDC5-429F-AE82-DB1C2571CF85}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{115BB8D9-8B86-4726-97F8-E06477FD353D}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="685" uniqueCount="443">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="687" uniqueCount="453">
   <si>
     <t>Lectura general</t>
   </si>
@@ -1606,6 +1606,40 @@
   </si>
   <si>
     <t xml:space="preserve"> Correlation coefficient (time-domain)</t>
+  </si>
+  <si>
+    <t>1. Research prototype
+2. FWI and  inverse Hessian for seismic imaging
+3. The asume scattered wavefields are small relative to the background wavefield. This is a standard linearization in seismic imaging and is clearly stated 
+4. A neural network trained to approximate the action of the inverse Hessian 
+5. The theoretical derivation connecting Born modeling to the Hessian approximation is rigorous </t>
+  </si>
+  <si>
+    <t>U-Net </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> U-Net is well suited for domain translation tasks where input and output share the same spatial resolution </t>
+  </si>
+  <si>
+    <t>PyTorch </t>
+  </si>
+  <si>
+    <t>FD </t>
+  </si>
+  <si>
+    <t> Both</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> The acoustic assumption simplifies the forward problem but limits applicability </t>
+  </si>
+  <si>
+    <t>The finite-difference solver handles all wave propagation, while the neural network learns to correct the FWI gradient by approximating the inverse Hessian. </t>
+  </si>
+  <si>
+    <t>Improving the model update direction by approximating the inverse Hessian, which conventionally requires prohibitive computation. </t>
+  </si>
+  <si>
+    <t>Visual comparison of inverted velocity models</t>
   </si>
 </sst>
 </file>
@@ -1740,9 +1774,6 @@
     <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1754,6 +1785,9 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2112,39 +2146,39 @@
   <sheetData>
     <row r="1" spans="1:16" ht="15" customHeight="1">
       <c r="A1" s="1"/>
-      <c r="B1" s="12" t="s">
+      <c r="B1" s="11" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="12" t="s">
+      <c r="C1" s="11" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="12"/>
-      <c r="E1" s="12"/>
-      <c r="F1" s="12" t="s">
+      <c r="D1" s="11"/>
+      <c r="E1" s="11"/>
+      <c r="F1" s="11" t="s">
         <v>2</v>
       </c>
-      <c r="G1" s="12"/>
+      <c r="G1" s="11"/>
       <c r="H1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="I1" s="12" t="s">
+      <c r="I1" s="11" t="s">
         <v>4</v>
       </c>
-      <c r="J1" s="12"/>
-      <c r="K1" s="12" t="s">
+      <c r="J1" s="11"/>
+      <c r="K1" s="11" t="s">
         <v>5</v>
       </c>
-      <c r="L1" s="12"/>
-      <c r="M1" s="12" t="s">
+      <c r="L1" s="11"/>
+      <c r="M1" s="11" t="s">
         <v>6</v>
       </c>
-      <c r="N1" s="12" t="s">
+      <c r="N1" s="11" t="s">
         <v>7</v>
       </c>
-      <c r="O1" s="12" t="s">
+      <c r="O1" s="11" t="s">
         <v>8</v>
       </c>
-      <c r="P1" s="11" t="s">
+      <c r="P1" s="10" t="s">
         <v>390</v>
       </c>
     </row>
@@ -2152,7 +2186,7 @@
       <c r="A2" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="B2" s="12"/>
+      <c r="B2" s="11"/>
       <c r="C2" s="2" t="s">
         <v>10</v>
       </c>
@@ -2183,10 +2217,10 @@
       <c r="L2" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="M2" s="12"/>
-      <c r="N2" s="12"/>
-      <c r="O2" s="12"/>
-      <c r="P2" s="11"/>
+      <c r="M2" s="11"/>
+      <c r="N2" s="11"/>
+      <c r="O2" s="11"/>
+      <c r="P2" s="10"/>
     </row>
     <row r="3" spans="1:16" s="4" customFormat="1" ht="250.8">
       <c r="A3" s="3" t="s">
@@ -3086,7 +3120,7 @@
         <v>314</v>
       </c>
     </row>
-    <row r="22" spans="1:16" s="4" customFormat="1" ht="158.4">
+    <row r="22" spans="1:16" s="4" customFormat="1" ht="189" customHeight="1">
       <c r="A22" s="3" t="s">
         <v>39</v>
       </c>
@@ -3626,383 +3660,388 @@
         <v>379</v>
       </c>
     </row>
-    <row r="33" spans="1:16" ht="290.39999999999998">
-      <c r="A33" s="1" t="s">
+    <row r="33" spans="1:16" s="4" customFormat="1" ht="290.39999999999998">
+      <c r="A33" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="B33" s="1" t="s">
+      <c r="B33" s="3" t="s">
         <v>252</v>
       </c>
-      <c r="C33" s="1" t="s">
+      <c r="C33" s="3" t="s">
         <v>253</v>
       </c>
-      <c r="D33" s="1" t="s">
+      <c r="D33" s="3" t="s">
         <v>254</v>
       </c>
-      <c r="E33" s="1" t="s">
+      <c r="E33" s="3" t="s">
         <v>78</v>
       </c>
-      <c r="F33" s="1" t="s">
+      <c r="F33" s="3" t="s">
         <v>255</v>
       </c>
-      <c r="G33" s="1" t="s">
+      <c r="G33" s="3" t="s">
         <v>212</v>
       </c>
-      <c r="H33" s="1" t="s">
+      <c r="H33" s="3" t="s">
         <v>256</v>
       </c>
-      <c r="I33" s="1" t="s">
+      <c r="I33" s="3" t="s">
         <v>257</v>
       </c>
-      <c r="J33" s="1" t="s">
+      <c r="J33" s="3" t="s">
         <v>258</v>
       </c>
-      <c r="K33" s="1" t="s">
+      <c r="K33" s="3" t="s">
         <v>259</v>
       </c>
-      <c r="L33" s="1" t="s">
+      <c r="L33" s="3" t="s">
         <v>212</v>
       </c>
-      <c r="M33" s="1" t="s">
+      <c r="M33" s="3" t="s">
         <v>260</v>
       </c>
-      <c r="N33" s="1" t="s">
+      <c r="N33" s="3" t="s">
         <v>261</v>
       </c>
-      <c r="O33" s="1"/>
+      <c r="O33" s="3"/>
     </row>
-    <row r="34" spans="1:16" ht="105.6">
-      <c r="A34" s="1" t="s">
+    <row r="34" spans="1:16" s="4" customFormat="1" ht="120" customHeight="1">
+      <c r="A34" s="3" t="s">
         <v>50</v>
       </c>
-      <c r="B34" s="1" t="s">
+      <c r="B34" s="3" t="s">
         <v>395</v>
       </c>
-      <c r="C34" s="1" t="s">
+      <c r="C34" s="3" t="s">
         <v>396</v>
       </c>
-      <c r="D34" s="1" t="s">
+      <c r="D34" s="3" t="s">
         <v>397</v>
       </c>
-      <c r="E34" s="1" t="s">
+      <c r="E34" s="3" t="s">
         <v>397</v>
       </c>
-      <c r="F34" s="1" t="s">
+      <c r="F34" s="3" t="s">
         <v>85</v>
       </c>
-      <c r="G34" s="1" t="s">
+      <c r="G34" s="3" t="s">
         <v>399</v>
       </c>
-      <c r="H34" s="1" t="s">
+      <c r="H34" s="3" t="s">
         <v>385</v>
       </c>
-      <c r="I34" s="1" t="s">
+      <c r="I34" s="3" t="s">
         <v>400</v>
       </c>
-      <c r="J34" s="1" t="s">
+      <c r="J34" s="3" t="s">
         <v>401</v>
       </c>
-      <c r="K34" s="1" t="s">
+      <c r="K34" s="3" t="s">
         <v>402</v>
       </c>
-      <c r="L34" s="1" t="s">
+      <c r="L34" s="3" t="s">
         <v>403</v>
       </c>
-      <c r="M34" s="1" t="s">
+      <c r="M34" s="3" t="s">
         <v>404</v>
       </c>
-      <c r="N34" s="1" t="s">
+      <c r="N34" s="3" t="s">
         <v>405</v>
       </c>
-      <c r="O34" s="1" t="s">
+      <c r="O34" s="3" t="s">
         <v>406</v>
       </c>
-      <c r="P34" s="5" t="s">
+      <c r="P34" s="4" t="s">
         <v>407</v>
       </c>
     </row>
-    <row r="35" spans="1:16" ht="79.2">
-      <c r="A35" s="1" t="s">
+    <row r="35" spans="1:16" s="4" customFormat="1" ht="79.2">
+      <c r="A35" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="B35" s="1" t="s">
+      <c r="B35" s="3" t="s">
         <v>408</v>
       </c>
-      <c r="C35" s="1" t="s">
+      <c r="C35" s="3" t="s">
         <v>409</v>
       </c>
-      <c r="D35" s="1" t="s">
+      <c r="D35" s="3" t="s">
         <v>410</v>
       </c>
-      <c r="E35" s="8" t="s">
+      <c r="E35" s="12" t="s">
         <v>318</v>
       </c>
-      <c r="F35" s="1" t="s">
+      <c r="F35" s="3" t="s">
         <v>411</v>
       </c>
-      <c r="G35" s="1" t="s">
+      <c r="G35" s="3" t="s">
         <v>398</v>
       </c>
-      <c r="H35" s="1" t="s">
+      <c r="H35" s="3" t="s">
         <v>412</v>
       </c>
-      <c r="I35" s="1" t="s">
+      <c r="I35" s="3" t="s">
         <v>413</v>
       </c>
-      <c r="J35" s="1" t="s">
+      <c r="J35" s="3" t="s">
         <v>414</v>
       </c>
-      <c r="K35" s="1" t="s">
+      <c r="K35" s="3" t="s">
         <v>402</v>
       </c>
-      <c r="L35" s="1" t="s">
+      <c r="L35" s="3" t="s">
         <v>269</v>
       </c>
-      <c r="M35" s="1" t="s">
+      <c r="M35" s="3" t="s">
         <v>415</v>
       </c>
-      <c r="N35" s="1" t="s">
+      <c r="N35" s="3" t="s">
         <v>416</v>
       </c>
-      <c r="O35" s="1" t="s">
+      <c r="O35" s="3" t="s">
         <v>417</v>
       </c>
-      <c r="P35" s="5" t="s">
+      <c r="P35" s="4" t="s">
         <v>418</v>
       </c>
     </row>
-    <row r="36" spans="1:16" ht="92.4">
-      <c r="A36" s="1" t="s">
+    <row r="36" spans="1:16" s="4" customFormat="1" ht="92.4">
+      <c r="A36" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="B36" s="1" t="s">
+      <c r="B36" s="3" t="s">
         <v>419</v>
       </c>
-      <c r="C36" s="1" t="s">
+      <c r="C36" s="3" t="s">
         <v>420</v>
       </c>
-      <c r="D36" s="1" t="s">
+      <c r="D36" s="3" t="s">
         <v>421</v>
       </c>
-      <c r="E36" s="1" t="s">
+      <c r="E36" s="3" t="s">
         <v>422</v>
       </c>
-      <c r="F36" s="1" t="s">
+      <c r="F36" s="3" t="s">
         <v>411</v>
       </c>
-      <c r="G36" s="1" t="s">
+      <c r="G36" s="3" t="s">
         <v>398</v>
       </c>
-      <c r="H36" s="1" t="s">
+      <c r="H36" s="3" t="s">
         <v>423</v>
       </c>
-      <c r="I36" s="1" t="s">
+      <c r="I36" s="3" t="s">
         <v>257</v>
       </c>
-      <c r="J36" s="1" t="s">
+      <c r="J36" s="3" t="s">
         <v>424</v>
       </c>
-      <c r="K36" s="1" t="s">
+      <c r="K36" s="3" t="s">
         <v>402</v>
       </c>
-      <c r="L36" s="1" t="s">
+      <c r="L36" s="3" t="s">
         <v>425</v>
       </c>
-      <c r="M36" s="1" t="s">
+      <c r="M36" s="3" t="s">
         <v>426</v>
       </c>
-      <c r="N36" s="1" t="s">
+      <c r="N36" s="3" t="s">
         <v>427</v>
       </c>
-      <c r="O36" s="1" t="s">
+      <c r="O36" s="3" t="s">
         <v>428</v>
       </c>
-      <c r="P36" s="5" t="s">
+      <c r="P36" s="4" t="s">
         <v>429</v>
       </c>
     </row>
-    <row r="37" spans="1:16" ht="79.2">
-      <c r="A37" s="1" t="s">
+    <row r="37" spans="1:16" s="4" customFormat="1" ht="79.2">
+      <c r="A37" s="3" t="s">
         <v>53</v>
       </c>
-      <c r="B37" s="1" t="s">
+      <c r="B37" s="3" t="s">
         <v>430</v>
       </c>
-      <c r="C37" s="1" t="s">
+      <c r="C37" s="3" t="s">
         <v>431</v>
       </c>
-      <c r="D37" s="1" t="s">
+      <c r="D37" s="3" t="s">
         <v>432</v>
       </c>
-      <c r="E37" s="1" t="s">
+      <c r="E37" s="3" t="s">
         <v>397</v>
       </c>
-      <c r="F37" s="1" t="s">
+      <c r="F37" s="3" t="s">
         <v>434</v>
       </c>
-      <c r="G37" s="1" t="s">
+      <c r="G37" s="3" t="s">
         <v>433</v>
       </c>
-      <c r="H37" s="1" t="s">
+      <c r="H37" s="3" t="s">
         <v>333</v>
       </c>
-      <c r="I37" s="1" t="s">
+      <c r="I37" s="3" t="s">
         <v>435</v>
       </c>
-      <c r="J37" s="1" t="s">
+      <c r="J37" s="3" t="s">
         <v>436</v>
       </c>
-      <c r="K37" s="1" t="s">
+      <c r="K37" s="3" t="s">
         <v>437</v>
       </c>
-      <c r="L37" s="1" t="s">
+      <c r="L37" s="3" t="s">
         <v>438</v>
       </c>
-      <c r="M37" s="1" t="s">
+      <c r="M37" s="3" t="s">
         <v>439</v>
       </c>
-      <c r="N37" s="1" t="s">
+      <c r="N37" s="3" t="s">
         <v>440</v>
       </c>
-      <c r="O37" s="1" t="s">
+      <c r="O37" s="3" t="s">
         <v>441</v>
       </c>
-      <c r="P37" s="5" t="s">
+      <c r="P37" s="4" t="s">
         <v>442</v>
       </c>
     </row>
-    <row r="38" spans="1:16" s="10" customFormat="1">
-      <c r="A38" s="9" t="s">
+    <row r="38" spans="1:16" s="9" customFormat="1">
+      <c r="A38" s="8" t="s">
         <v>54</v>
       </c>
-      <c r="B38" s="9" t="s">
-        <v>66</v>
-      </c>
-      <c r="C38" s="9" t="s">
-        <v>66</v>
-      </c>
-      <c r="D38" s="9" t="s">
-        <v>66</v>
-      </c>
-      <c r="E38" s="9" t="s">
-        <v>66</v>
-      </c>
-      <c r="F38" s="9" t="s">
-        <v>66</v>
-      </c>
-      <c r="G38" s="9" t="s">
-        <v>66</v>
-      </c>
-      <c r="H38" s="9" t="s">
-        <v>66</v>
-      </c>
-      <c r="I38" s="9" t="s">
-        <v>66</v>
-      </c>
-      <c r="J38" s="9" t="s">
-        <v>66</v>
-      </c>
-      <c r="K38" s="9" t="s">
-        <v>66</v>
-      </c>
-      <c r="L38" s="9" t="s">
-        <v>66</v>
-      </c>
-      <c r="M38" s="9" t="s">
-        <v>66</v>
-      </c>
-      <c r="N38" s="9"/>
-      <c r="O38" s="9" t="s">
+      <c r="B38" s="8" t="s">
+        <v>66</v>
+      </c>
+      <c r="C38" s="8" t="s">
+        <v>66</v>
+      </c>
+      <c r="D38" s="8" t="s">
+        <v>66</v>
+      </c>
+      <c r="E38" s="8" t="s">
+        <v>66</v>
+      </c>
+      <c r="F38" s="8" t="s">
+        <v>66</v>
+      </c>
+      <c r="G38" s="8" t="s">
+        <v>66</v>
+      </c>
+      <c r="H38" s="8" t="s">
+        <v>66</v>
+      </c>
+      <c r="I38" s="8" t="s">
+        <v>66</v>
+      </c>
+      <c r="J38" s="8" t="s">
+        <v>66</v>
+      </c>
+      <c r="K38" s="8" t="s">
+        <v>66</v>
+      </c>
+      <c r="L38" s="8" t="s">
+        <v>66</v>
+      </c>
+      <c r="M38" s="8" t="s">
+        <v>66</v>
+      </c>
+      <c r="N38" s="8"/>
+      <c r="O38" s="8" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="39" spans="1:16" ht="31.2" customHeight="1">
-      <c r="A39" s="1" t="s">
+    <row r="39" spans="1:16" s="4" customFormat="1" ht="31.2" customHeight="1">
+      <c r="A39" s="3" t="s">
         <v>55</v>
       </c>
-      <c r="B39" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="C39" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="D39" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="E39" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="F39" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="G39" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="H39" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="I39" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="J39" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="K39" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="L39" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="M39" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="N39" s="1"/>
-      <c r="O39" s="1" t="s">
-        <v>66</v>
+      <c r="B39" s="3" t="s">
+        <v>443</v>
+      </c>
+      <c r="C39" s="3" t="s">
+        <v>444</v>
+      </c>
+      <c r="D39" s="3" t="s">
+        <v>445</v>
+      </c>
+      <c r="E39" s="3" t="s">
+        <v>446</v>
+      </c>
+      <c r="F39" s="3" t="s">
+        <v>447</v>
+      </c>
+      <c r="G39" s="3" t="s">
+        <v>398</v>
+      </c>
+      <c r="H39" s="3" t="s">
+        <v>448</v>
+      </c>
+      <c r="I39" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="J39" s="3" t="s">
+        <v>445</v>
+      </c>
+      <c r="K39" s="3" t="s">
+        <v>402</v>
+      </c>
+      <c r="L39" s="3" t="s">
+        <v>449</v>
+      </c>
+      <c r="M39" s="3" t="s">
+        <v>450</v>
+      </c>
+      <c r="N39" s="3" t="s">
+        <v>427</v>
+      </c>
+      <c r="O39" s="3" t="s">
+        <v>451</v>
+      </c>
+      <c r="P39" s="4" t="s">
+        <v>452</v>
       </c>
     </row>
-    <row r="40" spans="1:16">
-      <c r="A40" s="1" t="s">
+    <row r="40" spans="1:16" s="4" customFormat="1">
+      <c r="A40" s="3" t="s">
         <v>56</v>
       </c>
-      <c r="B40" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="C40" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="D40" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="E40" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="F40" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="G40" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="H40" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="I40" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="J40" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="K40" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="L40" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="M40" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="N40" s="1"/>
-      <c r="O40" s="1" t="s">
+      <c r="B40" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="C40" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="D40" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="E40" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="F40" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="G40" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="H40" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="I40" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="J40" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="K40" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="L40" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="M40" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="N40" s="3"/>
+      <c r="O40" s="3" t="s">
         <v>66</v>
       </c>
     </row>
@@ -4300,12 +4339,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x01010009048CEEA230F14796749F6DFD5F5263" ma:contentTypeVersion="4" ma:contentTypeDescription="Crear nuevo documento." ma:contentTypeScope="" ma:versionID="5105af4e7c1b0ed6cdb04338eaf51f7a">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="96457c7a-bdfc-427e-9d05-5faa5ab5244b" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="0baee1a300280ca08e7397f1756276d6" ns2:_="">
     <xsd:import namespace="96457c7a-bdfc-427e-9d05-5faa5ab5244b"/>
@@ -4449,6 +4482,12 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
@@ -4459,15 +4498,6 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1160EB8C-E200-4916-A3B3-9BF8115D37F8}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{75ADFBF6-8C74-4292-833E-68A026E87063}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -4485,6 +4515,15 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1160EB8C-E200-4916-A3B3-9BF8115D37F8}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{24F2579D-323E-48EA-8FED-D372AFFF0A04}">
   <ds:schemaRefs>

</xml_diff>

<commit_message>
Add new documents for Oscar Andres Rincon Cardeño
- Created a new Word document for the paper by Zhang et al. (2024).
- Added a new Excel file for individual annotations related to Oscar Andres Rincon Cardeño.
</commit_message>
<xml_diff>
--- a/main/04_data_extraction/Individual AnnotationsORC.xlsx
+++ b/main/04_data_extraction/Individual AnnotationsORC.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\orincon\scoping-ml-wave-seismology\main\04_data_extraction\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{404DA315-B236-4537-BDC5-B1AAEF306003}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2C2D9E4D-0D48-4F9D-827F-4551C8BCD44B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{115BB8D9-8B86-4726-97F8-E06477FD353D}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="687" uniqueCount="453">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="695" uniqueCount="498">
   <si>
     <t>Lectura general</t>
   </si>
@@ -1640,6 +1640,161 @@
   </si>
   <si>
     <t>Visual comparison of inverted velocity models</t>
+  </si>
+  <si>
+    <t> 1. Analysis of an existing system/method
+2. acoustic wave equation, finite-difference numerical methods, and standard deep learning training theory
+3. that the acoustic wave equation sufficiently represents the subsurface physics
+4. A systematic empirical study of how the number of seismic sources and peak frequency affect FCN-based velocity model estimation
+5. The paper is clearly written and well structured</t>
+  </si>
+  <si>
+    <t>  FCN avoids fully connected layers, reducing the number of parameters</t>
+  </si>
+  <si>
+    <t>FCN U-Net </t>
+  </si>
+  <si>
+    <t>  Not explicitly stated in the paper</t>
+  </si>
+  <si>
+    <t> Training time increases with the number of shots because each additional shot adds a matrix of size nt × nx to the input, directly increasing data volume</t>
+  </si>
+  <si>
+    <t> Analysis of few-shot sufficiency for larger and more complex subsurfaces</t>
+  </si>
+  <si>
+    <t>MSE (also the loss function), MAE (in m/s, providing physically interpretable velocity error), R² (coefficient of determination), Pearson correlation coefficient r, and factor of two (fac2, measuring outlier fraction).</t>
+  </si>
+  <si>
+    <t>1. Research prototype 
+2.  Bayesian uncertainty quantification
+3. Seismic data can be represented as the convolution of the source wavelet with the reflectivity series
+4. An unsupervised training strategy that eliminates the need for labeled impedance models and integration of Bayesian layers into the encoder to produce uncertainty maps
+5. The architecture is described in sufficient detail for reproduction</t>
+  </si>
+  <si>
+    <t>A 1D CNN with two parts </t>
+  </si>
+  <si>
+    <t> TensorFlow</t>
+  </si>
+  <si>
+    <t>Bayesian layers provide principled uncertainty quantification</t>
+  </si>
+  <si>
+    <t>A simplified forward model based on convolution of the wavelet with the reflectivity series is used</t>
+  </si>
+  <si>
+    <t>1D </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> The trace-by-trace operation keeps computational cost low and makes the method scalable in practice </t>
+  </si>
+  <si>
+    <t>The convolutional model is computationally very cheap and differentiable, making it straightforward to embed in a neural network training loop.</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> The physics enters through the decoder, which acts as a physics-based forward operator embedded in the training loop </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Seismic impedance inversion from poststack data</t>
+  </si>
+  <si>
+    <t> Validated only on synthetic data</t>
+  </si>
+  <si>
+    <t>Mean square error between observed and simulated seismic traces</t>
+  </si>
+  <si>
+    <t>1. Research prototype
+2. ML for low-frequency extension in the frequency-space domain
+3 . The far-field signature is assumed to be representative of the actual source
+4. Successful validation on real field data (North Viking Graben), which is uncommon in the literatura
+5. Hyperparameters are reported</t>
+  </si>
+  <si>
+    <t>  Modified U-Net</t>
+  </si>
+  <si>
+    <t>  Encoder-decoder architecture with skip connections preserves high-resolution information</t>
+  </si>
+  <si>
+    <t>2D </t>
+  </si>
+  <si>
+    <t>  The neural network acts as a frequency mapping operator from band-limited to broadband data</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Low-frequency reconstruction is framed as a preprocessing step to improve the conditioning of downstream inverse problems</t>
+  </si>
+  <si>
+    <t> Ultra-low frequencies (&lt; 5 Hz) cannot be accurately reconstructed</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Error metrics used: MSE (Mean Square Error), RMSE (Root Mean Square Error) and  MAE (Mean Absolute Error).</t>
+  </si>
+  <si>
+    <t> 1. Research prototype
+2. Automatic differentiation
+3. The RNN analogy holds under the assumption that the FDM time-stepping scheme maps directly onto a recurrent structure
+4. Reimplementation of a FDM wave equation solver as a recurrent neural network within PyTorch, enabling GPU-accelerated seismic simulation
+5. The paper is readable and the three contributions are clearly separated</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> RNN </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> The RNN formulation allows direct use of PyTorch optimizers and autodiff without modifying the physics </t>
+  </si>
+  <si>
+    <t>  Dimensionality impact is not explicitly discussed</t>
+  </si>
+  <si>
+    <t> The acoustic formulation simplifies the time-stepping structure, making the RNN analogy straightforward to implement</t>
+  </si>
+  <si>
+    <t>  Better inversion accuracy through autoencoder-regularized FWI</t>
+  </si>
+  <si>
+    <t>  FWI</t>
+  </si>
+  <si>
+    <t> Results are demonstrated only on 2D synthetic models</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Visual comparison of reconstructed velocity models</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  1. Research prototype
+2. FWI, Recurrent neural networks for time-series processing and convolutional neural networks for spatial feature extraction 
+3. Well-logging data from exactly two boreholes is assumed available
+4. A dual-encoder U-Net that integrates well-logging data and seismic waveforms as separate inputs through two independent encoders
+5. Well structured and clearly written with detailed architectural descriptions </t>
+  </si>
+  <si>
+    <t>  Two coupled networks: U-Net and RNN</t>
+  </si>
+  <si>
+    <t>  The dual-encoder design captures both large-scale velocity structure from well logs and fine-scale features from seismic waveforms</t>
+  </si>
+  <si>
+    <t>  High memory consumption of the RNN forward network is explicitly acknowledged as a practical limitation</t>
+  </si>
+  <si>
+    <t>  The constant density acoustic formulation simplifies the RNN implementation since only one wavefield component needs to be tracked</t>
+  </si>
+  <si>
+    <t> The RNN forward solver is directly coupled with the U-Net inversion subnet; the predicted velocity model from the inversion subnet is passed as input to the RNN solver during training</t>
+  </si>
+  <si>
+    <t> Seismic velocity inversion</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  High memory consumption of the RNN forward network during joint training </t>
+  </si>
+  <si>
+    <t>Error metrics used: MSE (Mean Square Error), MAE (Mean Absolute Error) and SSIM (Structural Similarity Index) — used both as a loss function component and as an evaluation metric.</t>
   </si>
 </sst>
 </file>
@@ -1780,14 +1935,14 @@
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2146,39 +2301,39 @@
   <sheetData>
     <row r="1" spans="1:16" ht="15" customHeight="1">
       <c r="A1" s="1"/>
-      <c r="B1" s="11" t="s">
+      <c r="B1" s="12" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="11" t="s">
+      <c r="C1" s="12" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="11"/>
-      <c r="E1" s="11"/>
-      <c r="F1" s="11" t="s">
+      <c r="D1" s="12"/>
+      <c r="E1" s="12"/>
+      <c r="F1" s="12" t="s">
         <v>2</v>
       </c>
-      <c r="G1" s="11"/>
+      <c r="G1" s="12"/>
       <c r="H1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="I1" s="11" t="s">
+      <c r="I1" s="12" t="s">
         <v>4</v>
       </c>
-      <c r="J1" s="11"/>
-      <c r="K1" s="11" t="s">
+      <c r="J1" s="12"/>
+      <c r="K1" s="12" t="s">
         <v>5</v>
       </c>
-      <c r="L1" s="11"/>
-      <c r="M1" s="11" t="s">
+      <c r="L1" s="12"/>
+      <c r="M1" s="12" t="s">
         <v>6</v>
       </c>
-      <c r="N1" s="11" t="s">
+      <c r="N1" s="12" t="s">
         <v>7</v>
       </c>
-      <c r="O1" s="11" t="s">
+      <c r="O1" s="12" t="s">
         <v>8</v>
       </c>
-      <c r="P1" s="10" t="s">
+      <c r="P1" s="11" t="s">
         <v>390</v>
       </c>
     </row>
@@ -2186,7 +2341,7 @@
       <c r="A2" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="B2" s="11"/>
+      <c r="B2" s="12"/>
       <c r="C2" s="2" t="s">
         <v>10</v>
       </c>
@@ -2217,10 +2372,10 @@
       <c r="L2" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="M2" s="11"/>
-      <c r="N2" s="11"/>
-      <c r="O2" s="11"/>
-      <c r="P2" s="10"/>
+      <c r="M2" s="12"/>
+      <c r="N2" s="12"/>
+      <c r="O2" s="12"/>
+      <c r="P2" s="11"/>
     </row>
     <row r="3" spans="1:16" s="4" customFormat="1" ht="250.8">
       <c r="A3" s="3" t="s">
@@ -3768,7 +3923,7 @@
       <c r="D35" s="3" t="s">
         <v>410</v>
       </c>
-      <c r="E35" s="12" t="s">
+      <c r="E35" s="10" t="s">
         <v>318</v>
       </c>
       <c r="F35" s="3" t="s">
@@ -3950,7 +4105,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="39" spans="1:16" s="4" customFormat="1" ht="31.2" customHeight="1">
+    <row r="39" spans="1:16" s="4" customFormat="1" ht="132">
       <c r="A39" s="3" t="s">
         <v>55</v>
       </c>
@@ -4000,233 +4155,254 @@
         <v>452</v>
       </c>
     </row>
-    <row r="40" spans="1:16" s="4" customFormat="1">
+    <row r="40" spans="1:16" s="4" customFormat="1" ht="132">
       <c r="A40" s="3" t="s">
         <v>56</v>
       </c>
       <c r="B40" s="3" t="s">
-        <v>66</v>
+        <v>453</v>
       </c>
       <c r="C40" s="3" t="s">
-        <v>66</v>
+        <v>455</v>
       </c>
       <c r="D40" s="3" t="s">
-        <v>66</v>
+        <v>454</v>
       </c>
       <c r="E40" s="3" t="s">
-        <v>66</v>
+        <v>456</v>
       </c>
       <c r="F40" s="3" t="s">
-        <v>66</v>
+        <v>447</v>
       </c>
       <c r="G40" s="3" t="s">
-        <v>66</v>
+        <v>398</v>
       </c>
       <c r="H40" s="3" t="s">
-        <v>66</v>
+        <v>333</v>
       </c>
       <c r="I40" s="3" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="J40" s="3" t="s">
-        <v>66</v>
+        <v>457</v>
       </c>
       <c r="K40" s="3" t="s">
-        <v>66</v>
+        <v>402</v>
       </c>
       <c r="L40" s="3" t="s">
-        <v>66</v>
+        <v>449</v>
       </c>
       <c r="M40" s="3" t="s">
-        <v>66</v>
-      </c>
-      <c r="N40" s="3"/>
+        <v>439</v>
+      </c>
+      <c r="N40" s="3" t="s">
+        <v>427</v>
+      </c>
       <c r="O40" s="3" t="s">
-        <v>66</v>
+        <v>458</v>
+      </c>
+      <c r="P40" s="4" t="s">
+        <v>459</v>
       </c>
     </row>
-    <row r="41" spans="1:16" ht="23.4" customHeight="1">
-      <c r="A41" s="1" t="s">
+    <row r="41" spans="1:16" s="4" customFormat="1" ht="145.19999999999999">
+      <c r="A41" s="3" t="s">
         <v>57</v>
       </c>
-      <c r="B41" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="C41" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="D41" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="E41" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="F41" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="G41" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="H41" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="I41" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="J41" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="K41" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="L41" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="M41" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="N41" s="1"/>
-      <c r="O41" s="1" t="s">
-        <v>66</v>
+      <c r="B41" s="3" t="s">
+        <v>460</v>
+      </c>
+      <c r="C41" s="3" t="s">
+        <v>461</v>
+      </c>
+      <c r="D41" s="3" t="s">
+        <v>463</v>
+      </c>
+      <c r="E41" s="3" t="s">
+        <v>462</v>
+      </c>
+      <c r="F41" s="3" t="s">
+        <v>464</v>
+      </c>
+      <c r="G41" s="3" t="s">
+        <v>398</v>
+      </c>
+      <c r="H41" s="3" t="s">
+        <v>333</v>
+      </c>
+      <c r="I41" s="3" t="s">
+        <v>465</v>
+      </c>
+      <c r="J41" s="3" t="s">
+        <v>466</v>
+      </c>
+      <c r="K41" s="3" t="s">
+        <v>402</v>
+      </c>
+      <c r="L41" s="3" t="s">
+        <v>467</v>
+      </c>
+      <c r="M41" s="3" t="s">
+        <v>468</v>
+      </c>
+      <c r="N41" s="3" t="s">
+        <v>469</v>
+      </c>
+      <c r="O41" s="3" t="s">
+        <v>470</v>
+      </c>
+      <c r="P41" s="4" t="s">
+        <v>471</v>
       </c>
     </row>
-    <row r="42" spans="1:16">
-      <c r="A42" s="1" t="s">
+    <row r="42" spans="1:16" s="4" customFormat="1" ht="118.8">
+      <c r="A42" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="B42" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="C42" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="D42" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="E42" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="F42" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="G42" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="H42" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="I42" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="J42" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="K42" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="L42" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="M42" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="N42" s="1"/>
-      <c r="O42" s="1" t="s">
-        <v>66</v>
+      <c r="B42" s="3" t="s">
+        <v>472</v>
+      </c>
+      <c r="C42" s="3" t="s">
+        <v>473</v>
+      </c>
+      <c r="D42" s="3" t="s">
+        <v>474</v>
+      </c>
+      <c r="E42" s="3" t="s">
+        <v>456</v>
+      </c>
+      <c r="F42" s="3" t="s">
+        <v>447</v>
+      </c>
+      <c r="G42" s="3" t="s">
+        <v>398</v>
+      </c>
+      <c r="H42" s="3" t="s">
+        <v>448</v>
+      </c>
+      <c r="I42" s="3" t="s">
+        <v>475</v>
+      </c>
+      <c r="J42" s="3" t="s">
+        <v>373</v>
+      </c>
+      <c r="K42" s="3" t="s">
+        <v>402</v>
+      </c>
+      <c r="L42" s="3" t="s">
+        <v>449</v>
+      </c>
+      <c r="M42" s="3" t="s">
+        <v>476</v>
+      </c>
+      <c r="N42" s="3" t="s">
+        <v>477</v>
+      </c>
+      <c r="O42" s="3" t="s">
+        <v>478</v>
+      </c>
+      <c r="P42" s="4" t="s">
+        <v>479</v>
       </c>
     </row>
-    <row r="43" spans="1:16">
-      <c r="A43" s="1" t="s">
+    <row r="43" spans="1:16" s="4" customFormat="1" ht="145.19999999999999">
+      <c r="A43" s="3" t="s">
         <v>59</v>
       </c>
-      <c r="B43" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="C43" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="D43" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="E43" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="F43" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="G43" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="H43" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="I43" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="J43" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="K43" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="L43" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="M43" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="N43" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="O43" s="1" t="s">
-        <v>66</v>
+      <c r="B43" s="3" t="s">
+        <v>480</v>
+      </c>
+      <c r="C43" s="3" t="s">
+        <v>481</v>
+      </c>
+      <c r="D43" s="3" t="s">
+        <v>482</v>
+      </c>
+      <c r="E43" s="3" t="s">
+        <v>446</v>
+      </c>
+      <c r="F43" s="3" t="s">
+        <v>447</v>
+      </c>
+      <c r="G43" s="3" t="s">
+        <v>446</v>
+      </c>
+      <c r="H43" s="3" t="s">
+        <v>412</v>
+      </c>
+      <c r="I43" s="3" t="s">
+        <v>475</v>
+      </c>
+      <c r="J43" s="3" t="s">
+        <v>483</v>
+      </c>
+      <c r="K43" s="3" t="s">
+        <v>402</v>
+      </c>
+      <c r="L43" s="3" t="s">
+        <v>484</v>
+      </c>
+      <c r="M43" s="3" t="s">
+        <v>485</v>
+      </c>
+      <c r="N43" s="3" t="s">
+        <v>486</v>
+      </c>
+      <c r="O43" s="3" t="s">
+        <v>487</v>
+      </c>
+      <c r="P43" s="4" t="s">
+        <v>488</v>
       </c>
     </row>
-    <row r="44" spans="1:16">
-      <c r="A44" s="1" t="s">
+    <row r="44" spans="1:16" s="4" customFormat="1" ht="145.19999999999999">
+      <c r="A44" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="B44" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="C44" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="D44" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="E44" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="F44" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="G44" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="H44" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="I44" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="J44" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="K44" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="L44" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="M44" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="N44" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="O44" s="1" t="s">
-        <v>66</v>
+      <c r="B44" s="3" t="s">
+        <v>489</v>
+      </c>
+      <c r="C44" s="3" t="s">
+        <v>490</v>
+      </c>
+      <c r="D44" s="3" t="s">
+        <v>491</v>
+      </c>
+      <c r="E44" s="3" t="s">
+        <v>369</v>
+      </c>
+      <c r="F44" s="3" t="s">
+        <v>447</v>
+      </c>
+      <c r="G44" s="3" t="s">
+        <v>369</v>
+      </c>
+      <c r="H44" s="3" t="s">
+        <v>412</v>
+      </c>
+      <c r="I44" s="3" t="s">
+        <v>475</v>
+      </c>
+      <c r="J44" s="3" t="s">
+        <v>492</v>
+      </c>
+      <c r="K44" s="3" t="s">
+        <v>402</v>
+      </c>
+      <c r="L44" s="3" t="s">
+        <v>493</v>
+      </c>
+      <c r="M44" s="3" t="s">
+        <v>494</v>
+      </c>
+      <c r="N44" s="3" t="s">
+        <v>495</v>
+      </c>
+      <c r="O44" s="3" t="s">
+        <v>496</v>
+      </c>
+      <c r="P44" s="4" t="s">
+        <v>497</v>
       </c>
     </row>
     <row r="45" spans="1:16">
@@ -4339,6 +4515,12 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x01010009048CEEA230F14796749F6DFD5F5263" ma:contentTypeVersion="4" ma:contentTypeDescription="Crear nuevo documento." ma:contentTypeScope="" ma:versionID="5105af4e7c1b0ed6cdb04338eaf51f7a">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="96457c7a-bdfc-427e-9d05-5faa5ab5244b" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="0baee1a300280ca08e7397f1756276d6" ns2:_="">
     <xsd:import namespace="96457c7a-bdfc-427e-9d05-5faa5ab5244b"/>
@@ -4482,12 +4664,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
@@ -4498,6 +4674,15 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1160EB8C-E200-4916-A3B3-9BF8115D37F8}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{75ADFBF6-8C74-4292-833E-68A026E87063}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -4515,15 +4700,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1160EB8C-E200-4916-A3B3-9BF8115D37F8}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{24F2579D-323E-48EA-8FED-D372AFFF0A04}">
   <ds:schemaRefs>

</xml_diff>

<commit_message>
Add new paper names CSV and individual annotations Excel file
- Created a new CSV file containing a list of paper names with authors and publication years.
- Added an Excel file for individual annotations related to the papers.
</commit_message>
<xml_diff>
--- a/main/04_data_extraction/Individual AnnotationsORC.xlsx
+++ b/main/04_data_extraction/Individual AnnotationsORC.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\orincon\scoping-ml-wave-seismology\main\04_data_extraction\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{40D0FA0E-74F1-4D09-97B6-6A8B25CE1FF4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3AD872B6-6C07-4F95-AD83-FEB880C5AC7A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{115BB8D9-8B86-4726-97F8-E06477FD353D}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="697" uniqueCount="509">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="698" uniqueCount="509">
   <si>
     <t>Lectura general</t>
   </si>
@@ -1896,24 +1896,12 @@
       <family val="1"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFF0000"/>
-        <bgColor indexed="64"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="2">
@@ -1943,7 +1931,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1951,35 +1939,29 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2325,52 +2307,52 @@
   <dimension ref="A1:P46"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.09765625" defaultRowHeight="13.2"/>
   <cols>
-    <col min="1" max="1" width="36.59765625" style="5" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="39.296875" style="5" customWidth="1"/>
-    <col min="3" max="3" width="36.59765625" style="5" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="24.8984375" style="5" customWidth="1"/>
-    <col min="5" max="8" width="36.59765625" style="5" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="35.69921875" style="5" bestFit="1" customWidth="1"/>
-    <col min="10" max="15" width="36.59765625" style="5" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="32.296875" style="5" bestFit="1" customWidth="1"/>
-    <col min="17" max="16384" width="9.09765625" style="5"/>
+    <col min="1" max="1" width="36.59765625" style="3" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="39.296875" style="3" customWidth="1"/>
+    <col min="3" max="3" width="36.59765625" style="3" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="24.8984375" style="3" customWidth="1"/>
+    <col min="5" max="8" width="36.59765625" style="3" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="35.69921875" style="3" bestFit="1" customWidth="1"/>
+    <col min="10" max="15" width="36.59765625" style="3" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="32.296875" style="3" bestFit="1" customWidth="1"/>
+    <col min="17" max="16384" width="9.09765625" style="3"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:16" ht="15" customHeight="1">
       <c r="A1" s="1"/>
-      <c r="B1" s="12" t="s">
+      <c r="B1" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="12" t="s">
+      <c r="C1" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="12"/>
-      <c r="E1" s="12"/>
-      <c r="F1" s="12" t="s">
+      <c r="D1" s="5"/>
+      <c r="E1" s="5"/>
+      <c r="F1" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="G1" s="12"/>
+      <c r="G1" s="5"/>
       <c r="H1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="I1" s="12" t="s">
+      <c r="I1" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="J1" s="12"/>
-      <c r="K1" s="12" t="s">
+      <c r="J1" s="5"/>
+      <c r="K1" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="L1" s="12"/>
-      <c r="M1" s="12" t="s">
+      <c r="L1" s="5"/>
+      <c r="M1" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="N1" s="12" t="s">
+      <c r="N1" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="O1" s="12" t="s">
+      <c r="O1" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="P1" s="11" t="s">
+      <c r="P1" s="4" t="s">
         <v>390</v>
       </c>
     </row>
@@ -2378,7 +2360,7 @@
       <c r="A2" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="B2" s="12"/>
+      <c r="B2" s="5"/>
       <c r="C2" s="2" t="s">
         <v>10</v>
       </c>
@@ -2409,2134 +2391,2137 @@
       <c r="L2" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="M2" s="12"/>
-      <c r="N2" s="12"/>
-      <c r="O2" s="12"/>
-      <c r="P2" s="11"/>
+      <c r="M2" s="5"/>
+      <c r="N2" s="5"/>
+      <c r="O2" s="5"/>
+      <c r="P2" s="4"/>
     </row>
-    <row r="3" spans="1:16" s="4" customFormat="1" ht="250.8">
-      <c r="A3" s="3" t="s">
+    <row r="3" spans="1:16" s="7" customFormat="1" ht="250.8">
+      <c r="A3" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="B3" s="6" t="s">
         <v>71</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="C3" s="6" t="s">
         <v>72</v>
       </c>
-      <c r="D3" s="3" t="s">
+      <c r="D3" s="6" t="s">
         <v>73</v>
       </c>
-      <c r="E3" s="3" t="s">
+      <c r="E3" s="6" t="s">
         <v>63</v>
       </c>
-      <c r="F3" s="3" t="s">
+      <c r="F3" s="6" t="s">
         <v>74</v>
       </c>
-      <c r="G3" s="3" t="s">
+      <c r="G3" s="6" t="s">
         <v>75</v>
       </c>
-      <c r="H3" s="3" t="s">
+      <c r="H3" s="6" t="s">
         <v>64</v>
       </c>
-      <c r="I3" s="3" t="s">
+      <c r="I3" s="6" t="s">
         <v>68</v>
       </c>
-      <c r="J3" s="3" t="s">
+      <c r="J3" s="6" t="s">
         <v>76</v>
       </c>
-      <c r="K3" s="3" t="s">
+      <c r="K3" s="6" t="s">
         <v>77</v>
       </c>
-      <c r="L3" s="3" t="s">
+      <c r="L3" s="6" t="s">
         <v>78</v>
       </c>
-      <c r="M3" s="3" t="s">
+      <c r="M3" s="6" t="s">
         <v>79</v>
       </c>
-      <c r="N3" s="3" t="s">
+      <c r="N3" s="6" t="s">
         <v>66</v>
       </c>
-      <c r="O3" s="3" t="s">
+      <c r="O3" s="6" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="4" spans="1:16" s="4" customFormat="1" ht="171.6">
-      <c r="A4" s="3" t="s">
+    <row r="4" spans="1:16" s="7" customFormat="1" ht="171.6">
+      <c r="A4" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="B4" s="6" t="s">
         <v>81</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="C4" s="6" t="s">
         <v>82</v>
       </c>
-      <c r="D4" s="3" t="s">
+      <c r="D4" s="6" t="s">
         <v>83</v>
       </c>
-      <c r="E4" s="3" t="s">
+      <c r="E4" s="6" t="s">
         <v>84</v>
       </c>
-      <c r="F4" s="3" t="s">
+      <c r="F4" s="6" t="s">
         <v>85</v>
       </c>
-      <c r="G4" s="3" t="s">
+      <c r="G4" s="6" t="s">
         <v>78</v>
       </c>
-      <c r="H4" s="3" t="s">
+      <c r="H4" s="6" t="s">
         <v>86</v>
       </c>
-      <c r="I4" s="3" t="s">
+      <c r="I4" s="6" t="s">
         <v>68</v>
       </c>
-      <c r="J4" s="3" t="s">
+      <c r="J4" s="6" t="s">
         <v>87</v>
       </c>
-      <c r="K4" s="3" t="s">
+      <c r="K4" s="6" t="s">
         <v>88</v>
       </c>
-      <c r="L4" s="3" t="s">
+      <c r="L4" s="6" t="s">
         <v>89</v>
       </c>
-      <c r="M4" s="3"/>
-      <c r="N4" s="3"/>
-      <c r="O4" s="3" t="s">
+      <c r="M4" s="6"/>
+      <c r="N4" s="6"/>
+      <c r="O4" s="6" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="5" spans="1:16" s="4" customFormat="1" ht="201" customHeight="1">
-      <c r="A5" s="3" t="s">
+    <row r="5" spans="1:16" s="7" customFormat="1" ht="201" customHeight="1">
+      <c r="A5" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="B5" s="3" t="s">
+      <c r="B5" s="6" t="s">
         <v>91</v>
       </c>
-      <c r="C5" s="3" t="s">
+      <c r="C5" s="6" t="s">
         <v>65</v>
       </c>
-      <c r="D5" s="3" t="s">
+      <c r="D5" s="6" t="s">
         <v>92</v>
       </c>
-      <c r="E5" s="3" t="s">
+      <c r="E5" s="6" t="s">
         <v>93</v>
       </c>
-      <c r="F5" s="3" t="s">
+      <c r="F5" s="6" t="s">
         <v>85</v>
       </c>
-      <c r="G5" s="3" t="s">
+      <c r="G5" s="6" t="s">
         <v>78</v>
       </c>
-      <c r="H5" s="3" t="s">
+      <c r="H5" s="6" t="s">
         <v>94</v>
       </c>
-      <c r="I5" s="3" t="s">
+      <c r="I5" s="6" t="s">
         <v>68</v>
       </c>
-      <c r="J5" s="3" t="s">
+      <c r="J5" s="6" t="s">
         <v>78</v>
       </c>
-      <c r="K5" s="3" t="s">
+      <c r="K5" s="6" t="s">
         <v>70</v>
       </c>
-      <c r="L5" s="3" t="s">
+      <c r="L5" s="6" t="s">
         <v>78</v>
       </c>
-      <c r="M5" s="3" t="s">
+      <c r="M5" s="6" t="s">
         <v>95</v>
       </c>
-      <c r="N5" s="3" t="s">
+      <c r="N5" s="6" t="s">
         <v>96</v>
       </c>
-      <c r="O5" s="3" t="s">
+      <c r="O5" s="6" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="6" spans="1:16" s="4" customFormat="1" ht="210" customHeight="1">
-      <c r="A6" s="3" t="s">
+    <row r="6" spans="1:16" s="7" customFormat="1" ht="210" customHeight="1">
+      <c r="A6" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="B6" s="3" t="s">
+      <c r="B6" s="6" t="s">
         <v>98</v>
       </c>
-      <c r="C6" s="3" t="s">
+      <c r="C6" s="6" t="s">
         <v>99</v>
       </c>
-      <c r="D6" s="3" t="s">
+      <c r="D6" s="6" t="s">
         <v>100</v>
       </c>
-      <c r="E6" s="3" t="s">
+      <c r="E6" s="6" t="s">
         <v>78</v>
       </c>
-      <c r="F6" s="3" t="s">
+      <c r="F6" s="6" t="s">
         <v>85</v>
       </c>
-      <c r="G6" s="3" t="s">
+      <c r="G6" s="6" t="s">
         <v>78</v>
       </c>
-      <c r="H6" s="3" t="s">
+      <c r="H6" s="6" t="s">
         <v>101</v>
       </c>
-      <c r="I6" s="3" t="s">
+      <c r="I6" s="6" t="s">
         <v>68</v>
       </c>
-      <c r="J6" s="3" t="s">
+      <c r="J6" s="6" t="s">
         <v>78</v>
       </c>
-      <c r="K6" s="3" t="s">
+      <c r="K6" s="6" t="s">
         <v>88</v>
       </c>
-      <c r="L6" s="3" t="s">
+      <c r="L6" s="6" t="s">
         <v>78</v>
       </c>
-      <c r="M6" s="3" t="s">
+      <c r="M6" s="6" t="s">
         <v>102</v>
       </c>
-      <c r="N6" s="3" t="s">
+      <c r="N6" s="6" t="s">
         <v>66</v>
       </c>
-      <c r="O6" s="3" t="s">
+      <c r="O6" s="6" t="s">
         <v>103</v>
       </c>
     </row>
-    <row r="7" spans="1:16" s="4" customFormat="1" ht="250.8">
-      <c r="A7" s="3" t="s">
+    <row r="7" spans="1:16" s="7" customFormat="1" ht="250.8">
+      <c r="A7" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="B7" s="3" t="s">
+      <c r="B7" s="6" t="s">
         <v>104</v>
       </c>
-      <c r="C7" s="3" t="s">
+      <c r="C7" s="6" t="s">
         <v>105</v>
       </c>
-      <c r="D7" s="3" t="s">
+      <c r="D7" s="6" t="s">
         <v>106</v>
       </c>
-      <c r="E7" s="3" t="s">
+      <c r="E7" s="6" t="s">
         <v>107</v>
       </c>
-      <c r="F7" s="3" t="s">
+      <c r="F7" s="6" t="s">
         <v>108</v>
       </c>
-      <c r="G7" s="3" t="s">
+      <c r="G7" s="6" t="s">
         <v>109</v>
       </c>
-      <c r="H7" s="3" t="s">
+      <c r="H7" s="6" t="s">
         <v>110</v>
       </c>
-      <c r="I7" s="3" t="s">
+      <c r="I7" s="6" t="s">
         <v>67</v>
       </c>
-      <c r="J7" s="3" t="s">
+      <c r="J7" s="6" t="s">
         <v>111</v>
       </c>
-      <c r="K7" s="3" t="s">
+      <c r="K7" s="6" t="s">
         <v>70</v>
       </c>
-      <c r="L7" s="3" t="s">
+      <c r="L7" s="6" t="s">
         <v>78</v>
       </c>
-      <c r="M7" s="3" t="s">
+      <c r="M7" s="6" t="s">
         <v>112</v>
       </c>
-      <c r="N7" s="3" t="s">
+      <c r="N7" s="6" t="s">
         <v>66</v>
       </c>
-      <c r="O7" s="3" t="s">
+      <c r="O7" s="6" t="s">
         <v>113</v>
       </c>
     </row>
-    <row r="8" spans="1:16" s="4" customFormat="1" ht="250.8">
-      <c r="A8" s="3" t="s">
+    <row r="8" spans="1:16" s="7" customFormat="1" ht="250.8">
+      <c r="A8" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="B8" s="3" t="s">
+      <c r="B8" s="6" t="s">
         <v>114</v>
       </c>
-      <c r="C8" s="3" t="s">
+      <c r="C8" s="6" t="s">
         <v>115</v>
       </c>
-      <c r="D8" s="3" t="s">
+      <c r="D8" s="6" t="s">
         <v>116</v>
       </c>
-      <c r="E8" s="3" t="s">
+      <c r="E8" s="6" t="s">
         <v>117</v>
       </c>
-      <c r="F8" s="3" t="s">
+      <c r="F8" s="6" t="s">
         <v>85</v>
       </c>
-      <c r="G8" s="3" t="s">
+      <c r="G8" s="6" t="s">
         <v>78</v>
       </c>
-      <c r="H8" s="3" t="s">
+      <c r="H8" s="6" t="s">
         <v>66</v>
       </c>
-      <c r="I8" s="3" t="s">
+      <c r="I8" s="6" t="s">
         <v>67</v>
       </c>
-      <c r="J8" s="3" t="s">
+      <c r="J8" s="6" t="s">
         <v>118</v>
       </c>
-      <c r="K8" s="3" t="s">
+      <c r="K8" s="6" t="s">
         <v>119</v>
       </c>
-      <c r="L8" s="3" t="s">
+      <c r="L8" s="6" t="s">
         <v>120</v>
       </c>
-      <c r="M8" s="3" t="s">
+      <c r="M8" s="6" t="s">
         <v>121</v>
       </c>
-      <c r="N8" s="3" t="s">
+      <c r="N8" s="6" t="s">
         <v>66</v>
       </c>
-      <c r="O8" s="3" t="s">
+      <c r="O8" s="6" t="s">
         <v>122</v>
       </c>
     </row>
-    <row r="9" spans="1:16" s="4" customFormat="1" ht="184.8">
-      <c r="A9" s="3" t="s">
+    <row r="9" spans="1:16" s="7" customFormat="1" ht="184.8">
+      <c r="A9" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="B9" s="3" t="s">
+      <c r="B9" s="6" t="s">
         <v>123</v>
       </c>
-      <c r="C9" s="3" t="s">
+      <c r="C9" s="6" t="s">
         <v>124</v>
       </c>
-      <c r="D9" s="3" t="s">
+      <c r="D9" s="6" t="s">
         <v>125</v>
       </c>
-      <c r="E9" s="3" t="s">
+      <c r="E9" s="6" t="s">
         <v>126</v>
       </c>
-      <c r="F9" s="3" t="s">
+      <c r="F9" s="6" t="s">
         <v>85</v>
       </c>
-      <c r="G9" s="3" t="s">
+      <c r="G9" s="6" t="s">
         <v>127</v>
       </c>
-      <c r="H9" s="3" t="s">
+      <c r="H9" s="6" t="s">
         <v>128</v>
       </c>
-      <c r="I9" s="3" t="s">
+      <c r="I9" s="6" t="s">
         <v>329</v>
       </c>
-      <c r="J9" s="3" t="s">
+      <c r="J9" s="6" t="s">
         <v>129</v>
       </c>
-      <c r="K9" s="3" t="s">
+      <c r="K9" s="6" t="s">
         <v>77</v>
       </c>
-      <c r="L9" s="3" t="s">
+      <c r="L9" s="6" t="s">
         <v>78</v>
       </c>
-      <c r="M9" s="3" t="s">
+      <c r="M9" s="6" t="s">
         <v>130</v>
       </c>
-      <c r="N9" s="3" t="s">
+      <c r="N9" s="6" t="s">
         <v>66</v>
       </c>
-      <c r="O9" s="3" t="s">
+      <c r="O9" s="6" t="s">
         <v>131</v>
       </c>
     </row>
-    <row r="10" spans="1:16" s="4" customFormat="1" ht="290.39999999999998">
-      <c r="A10" s="3" t="s">
+    <row r="10" spans="1:16" s="7" customFormat="1" ht="290.39999999999998">
+      <c r="A10" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="B10" s="3" t="s">
+      <c r="B10" s="6" t="s">
         <v>132</v>
       </c>
-      <c r="C10" s="3" t="s">
+      <c r="C10" s="6" t="s">
         <v>133</v>
       </c>
-      <c r="D10" s="3" t="s">
+      <c r="D10" s="6" t="s">
         <v>134</v>
       </c>
-      <c r="E10" s="3" t="s">
+      <c r="E10" s="6" t="s">
         <v>135</v>
       </c>
-      <c r="F10" s="3" t="s">
+      <c r="F10" s="6" t="s">
         <v>85</v>
       </c>
-      <c r="G10" s="3" t="s">
+      <c r="G10" s="6" t="s">
         <v>78</v>
       </c>
-      <c r="H10" s="3" t="s">
+      <c r="H10" s="6" t="s">
         <v>136</v>
       </c>
-      <c r="I10" s="3" t="s">
+      <c r="I10" s="6" t="s">
         <v>329</v>
       </c>
-      <c r="J10" s="3" t="s">
+      <c r="J10" s="6" t="s">
         <v>78</v>
       </c>
-      <c r="K10" s="3" t="s">
+      <c r="K10" s="6" t="s">
         <v>137</v>
       </c>
-      <c r="L10" s="3" t="s">
+      <c r="L10" s="6" t="s">
         <v>138</v>
       </c>
-      <c r="M10" s="3" t="s">
+      <c r="M10" s="6" t="s">
         <v>139</v>
       </c>
-      <c r="N10" s="3" t="s">
+      <c r="N10" s="6" t="s">
         <v>66</v>
       </c>
-      <c r="O10" s="3" t="s">
+      <c r="O10" s="6" t="s">
         <v>140</v>
       </c>
     </row>
-    <row r="11" spans="1:16" s="4" customFormat="1" ht="211.2">
-      <c r="A11" s="3" t="s">
+    <row r="11" spans="1:16" s="7" customFormat="1" ht="211.2">
+      <c r="A11" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="B11" s="3" t="s">
+      <c r="B11" s="6" t="s">
         <v>141</v>
       </c>
-      <c r="C11" s="3" t="s">
+      <c r="C11" s="6" t="s">
         <v>142</v>
       </c>
-      <c r="D11" s="3" t="s">
+      <c r="D11" s="6" t="s">
         <v>143</v>
       </c>
-      <c r="E11" s="3" t="s">
+      <c r="E11" s="6" t="s">
         <v>78</v>
       </c>
-      <c r="F11" s="3" t="s">
+      <c r="F11" s="6" t="s">
         <v>85</v>
       </c>
-      <c r="G11" s="3" t="s">
+      <c r="G11" s="6" t="s">
         <v>78</v>
       </c>
-      <c r="H11" s="3" t="s">
+      <c r="H11" s="6" t="s">
         <v>144</v>
       </c>
-      <c r="I11" s="3" t="s">
+      <c r="I11" s="6" t="s">
         <v>68</v>
       </c>
-      <c r="J11" s="3" t="s">
+      <c r="J11" s="6" t="s">
         <v>78</v>
       </c>
-      <c r="K11" s="3" t="s">
+      <c r="K11" s="6" t="s">
         <v>69</v>
       </c>
-      <c r="L11" s="3" t="s">
+      <c r="L11" s="6" t="s">
         <v>78</v>
       </c>
-      <c r="M11" s="3" t="s">
+      <c r="M11" s="6" t="s">
         <v>145</v>
       </c>
-      <c r="N11" s="3" t="s">
+      <c r="N11" s="6" t="s">
         <v>66</v>
       </c>
-      <c r="O11" s="3" t="s">
+      <c r="O11" s="6" t="s">
         <v>146</v>
       </c>
     </row>
-    <row r="12" spans="1:16" s="4" customFormat="1" ht="198">
-      <c r="A12" s="3" t="s">
+    <row r="12" spans="1:16" s="7" customFormat="1" ht="198">
+      <c r="A12" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="B12" s="3" t="s">
+      <c r="B12" s="6" t="s">
         <v>147</v>
       </c>
-      <c r="C12" s="3" t="s">
+      <c r="C12" s="6" t="s">
         <v>148</v>
       </c>
-      <c r="D12" s="3" t="s">
+      <c r="D12" s="6" t="s">
         <v>149</v>
       </c>
-      <c r="E12" s="3" t="s">
+      <c r="E12" s="6" t="s">
         <v>78</v>
       </c>
-      <c r="F12" s="3" t="s">
+      <c r="F12" s="6" t="s">
         <v>150</v>
       </c>
-      <c r="G12" s="3" t="s">
+      <c r="G12" s="6" t="s">
         <v>151</v>
       </c>
-      <c r="H12" s="3" t="s">
+      <c r="H12" s="6" t="s">
         <v>152</v>
       </c>
-      <c r="I12" s="3" t="s">
+      <c r="I12" s="6" t="s">
         <v>67</v>
       </c>
-      <c r="J12" s="3" t="s">
+      <c r="J12" s="6" t="s">
         <v>78</v>
       </c>
-      <c r="K12" s="3" t="s">
+      <c r="K12" s="6" t="s">
         <v>70</v>
       </c>
-      <c r="L12" s="3" t="s">
+      <c r="L12" s="6" t="s">
         <v>78</v>
       </c>
-      <c r="M12" s="3" t="s">
+      <c r="M12" s="6" t="s">
         <v>153</v>
       </c>
-      <c r="N12" s="3" t="s">
+      <c r="N12" s="6" t="s">
         <v>66</v>
       </c>
-      <c r="O12" s="3" t="s">
+      <c r="O12" s="6" t="s">
         <v>154</v>
       </c>
     </row>
-    <row r="13" spans="1:16" s="4" customFormat="1" ht="264">
-      <c r="A13" s="3" t="s">
+    <row r="13" spans="1:16" s="7" customFormat="1" ht="264">
+      <c r="A13" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="B13" s="3" t="s">
+      <c r="B13" s="6" t="s">
         <v>155</v>
       </c>
-      <c r="C13" s="3" t="s">
+      <c r="C13" s="6" t="s">
         <v>156</v>
       </c>
-      <c r="D13" s="3" t="s">
+      <c r="D13" s="6" t="s">
         <v>157</v>
       </c>
-      <c r="E13" s="3" t="s">
+      <c r="E13" s="6" t="s">
         <v>78</v>
       </c>
-      <c r="F13" s="3" t="s">
+      <c r="F13" s="6" t="s">
         <v>85</v>
       </c>
-      <c r="G13" s="3" t="s">
+      <c r="G13" s="6" t="s">
         <v>158</v>
       </c>
-      <c r="H13" s="3" t="s">
+      <c r="H13" s="6" t="s">
         <v>144</v>
       </c>
-      <c r="I13" s="3" t="s">
+      <c r="I13" s="6" t="s">
         <v>68</v>
       </c>
-      <c r="J13" s="3" t="s">
+      <c r="J13" s="6" t="s">
         <v>159</v>
       </c>
-      <c r="K13" s="3" t="s">
+      <c r="K13" s="6" t="s">
         <v>69</v>
       </c>
-      <c r="L13" s="3" t="s">
+      <c r="L13" s="6" t="s">
         <v>78</v>
       </c>
-      <c r="M13" s="3" t="s">
+      <c r="M13" s="6" t="s">
         <v>160</v>
       </c>
-      <c r="N13" s="3" t="s">
+      <c r="N13" s="6" t="s">
         <v>161</v>
       </c>
-      <c r="O13" s="3" t="s">
+      <c r="O13" s="6" t="s">
         <v>162</v>
       </c>
     </row>
-    <row r="14" spans="1:16" s="4" customFormat="1" ht="290.39999999999998">
-      <c r="A14" s="3" t="s">
+    <row r="14" spans="1:16" s="7" customFormat="1" ht="290.39999999999998">
+      <c r="A14" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="B14" s="3" t="s">
+      <c r="B14" s="6" t="s">
         <v>163</v>
       </c>
-      <c r="C14" s="3" t="s">
+      <c r="C14" s="6" t="s">
         <v>164</v>
       </c>
-      <c r="D14" s="3" t="s">
+      <c r="D14" s="6" t="s">
         <v>165</v>
       </c>
-      <c r="E14" s="3" t="s">
+      <c r="E14" s="6" t="s">
         <v>78</v>
       </c>
-      <c r="F14" s="3" t="s">
+      <c r="F14" s="6" t="s">
         <v>166</v>
       </c>
-      <c r="G14" s="3" t="s">
+      <c r="G14" s="6" t="s">
         <v>78</v>
       </c>
-      <c r="H14" s="3" t="s">
+      <c r="H14" s="6" t="s">
         <v>167</v>
       </c>
-      <c r="I14" s="3" t="s">
+      <c r="I14" s="6" t="s">
         <v>329</v>
       </c>
-      <c r="J14" s="3" t="s">
+      <c r="J14" s="6" t="s">
         <v>168</v>
       </c>
-      <c r="K14" s="3" t="s">
+      <c r="K14" s="6" t="s">
         <v>69</v>
       </c>
-      <c r="L14" s="3" t="s">
+      <c r="L14" s="6" t="s">
         <v>78</v>
       </c>
-      <c r="M14" s="3" t="s">
+      <c r="M14" s="6" t="s">
         <v>66</v>
       </c>
-      <c r="N14" s="3" t="s">
+      <c r="N14" s="6" t="s">
         <v>66</v>
       </c>
-      <c r="O14" s="3" t="s">
+      <c r="O14" s="6" t="s">
         <v>169</v>
       </c>
     </row>
-    <row r="15" spans="1:16" s="4" customFormat="1" ht="198">
-      <c r="A15" s="3" t="s">
+    <row r="15" spans="1:16" s="7" customFormat="1" ht="198">
+      <c r="A15" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="B15" s="3" t="s">
+      <c r="B15" s="6" t="s">
         <v>170</v>
       </c>
-      <c r="C15" s="3" t="s">
+      <c r="C15" s="6" t="s">
         <v>171</v>
       </c>
-      <c r="D15" s="3" t="s">
+      <c r="D15" s="6" t="s">
         <v>172</v>
       </c>
-      <c r="E15" s="3" t="s">
+      <c r="E15" s="6" t="s">
         <v>135</v>
       </c>
-      <c r="F15" s="3" t="s">
+      <c r="F15" s="6" t="s">
         <v>66</v>
       </c>
-      <c r="G15" s="3" t="s">
+      <c r="G15" s="6" t="s">
         <v>66</v>
       </c>
-      <c r="H15" s="3" t="s">
+      <c r="H15" s="6" t="s">
         <v>66</v>
       </c>
-      <c r="I15" s="3">
+      <c r="I15" s="6">
         <v>2</v>
       </c>
-      <c r="J15" s="3" t="s">
+      <c r="J15" s="6" t="s">
         <v>66</v>
       </c>
-      <c r="K15" s="3" t="s">
+      <c r="K15" s="6" t="s">
         <v>69</v>
       </c>
-      <c r="L15" s="3" t="s">
+      <c r="L15" s="6" t="s">
         <v>173</v>
       </c>
-      <c r="M15" s="3" t="s">
+      <c r="M15" s="6" t="s">
         <v>66</v>
       </c>
-      <c r="N15" s="3" t="s">
+      <c r="N15" s="6" t="s">
         <v>66</v>
       </c>
-      <c r="O15" s="3" t="s">
+      <c r="O15" s="6" t="s">
         <v>174</v>
       </c>
     </row>
-    <row r="16" spans="1:16" s="4" customFormat="1" ht="290.39999999999998">
-      <c r="A16" s="3" t="s">
+    <row r="16" spans="1:16" s="7" customFormat="1" ht="290.39999999999998">
+      <c r="A16" s="6" t="s">
         <v>33</v>
       </c>
-      <c r="B16" s="3" t="s">
+      <c r="B16" s="6" t="s">
         <v>175</v>
       </c>
-      <c r="C16" s="3" t="s">
+      <c r="C16" s="6" t="s">
         <v>330</v>
       </c>
-      <c r="D16" s="3" t="s">
+      <c r="D16" s="6" t="s">
         <v>176</v>
       </c>
-      <c r="E16" s="3" t="s">
+      <c r="E16" s="6" t="s">
         <v>135</v>
       </c>
-      <c r="F16" s="3" t="s">
+      <c r="F16" s="6" t="s">
         <v>331</v>
       </c>
-      <c r="G16" s="3" t="s">
+      <c r="G16" s="6" t="s">
         <v>332</v>
       </c>
-      <c r="H16" s="3" t="s">
+      <c r="H16" s="6" t="s">
         <v>333</v>
       </c>
-      <c r="I16" s="3" t="s">
+      <c r="I16" s="6" t="s">
         <v>68</v>
       </c>
-      <c r="J16" s="3" t="s">
+      <c r="J16" s="6" t="s">
         <v>334</v>
       </c>
-      <c r="K16" s="3" t="s">
+      <c r="K16" s="6" t="s">
         <v>69</v>
       </c>
-      <c r="L16" s="3" t="s">
+      <c r="L16" s="6" t="s">
         <v>335</v>
       </c>
-      <c r="M16" s="3" t="s">
+      <c r="M16" s="6" t="s">
         <v>336</v>
       </c>
-      <c r="N16" s="3" t="s">
+      <c r="N16" s="6" t="s">
         <v>177</v>
       </c>
-      <c r="O16" s="3" t="s">
+      <c r="O16" s="6" t="s">
         <v>178</v>
       </c>
     </row>
-    <row r="17" spans="1:16" s="4" customFormat="1" ht="132">
-      <c r="A17" s="3" t="s">
+    <row r="17" spans="1:16" s="7" customFormat="1" ht="132">
+      <c r="A17" s="6" t="s">
         <v>34</v>
       </c>
-      <c r="B17" s="3" t="s">
+      <c r="B17" s="6" t="s">
         <v>301</v>
       </c>
-      <c r="C17" s="3" t="s">
+      <c r="C17" s="6" t="s">
         <v>289</v>
       </c>
-      <c r="D17" s="3" t="s">
+      <c r="D17" s="6" t="s">
         <v>290</v>
       </c>
-      <c r="E17" s="3" t="s">
+      <c r="E17" s="6" t="s">
         <v>291</v>
       </c>
-      <c r="F17" s="3" t="s">
+      <c r="F17" s="6" t="s">
         <v>292</v>
       </c>
-      <c r="G17" s="3" t="s">
+      <c r="G17" s="6" t="s">
         <v>293</v>
       </c>
-      <c r="H17" s="3" t="s">
+      <c r="H17" s="6" t="s">
         <v>294</v>
       </c>
-      <c r="I17" s="3" t="s">
+      <c r="I17" s="6" t="s">
         <v>295</v>
       </c>
-      <c r="J17" s="3" t="s">
+      <c r="J17" s="6" t="s">
         <v>296</v>
       </c>
-      <c r="K17" s="3" t="s">
+      <c r="K17" s="6" t="s">
         <v>69</v>
       </c>
-      <c r="L17" s="3" t="s">
+      <c r="L17" s="6" t="s">
         <v>297</v>
       </c>
-      <c r="M17" s="3" t="s">
+      <c r="M17" s="6" t="s">
         <v>298</v>
       </c>
-      <c r="N17" s="3" t="s">
+      <c r="N17" s="6" t="s">
         <v>300</v>
       </c>
-      <c r="O17" s="3" t="s">
+      <c r="O17" s="6" t="s">
         <v>391</v>
       </c>
-      <c r="P17" s="3" t="s">
+      <c r="P17" s="6" t="s">
         <v>299</v>
       </c>
     </row>
-    <row r="18" spans="1:16" s="4" customFormat="1" ht="379.5" customHeight="1">
-      <c r="A18" s="3" t="s">
+    <row r="18" spans="1:16" s="7" customFormat="1" ht="379.5" customHeight="1">
+      <c r="A18" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="B18" s="3" t="s">
+      <c r="B18" s="6" t="s">
         <v>179</v>
       </c>
-      <c r="C18" s="3" t="s">
+      <c r="C18" s="6" t="s">
         <v>180</v>
       </c>
-      <c r="D18" s="3" t="s">
+      <c r="D18" s="6" t="s">
         <v>181</v>
       </c>
-      <c r="E18" s="3" t="s">
+      <c r="E18" s="6" t="s">
         <v>182</v>
       </c>
-      <c r="F18" s="3" t="s">
+      <c r="F18" s="6" t="s">
         <v>183</v>
       </c>
-      <c r="G18" s="3" t="s">
+      <c r="G18" s="6" t="s">
         <v>78</v>
       </c>
-      <c r="H18" s="3" t="s">
+      <c r="H18" s="6" t="s">
         <v>184</v>
       </c>
-      <c r="I18" s="3" t="s">
+      <c r="I18" s="6" t="s">
         <v>185</v>
       </c>
-      <c r="J18" s="3" t="s">
+      <c r="J18" s="6" t="s">
         <v>186</v>
       </c>
-      <c r="K18" s="3" t="s">
+      <c r="K18" s="6" t="s">
         <v>187</v>
       </c>
-      <c r="L18" s="3" t="s">
+      <c r="L18" s="6" t="s">
         <v>188</v>
       </c>
-      <c r="M18" s="3" t="s">
+      <c r="M18" s="6" t="s">
         <v>189</v>
       </c>
-      <c r="N18" s="3" t="s">
+      <c r="N18" s="6" t="s">
         <v>190</v>
       </c>
-      <c r="O18" s="3" t="s">
+      <c r="O18" s="6" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="19" spans="1:16" s="4" customFormat="1" ht="61.5" customHeight="1">
-      <c r="A19" s="3" t="s">
+    <row r="19" spans="1:16" s="7" customFormat="1" ht="61.5" customHeight="1">
+      <c r="A19" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="B19" s="3" t="s">
+      <c r="B19" s="6" t="s">
         <v>191</v>
       </c>
-      <c r="C19" s="3" t="s">
+      <c r="C19" s="6" t="s">
         <v>192</v>
       </c>
-      <c r="D19" s="3" t="s">
+      <c r="D19" s="6" t="s">
         <v>193</v>
       </c>
-      <c r="E19" s="3" t="s">
+      <c r="E19" s="6" t="s">
         <v>194</v>
       </c>
-      <c r="F19" s="3" t="s">
+      <c r="F19" s="6" t="s">
         <v>195</v>
       </c>
-      <c r="G19" s="3" t="s">
+      <c r="G19" s="6" t="s">
         <v>194</v>
       </c>
-      <c r="H19" s="3" t="s">
+      <c r="H19" s="6" t="s">
         <v>196</v>
       </c>
-      <c r="I19" s="3" t="s">
+      <c r="I19" s="6" t="s">
         <v>197</v>
       </c>
-      <c r="J19" s="3" t="s">
+      <c r="J19" s="6" t="s">
         <v>198</v>
       </c>
-      <c r="K19" s="3" t="s">
+      <c r="K19" s="6" t="s">
         <v>199</v>
       </c>
-      <c r="L19" s="3" t="s">
+      <c r="L19" s="6" t="s">
         <v>200</v>
       </c>
-      <c r="M19" s="3" t="s">
+      <c r="M19" s="6" t="s">
         <v>201</v>
       </c>
-      <c r="N19" s="3" t="s">
+      <c r="N19" s="6" t="s">
         <v>202</v>
       </c>
-      <c r="O19" s="3" t="s">
+      <c r="O19" s="6" t="s">
         <v>194</v>
       </c>
-      <c r="P19" s="4" t="s">
+      <c r="P19" s="7" t="s">
         <v>203</v>
       </c>
     </row>
-    <row r="20" spans="1:16" s="4" customFormat="1" ht="409.6">
-      <c r="A20" s="3" t="s">
+    <row r="20" spans="1:16" s="7" customFormat="1" ht="409.6">
+      <c r="A20" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="B20" s="3" t="s">
+      <c r="B20" s="6" t="s">
         <v>204</v>
       </c>
-      <c r="C20" s="3" t="s">
+      <c r="C20" s="6" t="s">
         <v>205</v>
       </c>
-      <c r="D20" s="3" t="s">
+      <c r="D20" s="6" t="s">
         <v>206</v>
       </c>
-      <c r="E20" s="3" t="s">
+      <c r="E20" s="6" t="s">
         <v>78</v>
       </c>
-      <c r="F20" s="3" t="s">
+      <c r="F20" s="6" t="s">
         <v>85</v>
       </c>
-      <c r="G20" s="3" t="s">
+      <c r="G20" s="6" t="s">
         <v>78</v>
       </c>
-      <c r="H20" s="3" t="s">
+      <c r="H20" s="6" t="s">
         <v>78</v>
       </c>
-      <c r="I20" s="3" t="s">
+      <c r="I20" s="6" t="s">
         <v>68</v>
       </c>
-      <c r="J20" s="3" t="s">
+      <c r="J20" s="6" t="s">
         <v>207</v>
       </c>
-      <c r="K20" s="3" t="s">
+      <c r="K20" s="6" t="s">
         <v>77</v>
       </c>
-      <c r="L20" s="3" t="s">
+      <c r="L20" s="6" t="s">
         <v>78</v>
       </c>
-      <c r="M20" s="3" t="s">
+      <c r="M20" s="6" t="s">
         <v>95</v>
       </c>
-      <c r="N20" s="3" t="s">
+      <c r="N20" s="6" t="s">
         <v>66</v>
       </c>
-      <c r="O20" s="3" t="s">
+      <c r="O20" s="6" t="s">
         <v>208</v>
       </c>
     </row>
-    <row r="21" spans="1:16" s="4" customFormat="1" ht="132">
-      <c r="A21" s="3" t="s">
+    <row r="21" spans="1:16" s="7" customFormat="1" ht="132">
+      <c r="A21" s="6" t="s">
         <v>38</v>
       </c>
-      <c r="B21" s="3" t="s">
+      <c r="B21" s="6" t="s">
         <v>302</v>
       </c>
-      <c r="C21" s="3" t="s">
+      <c r="C21" s="6" t="s">
         <v>303</v>
       </c>
-      <c r="D21" s="3" t="s">
+      <c r="D21" s="6" t="s">
         <v>304</v>
       </c>
-      <c r="E21" s="3" t="s">
+      <c r="E21" s="6" t="s">
         <v>305</v>
       </c>
-      <c r="F21" s="3" t="s">
+      <c r="F21" s="6" t="s">
         <v>306</v>
       </c>
-      <c r="G21" s="3" t="s">
+      <c r="G21" s="6" t="s">
         <v>267</v>
       </c>
-      <c r="H21" s="3" t="s">
+      <c r="H21" s="6" t="s">
         <v>307</v>
       </c>
-      <c r="I21" s="3" t="s">
+      <c r="I21" s="6" t="s">
         <v>308</v>
       </c>
-      <c r="J21" s="3" t="s">
+      <c r="J21" s="6" t="s">
         <v>309</v>
       </c>
-      <c r="K21" s="3" t="s">
+      <c r="K21" s="6" t="s">
         <v>311</v>
       </c>
-      <c r="L21" s="3" t="s">
+      <c r="L21" s="6" t="s">
         <v>310</v>
       </c>
-      <c r="M21" s="3" t="s">
+      <c r="M21" s="6" t="s">
         <v>312</v>
       </c>
-      <c r="N21" s="3" t="s">
+      <c r="N21" s="6" t="s">
         <v>315</v>
       </c>
-      <c r="O21" s="3" t="s">
+      <c r="O21" s="6" t="s">
         <v>313</v>
       </c>
-      <c r="P21" s="4" t="s">
+      <c r="P21" s="7" t="s">
         <v>314</v>
       </c>
     </row>
-    <row r="22" spans="1:16" s="4" customFormat="1" ht="189" customHeight="1">
-      <c r="A22" s="3" t="s">
+    <row r="22" spans="1:16" s="7" customFormat="1" ht="189" customHeight="1">
+      <c r="A22" s="6" t="s">
         <v>39</v>
       </c>
-      <c r="B22" s="3" t="s">
+      <c r="B22" s="6" t="s">
         <v>316</v>
       </c>
-      <c r="C22" s="3" t="s">
+      <c r="C22" s="6" t="s">
         <v>317</v>
       </c>
-      <c r="D22" s="3" t="s">
+      <c r="D22" s="6" t="s">
         <v>319</v>
       </c>
-      <c r="E22" s="3" t="s">
+      <c r="E22" s="6" t="s">
         <v>318</v>
       </c>
-      <c r="F22" s="3" t="s">
+      <c r="F22" s="6" t="s">
         <v>321</v>
       </c>
-      <c r="G22" s="3" t="s">
+      <c r="G22" s="6" t="s">
         <v>320</v>
       </c>
-      <c r="H22" s="3" t="s">
+      <c r="H22" s="6" t="s">
         <v>322</v>
       </c>
-      <c r="I22" s="3" t="s">
+      <c r="I22" s="6" t="s">
         <v>68</v>
       </c>
-      <c r="J22" s="3" t="s">
+      <c r="J22" s="6" t="s">
         <v>269</v>
       </c>
-      <c r="K22" s="3" t="s">
+      <c r="K22" s="6" t="s">
         <v>323</v>
       </c>
-      <c r="L22" s="3" t="s">
+      <c r="L22" s="6" t="s">
         <v>324</v>
       </c>
-      <c r="M22" s="3" t="s">
+      <c r="M22" s="6" t="s">
         <v>325</v>
       </c>
-      <c r="N22" s="3" t="s">
+      <c r="N22" s="6" t="s">
         <v>326</v>
       </c>
-      <c r="O22" s="3" t="s">
+      <c r="O22" s="6" t="s">
         <v>327</v>
       </c>
-      <c r="P22" s="4" t="s">
+      <c r="P22" s="7" t="s">
         <v>328</v>
       </c>
     </row>
-    <row r="23" spans="1:16" s="4" customFormat="1" ht="250.8">
-      <c r="A23" s="3" t="s">
+    <row r="23" spans="1:16" s="7" customFormat="1" ht="250.8">
+      <c r="A23" s="6" t="s">
         <v>40</v>
       </c>
-      <c r="B23" s="3" t="s">
+      <c r="B23" s="6" t="s">
         <v>209</v>
       </c>
-      <c r="C23" s="3" t="s">
+      <c r="C23" s="6" t="s">
         <v>210</v>
       </c>
-      <c r="D23" s="3" t="s">
+      <c r="D23" s="6" t="s">
         <v>211</v>
       </c>
-      <c r="E23" s="3" t="s">
+      <c r="E23" s="6" t="s">
         <v>135</v>
       </c>
-      <c r="F23" s="3" t="s">
+      <c r="F23" s="6" t="s">
         <v>212</v>
       </c>
-      <c r="G23" s="3" t="s">
+      <c r="G23" s="6" t="s">
         <v>212</v>
       </c>
-      <c r="H23" s="3" t="s">
+      <c r="H23" s="6" t="s">
         <v>213</v>
       </c>
-      <c r="I23" s="3" t="s">
+      <c r="I23" s="6" t="s">
         <v>67</v>
       </c>
-      <c r="J23" s="3" t="s">
+      <c r="J23" s="6" t="s">
         <v>214</v>
       </c>
-      <c r="K23" s="3" t="s">
+      <c r="K23" s="6" t="s">
         <v>77</v>
       </c>
-      <c r="L23" s="3" t="s">
+      <c r="L23" s="6" t="s">
         <v>66</v>
       </c>
-      <c r="M23" s="3" t="s">
+      <c r="M23" s="6" t="s">
         <v>215</v>
       </c>
-      <c r="N23" s="3"/>
-      <c r="O23" s="3" t="s">
+      <c r="N23" s="6"/>
+      <c r="O23" s="6" t="s">
         <v>216</v>
       </c>
-      <c r="P23" s="3" t="s">
+      <c r="P23" s="6" t="s">
         <v>217</v>
       </c>
     </row>
-    <row r="24" spans="1:16" s="4" customFormat="1" ht="145.19999999999999">
-      <c r="A24" s="3" t="s">
+    <row r="24" spans="1:16" s="7" customFormat="1" ht="145.19999999999999">
+      <c r="A24" s="6" t="s">
         <v>337</v>
       </c>
-      <c r="B24" s="3" t="s">
+      <c r="B24" s="6" t="s">
         <v>338</v>
       </c>
-      <c r="C24" s="3" t="s">
+      <c r="C24" s="6" t="s">
         <v>339</v>
       </c>
-      <c r="D24" s="3" t="s">
+      <c r="D24" s="6" t="s">
         <v>340</v>
       </c>
-      <c r="E24" s="3" t="s">
+      <c r="E24" s="6" t="s">
         <v>341</v>
       </c>
-      <c r="F24" s="3" t="s">
+      <c r="F24" s="6" t="s">
         <v>343</v>
       </c>
-      <c r="G24" s="3" t="s">
+      <c r="G24" s="6" t="s">
         <v>342</v>
       </c>
-      <c r="H24" s="3" t="s">
+      <c r="H24" s="6" t="s">
         <v>344</v>
       </c>
-      <c r="I24" s="3" t="s">
+      <c r="I24" s="6" t="s">
         <v>345</v>
       </c>
-      <c r="J24" s="3" t="s">
+      <c r="J24" s="6" t="s">
         <v>346</v>
       </c>
-      <c r="K24" s="3" t="s">
+      <c r="K24" s="6" t="s">
         <v>347</v>
       </c>
-      <c r="L24" s="3" t="s">
+      <c r="L24" s="6" t="s">
         <v>348</v>
       </c>
-      <c r="M24" s="3" t="s">
+      <c r="M24" s="6" t="s">
         <v>352</v>
       </c>
-      <c r="N24" s="3" t="s">
+      <c r="N24" s="6" t="s">
         <v>351</v>
       </c>
-      <c r="O24" s="3" t="s">
+      <c r="O24" s="6" t="s">
         <v>349</v>
       </c>
-      <c r="P24" s="4" t="s">
+      <c r="P24" s="7" t="s">
         <v>350</v>
       </c>
     </row>
-    <row r="25" spans="1:16" s="4" customFormat="1" ht="118.8">
-      <c r="A25" s="3" t="s">
+    <row r="25" spans="1:16" s="7" customFormat="1" ht="118.8">
+      <c r="A25" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="B25" s="3" t="s">
+      <c r="B25" s="6" t="s">
         <v>353</v>
       </c>
-      <c r="C25" s="3" t="s">
+      <c r="C25" s="6" t="s">
         <v>363</v>
       </c>
-      <c r="D25" s="3" t="s">
+      <c r="D25" s="6" t="s">
         <v>354</v>
       </c>
-      <c r="E25" s="4" t="s">
+      <c r="E25" s="7" t="s">
         <v>318</v>
       </c>
-      <c r="F25" s="3" t="s">
+      <c r="F25" s="6" t="s">
         <v>331</v>
       </c>
-      <c r="G25" s="3" t="s">
+      <c r="G25" s="6" t="s">
         <v>355</v>
       </c>
-      <c r="H25" s="3" t="s">
+      <c r="H25" s="6" t="s">
         <v>356</v>
       </c>
-      <c r="I25" s="3" t="s">
+      <c r="I25" s="6" t="s">
         <v>257</v>
       </c>
-      <c r="J25" s="3" t="s">
+      <c r="J25" s="6" t="s">
         <v>269</v>
       </c>
-      <c r="K25" s="3" t="s">
+      <c r="K25" s="6" t="s">
         <v>357</v>
       </c>
-      <c r="L25" s="3" t="s">
+      <c r="L25" s="6" t="s">
         <v>358</v>
       </c>
-      <c r="M25" s="3" t="s">
+      <c r="M25" s="6" t="s">
         <v>359</v>
       </c>
-      <c r="N25" s="3" t="s">
+      <c r="N25" s="6" t="s">
         <v>360</v>
       </c>
-      <c r="O25" s="3" t="s">
+      <c r="O25" s="6" t="s">
         <v>361</v>
       </c>
-      <c r="P25" s="4" t="s">
+      <c r="P25" s="7" t="s">
         <v>362</v>
       </c>
     </row>
-    <row r="26" spans="1:16" s="4" customFormat="1" ht="184.8">
-      <c r="A26" s="3" t="s">
+    <row r="26" spans="1:16" s="7" customFormat="1" ht="184.8">
+      <c r="A26" s="6" t="s">
         <v>42</v>
       </c>
-      <c r="B26" s="3" t="s">
+      <c r="B26" s="6" t="s">
         <v>394</v>
       </c>
-      <c r="C26" s="3" t="s">
+      <c r="C26" s="6" t="s">
         <v>218</v>
       </c>
-      <c r="D26" s="3" t="s">
+      <c r="D26" s="6" t="s">
         <v>219</v>
       </c>
-      <c r="E26" s="3" t="s">
+      <c r="E26" s="6" t="s">
         <v>220</v>
       </c>
-      <c r="F26" s="3" t="s">
+      <c r="F26" s="6" t="s">
         <v>384</v>
       </c>
-      <c r="G26" s="3" t="s">
+      <c r="G26" s="6" t="s">
         <v>212</v>
       </c>
-      <c r="H26" s="3" t="s">
+      <c r="H26" s="6" t="s">
         <v>221</v>
       </c>
-      <c r="I26" s="3" t="s">
+      <c r="I26" s="6" t="s">
         <v>68</v>
       </c>
-      <c r="J26" s="3" t="s">
+      <c r="J26" s="6" t="s">
         <v>78</v>
       </c>
-      <c r="K26" s="3" t="s">
+      <c r="K26" s="6" t="s">
         <v>77</v>
       </c>
-      <c r="L26" s="3" t="s">
+      <c r="L26" s="6" t="s">
         <v>78</v>
       </c>
-      <c r="M26" s="3" t="s">
+      <c r="M26" s="6" t="s">
         <v>66</v>
       </c>
-      <c r="N26" s="3"/>
-      <c r="O26" s="3" t="s">
+      <c r="N26" s="6"/>
+      <c r="O26" s="6" t="s">
         <v>222</v>
       </c>
     </row>
-    <row r="27" spans="1:16" s="4" customFormat="1" ht="132">
-      <c r="A27" s="3" t="s">
+    <row r="27" spans="1:16" s="7" customFormat="1" ht="132">
+      <c r="A27" s="6" t="s">
         <v>43</v>
       </c>
-      <c r="B27" s="3" t="s">
+      <c r="B27" s="6" t="s">
         <v>380</v>
       </c>
-      <c r="C27" s="3" t="s">
+      <c r="C27" s="6" t="s">
         <v>381</v>
       </c>
-      <c r="D27" s="3" t="s">
+      <c r="D27" s="6" t="s">
         <v>382</v>
       </c>
-      <c r="E27" s="3" t="s">
+      <c r="E27" s="6" t="s">
         <v>383</v>
       </c>
-      <c r="F27" s="3" t="s">
+      <c r="F27" s="6" t="s">
         <v>384</v>
       </c>
-      <c r="G27" s="3" t="s">
+      <c r="G27" s="6" t="s">
         <v>212</v>
       </c>
-      <c r="H27" s="3" t="s">
+      <c r="H27" s="6" t="s">
         <v>385</v>
       </c>
-      <c r="I27" s="3" t="s">
+      <c r="I27" s="6" t="s">
         <v>257</v>
       </c>
-      <c r="J27" s="3" t="s">
+      <c r="J27" s="6" t="s">
         <v>78</v>
       </c>
-      <c r="K27" s="3" t="s">
+      <c r="K27" s="6" t="s">
         <v>386</v>
       </c>
-      <c r="L27" s="3" t="s">
+      <c r="L27" s="6" t="s">
         <v>387</v>
       </c>
-      <c r="M27" s="3" t="s">
+      <c r="M27" s="6" t="s">
         <v>388</v>
       </c>
-      <c r="N27" s="3" t="s">
+      <c r="N27" s="6" t="s">
         <v>393</v>
       </c>
-      <c r="O27" s="3" t="s">
+      <c r="O27" s="6" t="s">
         <v>389</v>
       </c>
-      <c r="P27" s="4" t="s">
+      <c r="P27" s="7" t="s">
         <v>392</v>
       </c>
     </row>
-    <row r="28" spans="1:16" s="4" customFormat="1" ht="224.4">
-      <c r="A28" s="3" t="s">
+    <row r="28" spans="1:16" s="7" customFormat="1" ht="224.4">
+      <c r="A28" s="6" t="s">
         <v>44</v>
       </c>
-      <c r="B28" s="3" t="s">
+      <c r="B28" s="6" t="s">
         <v>223</v>
       </c>
-      <c r="C28" s="3" t="s">
+      <c r="C28" s="6" t="s">
         <v>224</v>
       </c>
-      <c r="D28" s="3" t="s">
+      <c r="D28" s="6" t="s">
         <v>225</v>
       </c>
-      <c r="E28" s="3" t="s">
+      <c r="E28" s="6" t="s">
         <v>226</v>
       </c>
-      <c r="F28" s="3" t="s">
+      <c r="F28" s="6" t="s">
         <v>227</v>
       </c>
-      <c r="G28" s="3" t="s">
+      <c r="G28" s="6" t="s">
         <v>228</v>
       </c>
-      <c r="H28" s="3" t="s">
+      <c r="H28" s="6" t="s">
         <v>229</v>
       </c>
-      <c r="I28" s="3" t="s">
+      <c r="I28" s="6" t="s">
         <v>230</v>
       </c>
-      <c r="J28" s="3" t="s">
+      <c r="J28" s="6" t="s">
         <v>231</v>
       </c>
-      <c r="K28" s="3" t="s">
+      <c r="K28" s="6" t="s">
         <v>232</v>
       </c>
-      <c r="L28" s="3" t="s">
+      <c r="L28" s="6" t="s">
         <v>233</v>
       </c>
-      <c r="M28" s="3" t="s">
+      <c r="M28" s="6" t="s">
         <v>234</v>
       </c>
-      <c r="N28" s="3" t="s">
+      <c r="N28" s="6" t="s">
         <v>235</v>
       </c>
-      <c r="O28" s="3" t="s">
+      <c r="O28" s="6" t="s">
         <v>236</v>
       </c>
     </row>
-    <row r="29" spans="1:16" s="4" customFormat="1" ht="409.6">
-      <c r="A29" s="3" t="s">
+    <row r="29" spans="1:16" s="7" customFormat="1" ht="409.6">
+      <c r="A29" s="6" t="s">
         <v>45</v>
       </c>
-      <c r="B29" s="3" t="s">
+      <c r="B29" s="6" t="s">
         <v>237</v>
       </c>
-      <c r="C29" s="3" t="s">
+      <c r="C29" s="6" t="s">
         <v>238</v>
       </c>
-      <c r="D29" s="3" t="s">
+      <c r="D29" s="6" t="s">
         <v>239</v>
       </c>
-      <c r="E29" s="3" t="s">
+      <c r="E29" s="6" t="s">
         <v>240</v>
       </c>
-      <c r="F29" s="3" t="s">
+      <c r="F29" s="6" t="s">
         <v>241</v>
       </c>
-      <c r="G29" s="3" t="s">
+      <c r="G29" s="6" t="s">
         <v>242</v>
       </c>
-      <c r="H29" s="3" t="s">
+      <c r="H29" s="6" t="s">
         <v>243</v>
       </c>
-      <c r="I29" s="3" t="s">
+      <c r="I29" s="6" t="s">
         <v>244</v>
       </c>
-      <c r="J29" s="3" t="s">
+      <c r="J29" s="6" t="s">
         <v>245</v>
       </c>
-      <c r="K29" s="3" t="s">
+      <c r="K29" s="6" t="s">
         <v>246</v>
       </c>
-      <c r="L29" s="3" t="s">
+      <c r="L29" s="6" t="s">
         <v>247</v>
       </c>
-      <c r="M29" s="3" t="s">
+      <c r="M29" s="6" t="s">
         <v>248</v>
       </c>
-      <c r="N29" s="3" t="s">
+      <c r="N29" s="6" t="s">
         <v>249</v>
       </c>
-      <c r="O29" s="3" t="s">
+      <c r="O29" s="6" t="s">
         <v>250</v>
       </c>
-      <c r="P29" s="4" t="s">
+      <c r="P29" s="7" t="s">
         <v>251</v>
       </c>
     </row>
-    <row r="30" spans="1:16" s="4" customFormat="1" ht="250.8">
-      <c r="A30" s="3" t="s">
+    <row r="30" spans="1:16" s="7" customFormat="1" ht="250.8">
+      <c r="A30" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="B30" s="3" t="s">
+      <c r="B30" s="6" t="s">
         <v>262</v>
       </c>
-      <c r="C30" s="3" t="s">
+      <c r="C30" s="6" t="s">
         <v>263</v>
       </c>
-      <c r="D30" s="3" t="s">
+      <c r="D30" s="6" t="s">
         <v>264</v>
       </c>
-      <c r="E30" s="3" t="s">
+      <c r="E30" s="6" t="s">
         <v>265</v>
       </c>
-      <c r="F30" s="3" t="s">
+      <c r="F30" s="6" t="s">
         <v>266</v>
       </c>
-      <c r="G30" s="3" t="s">
+      <c r="G30" s="6" t="s">
         <v>267</v>
       </c>
-      <c r="H30" s="3" t="s">
+      <c r="H30" s="6" t="s">
         <v>275</v>
       </c>
-      <c r="I30" s="3" t="s">
+      <c r="I30" s="6" t="s">
         <v>268</v>
       </c>
-      <c r="J30" s="3" t="s">
+      <c r="J30" s="6" t="s">
         <v>269</v>
       </c>
-      <c r="K30" s="3" t="s">
+      <c r="K30" s="6" t="s">
         <v>270</v>
       </c>
-      <c r="L30" s="3" t="s">
+      <c r="L30" s="6" t="s">
         <v>271</v>
       </c>
-      <c r="M30" s="6" t="s">
+      <c r="M30" s="8" t="s">
         <v>364</v>
       </c>
-      <c r="N30" s="3" t="s">
+      <c r="N30" s="6" t="s">
         <v>272</v>
       </c>
-      <c r="O30" s="3" t="s">
+      <c r="O30" s="6" t="s">
         <v>274</v>
       </c>
-      <c r="P30" s="4" t="s">
+      <c r="P30" s="7" t="s">
         <v>273</v>
       </c>
     </row>
-    <row r="31" spans="1:16" s="4" customFormat="1" ht="132">
-      <c r="A31" s="3" t="s">
+    <row r="31" spans="1:16" s="7" customFormat="1" ht="132">
+      <c r="A31" s="6" t="s">
         <v>47</v>
       </c>
-      <c r="B31" s="3" t="s">
+      <c r="B31" s="6" t="s">
         <v>276</v>
       </c>
-      <c r="C31" s="3" t="s">
+      <c r="C31" s="6" t="s">
         <v>277</v>
       </c>
-      <c r="D31" s="3" t="s">
+      <c r="D31" s="6" t="s">
         <v>278</v>
       </c>
-      <c r="E31" s="7" t="s">
+      <c r="E31" s="9" t="s">
         <v>365</v>
       </c>
-      <c r="F31" s="3" t="s">
+      <c r="F31" s="6" t="s">
         <v>279</v>
       </c>
-      <c r="G31" s="3" t="s">
+      <c r="G31" s="6" t="s">
         <v>280</v>
       </c>
-      <c r="H31" s="3" t="s">
+      <c r="H31" s="6" t="s">
         <v>281</v>
       </c>
-      <c r="I31" s="3" t="s">
+      <c r="I31" s="6" t="s">
         <v>282</v>
       </c>
-      <c r="J31" s="3" t="s">
+      <c r="J31" s="6" t="s">
         <v>269</v>
       </c>
-      <c r="K31" s="3" t="s">
+      <c r="K31" s="6" t="s">
         <v>283</v>
       </c>
-      <c r="L31" s="3" t="s">
+      <c r="L31" s="6" t="s">
         <v>284</v>
       </c>
-      <c r="M31" s="3" t="s">
+      <c r="M31" s="6" t="s">
         <v>285</v>
       </c>
-      <c r="N31" s="3" t="s">
+      <c r="N31" s="6" t="s">
         <v>286</v>
       </c>
-      <c r="O31" s="3" t="s">
+      <c r="O31" s="6" t="s">
         <v>288</v>
       </c>
-      <c r="P31" s="3" t="s">
+      <c r="P31" s="6" t="s">
         <v>287</v>
       </c>
     </row>
-    <row r="32" spans="1:16" s="4" customFormat="1" ht="105.6">
-      <c r="A32" s="3" t="s">
+    <row r="32" spans="1:16" s="7" customFormat="1" ht="105.6">
+      <c r="A32" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="B32" s="3" t="s">
+      <c r="B32" s="6" t="s">
         <v>366</v>
       </c>
-      <c r="C32" s="3" t="s">
+      <c r="C32" s="6" t="s">
         <v>367</v>
       </c>
-      <c r="D32" s="3" t="s">
+      <c r="D32" s="6" t="s">
         <v>368</v>
       </c>
-      <c r="E32" s="3" t="s">
+      <c r="E32" s="6" t="s">
         <v>369</v>
       </c>
-      <c r="F32" s="3" t="s">
+      <c r="F32" s="6" t="s">
         <v>370</v>
       </c>
-      <c r="G32" s="3" t="s">
+      <c r="G32" s="6" t="s">
         <v>371</v>
       </c>
-      <c r="H32" s="3" t="s">
+      <c r="H32" s="6" t="s">
         <v>372</v>
       </c>
-      <c r="I32" s="3" t="s">
+      <c r="I32" s="6" t="s">
         <v>295</v>
       </c>
-      <c r="J32" s="3" t="s">
+      <c r="J32" s="6" t="s">
         <v>373</v>
       </c>
-      <c r="K32" s="3" t="s">
+      <c r="K32" s="6" t="s">
         <v>374</v>
       </c>
-      <c r="L32" s="3" t="s">
+      <c r="L32" s="6" t="s">
         <v>375</v>
       </c>
-      <c r="M32" s="3" t="s">
+      <c r="M32" s="6" t="s">
         <v>376</v>
       </c>
-      <c r="N32" s="3" t="s">
+      <c r="N32" s="6" t="s">
         <v>377</v>
       </c>
-      <c r="O32" s="3" t="s">
+      <c r="O32" s="6" t="s">
         <v>378</v>
       </c>
-      <c r="P32" s="4" t="s">
+      <c r="P32" s="7" t="s">
         <v>379</v>
       </c>
     </row>
-    <row r="33" spans="1:16" s="4" customFormat="1" ht="290.39999999999998">
-      <c r="A33" s="3" t="s">
+    <row r="33" spans="1:16" s="7" customFormat="1" ht="290.39999999999998">
+      <c r="A33" s="6" t="s">
         <v>49</v>
       </c>
-      <c r="B33" s="3" t="s">
+      <c r="B33" s="6" t="s">
         <v>252</v>
       </c>
-      <c r="C33" s="3" t="s">
+      <c r="C33" s="6" t="s">
         <v>253</v>
       </c>
-      <c r="D33" s="3" t="s">
+      <c r="D33" s="6" t="s">
         <v>254</v>
       </c>
-      <c r="E33" s="3" t="s">
+      <c r="E33" s="6" t="s">
         <v>78</v>
       </c>
-      <c r="F33" s="3" t="s">
+      <c r="F33" s="6" t="s">
         <v>255</v>
       </c>
-      <c r="G33" s="3" t="s">
+      <c r="G33" s="6" t="s">
         <v>212</v>
       </c>
-      <c r="H33" s="3" t="s">
+      <c r="H33" s="6" t="s">
         <v>256</v>
       </c>
-      <c r="I33" s="3" t="s">
+      <c r="I33" s="6" t="s">
         <v>257</v>
       </c>
-      <c r="J33" s="3" t="s">
+      <c r="J33" s="6" t="s">
         <v>258</v>
       </c>
-      <c r="K33" s="3" t="s">
+      <c r="K33" s="6" t="s">
         <v>259</v>
       </c>
-      <c r="L33" s="3" t="s">
+      <c r="L33" s="6" t="s">
         <v>212</v>
       </c>
-      <c r="M33" s="3" t="s">
+      <c r="M33" s="6" t="s">
         <v>260</v>
       </c>
-      <c r="N33" s="3" t="s">
+      <c r="N33" s="6" t="s">
         <v>261</v>
       </c>
-      <c r="O33" s="3"/>
+      <c r="O33" s="6"/>
     </row>
-    <row r="34" spans="1:16" s="4" customFormat="1" ht="120" customHeight="1">
-      <c r="A34" s="3" t="s">
+    <row r="34" spans="1:16" s="7" customFormat="1" ht="120" customHeight="1">
+      <c r="A34" s="6" t="s">
         <v>50</v>
       </c>
-      <c r="B34" s="3" t="s">
+      <c r="B34" s="6" t="s">
         <v>395</v>
       </c>
-      <c r="C34" s="3" t="s">
+      <c r="C34" s="6" t="s">
         <v>396</v>
       </c>
-      <c r="D34" s="3" t="s">
+      <c r="D34" s="6" t="s">
         <v>397</v>
       </c>
-      <c r="E34" s="3" t="s">
+      <c r="E34" s="6" t="s">
         <v>397</v>
       </c>
-      <c r="F34" s="3" t="s">
+      <c r="F34" s="6" t="s">
         <v>85</v>
       </c>
-      <c r="G34" s="3" t="s">
+      <c r="G34" s="6" t="s">
         <v>399</v>
       </c>
-      <c r="H34" s="3" t="s">
+      <c r="H34" s="6" t="s">
         <v>385</v>
       </c>
-      <c r="I34" s="3" t="s">
+      <c r="I34" s="6" t="s">
         <v>400</v>
       </c>
-      <c r="J34" s="3" t="s">
+      <c r="J34" s="6" t="s">
         <v>401</v>
       </c>
-      <c r="K34" s="3" t="s">
+      <c r="K34" s="6" t="s">
         <v>402</v>
       </c>
-      <c r="L34" s="3" t="s">
+      <c r="L34" s="6" t="s">
         <v>403</v>
       </c>
-      <c r="M34" s="3" t="s">
+      <c r="M34" s="6" t="s">
         <v>404</v>
       </c>
-      <c r="N34" s="3" t="s">
+      <c r="N34" s="6" t="s">
         <v>405</v>
       </c>
-      <c r="O34" s="3" t="s">
+      <c r="O34" s="6" t="s">
         <v>406</v>
       </c>
-      <c r="P34" s="4" t="s">
+      <c r="P34" s="7" t="s">
         <v>407</v>
       </c>
     </row>
-    <row r="35" spans="1:16" s="4" customFormat="1" ht="79.2">
-      <c r="A35" s="3" t="s">
+    <row r="35" spans="1:16" s="7" customFormat="1" ht="79.2">
+      <c r="A35" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="B35" s="3" t="s">
+      <c r="B35" s="6" t="s">
         <v>408</v>
       </c>
-      <c r="C35" s="3" t="s">
+      <c r="C35" s="6" t="s">
         <v>409</v>
       </c>
-      <c r="D35" s="3" t="s">
+      <c r="D35" s="6" t="s">
         <v>410</v>
       </c>
       <c r="E35" s="10" t="s">
         <v>318</v>
       </c>
-      <c r="F35" s="3" t="s">
+      <c r="F35" s="6" t="s">
         <v>411</v>
       </c>
-      <c r="G35" s="3" t="s">
+      <c r="G35" s="6" t="s">
         <v>398</v>
       </c>
-      <c r="H35" s="3" t="s">
+      <c r="H35" s="6" t="s">
         <v>412</v>
       </c>
-      <c r="I35" s="3" t="s">
+      <c r="I35" s="6" t="s">
         <v>413</v>
       </c>
-      <c r="J35" s="3" t="s">
+      <c r="J35" s="6" t="s">
         <v>414</v>
       </c>
-      <c r="K35" s="3" t="s">
+      <c r="K35" s="6" t="s">
         <v>402</v>
       </c>
-      <c r="L35" s="3" t="s">
+      <c r="L35" s="6" t="s">
         <v>269</v>
       </c>
-      <c r="M35" s="3" t="s">
+      <c r="M35" s="6" t="s">
         <v>415</v>
       </c>
-      <c r="N35" s="3" t="s">
+      <c r="N35" s="6" t="s">
         <v>416</v>
       </c>
-      <c r="O35" s="3" t="s">
+      <c r="O35" s="6" t="s">
         <v>417</v>
       </c>
-      <c r="P35" s="4" t="s">
+      <c r="P35" s="7" t="s">
         <v>418</v>
       </c>
     </row>
-    <row r="36" spans="1:16" s="4" customFormat="1" ht="92.4">
-      <c r="A36" s="3" t="s">
+    <row r="36" spans="1:16" s="7" customFormat="1" ht="92.4">
+      <c r="A36" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="B36" s="3" t="s">
+      <c r="B36" s="6" t="s">
         <v>419</v>
       </c>
-      <c r="C36" s="3" t="s">
+      <c r="C36" s="6" t="s">
         <v>420</v>
       </c>
-      <c r="D36" s="3" t="s">
+      <c r="D36" s="6" t="s">
         <v>421</v>
       </c>
-      <c r="E36" s="3" t="s">
+      <c r="E36" s="6" t="s">
         <v>422</v>
       </c>
-      <c r="F36" s="3" t="s">
+      <c r="F36" s="6" t="s">
         <v>411</v>
       </c>
-      <c r="G36" s="3" t="s">
+      <c r="G36" s="6" t="s">
         <v>398</v>
       </c>
-      <c r="H36" s="3" t="s">
+      <c r="H36" s="6" t="s">
         <v>423</v>
       </c>
-      <c r="I36" s="3" t="s">
+      <c r="I36" s="6" t="s">
         <v>257</v>
       </c>
-      <c r="J36" s="3" t="s">
+      <c r="J36" s="6" t="s">
         <v>424</v>
       </c>
-      <c r="K36" s="3" t="s">
+      <c r="K36" s="6" t="s">
         <v>402</v>
       </c>
-      <c r="L36" s="3" t="s">
+      <c r="L36" s="6" t="s">
         <v>425</v>
       </c>
-      <c r="M36" s="3" t="s">
+      <c r="M36" s="6" t="s">
         <v>426</v>
       </c>
-      <c r="N36" s="3" t="s">
+      <c r="N36" s="6" t="s">
         <v>427</v>
       </c>
-      <c r="O36" s="3" t="s">
+      <c r="O36" s="6" t="s">
         <v>428</v>
       </c>
-      <c r="P36" s="4" t="s">
+      <c r="P36" s="7" t="s">
         <v>429</v>
       </c>
     </row>
-    <row r="37" spans="1:16" s="4" customFormat="1" ht="79.2">
-      <c r="A37" s="3" t="s">
+    <row r="37" spans="1:16" s="7" customFormat="1" ht="79.2">
+      <c r="A37" s="6" t="s">
         <v>53</v>
       </c>
-      <c r="B37" s="3" t="s">
+      <c r="B37" s="6" t="s">
         <v>430</v>
       </c>
-      <c r="C37" s="3" t="s">
+      <c r="C37" s="6" t="s">
         <v>431</v>
       </c>
-      <c r="D37" s="3" t="s">
+      <c r="D37" s="6" t="s">
         <v>432</v>
       </c>
-      <c r="E37" s="3" t="s">
+      <c r="E37" s="6" t="s">
         <v>397</v>
       </c>
-      <c r="F37" s="3" t="s">
+      <c r="F37" s="6" t="s">
         <v>434</v>
       </c>
-      <c r="G37" s="3" t="s">
+      <c r="G37" s="6" t="s">
         <v>433</v>
       </c>
-      <c r="H37" s="3" t="s">
+      <c r="H37" s="6" t="s">
         <v>333</v>
       </c>
-      <c r="I37" s="3" t="s">
+      <c r="I37" s="6" t="s">
         <v>435</v>
       </c>
-      <c r="J37" s="3" t="s">
+      <c r="J37" s="6" t="s">
         <v>436</v>
       </c>
-      <c r="K37" s="3" t="s">
+      <c r="K37" s="6" t="s">
         <v>437</v>
       </c>
-      <c r="L37" s="3" t="s">
+      <c r="L37" s="6" t="s">
         <v>438</v>
       </c>
-      <c r="M37" s="3" t="s">
+      <c r="M37" s="6" t="s">
         <v>439</v>
       </c>
-      <c r="N37" s="3" t="s">
+      <c r="N37" s="6" t="s">
         <v>440</v>
       </c>
-      <c r="O37" s="3" t="s">
+      <c r="O37" s="6" t="s">
         <v>441</v>
       </c>
-      <c r="P37" s="4" t="s">
+      <c r="P37" s="7" t="s">
         <v>442</v>
       </c>
     </row>
-    <row r="38" spans="1:16" s="9" customFormat="1">
-      <c r="A38" s="8" t="s">
+    <row r="38" spans="1:16" s="7" customFormat="1">
+      <c r="A38" s="6" t="s">
         <v>54</v>
       </c>
-      <c r="B38" s="8" t="s">
+      <c r="B38" s="6" t="s">
         <v>66</v>
       </c>
-      <c r="C38" s="8" t="s">
+      <c r="C38" s="6" t="s">
         <v>66</v>
       </c>
-      <c r="D38" s="8" t="s">
+      <c r="D38" s="6" t="s">
         <v>66</v>
       </c>
-      <c r="E38" s="8" t="s">
+      <c r="E38" s="6" t="s">
         <v>66</v>
       </c>
-      <c r="F38" s="8" t="s">
+      <c r="F38" s="6" t="s">
         <v>66</v>
       </c>
-      <c r="G38" s="8" t="s">
+      <c r="G38" s="6" t="s">
         <v>66</v>
       </c>
-      <c r="H38" s="8" t="s">
+      <c r="H38" s="6" t="s">
         <v>66</v>
       </c>
-      <c r="I38" s="8" t="s">
+      <c r="I38" s="6" t="s">
         <v>66</v>
       </c>
-      <c r="J38" s="8" t="s">
+      <c r="J38" s="6" t="s">
         <v>66</v>
       </c>
-      <c r="K38" s="8" t="s">
+      <c r="K38" s="6" t="s">
         <v>66</v>
       </c>
-      <c r="L38" s="8" t="s">
+      <c r="L38" s="6" t="s">
         <v>66</v>
       </c>
-      <c r="M38" s="8" t="s">
+      <c r="M38" s="6" t="s">
         <v>66</v>
       </c>
-      <c r="N38" s="8"/>
-      <c r="O38" s="8" t="s">
+      <c r="N38" s="6"/>
+      <c r="O38" s="6" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="39" spans="1:16" s="4" customFormat="1" ht="132">
-      <c r="A39" s="3" t="s">
+    <row r="39" spans="1:16" s="7" customFormat="1" ht="132">
+      <c r="A39" s="6" t="s">
         <v>55</v>
       </c>
-      <c r="B39" s="3" t="s">
+      <c r="B39" s="6" t="s">
         <v>443</v>
       </c>
-      <c r="C39" s="3" t="s">
+      <c r="C39" s="6" t="s">
         <v>444</v>
       </c>
-      <c r="D39" s="3" t="s">
+      <c r="D39" s="6" t="s">
         <v>445</v>
       </c>
-      <c r="E39" s="3" t="s">
+      <c r="E39" s="6" t="s">
         <v>446</v>
       </c>
-      <c r="F39" s="3" t="s">
+      <c r="F39" s="6" t="s">
         <v>447</v>
       </c>
-      <c r="G39" s="3" t="s">
+      <c r="G39" s="6" t="s">
         <v>398</v>
       </c>
-      <c r="H39" s="3" t="s">
+      <c r="H39" s="6" t="s">
         <v>448</v>
       </c>
-      <c r="I39" s="3" t="s">
+      <c r="I39" s="6" t="s">
         <v>68</v>
       </c>
-      <c r="J39" s="3" t="s">
+      <c r="J39" s="6" t="s">
         <v>445</v>
       </c>
-      <c r="K39" s="3" t="s">
+      <c r="K39" s="6" t="s">
         <v>402</v>
       </c>
-      <c r="L39" s="3" t="s">
+      <c r="L39" s="6" t="s">
         <v>449</v>
       </c>
-      <c r="M39" s="3" t="s">
+      <c r="M39" s="6" t="s">
         <v>450</v>
       </c>
-      <c r="N39" s="3" t="s">
+      <c r="N39" s="6" t="s">
         <v>427</v>
       </c>
-      <c r="O39" s="3" t="s">
+      <c r="O39" s="6" t="s">
         <v>451</v>
       </c>
-      <c r="P39" s="4" t="s">
+      <c r="P39" s="7" t="s">
         <v>452</v>
       </c>
     </row>
-    <row r="40" spans="1:16" s="4" customFormat="1" ht="132">
-      <c r="A40" s="3" t="s">
+    <row r="40" spans="1:16" s="7" customFormat="1" ht="132">
+      <c r="A40" s="6" t="s">
         <v>56</v>
       </c>
-      <c r="B40" s="3" t="s">
+      <c r="B40" s="6" t="s">
         <v>453</v>
       </c>
-      <c r="C40" s="3" t="s">
+      <c r="C40" s="6" t="s">
         <v>455</v>
       </c>
-      <c r="D40" s="3" t="s">
+      <c r="D40" s="6" t="s">
         <v>454</v>
       </c>
-      <c r="E40" s="3" t="s">
+      <c r="E40" s="6" t="s">
         <v>456</v>
       </c>
-      <c r="F40" s="3" t="s">
+      <c r="F40" s="6" t="s">
         <v>447</v>
       </c>
-      <c r="G40" s="3" t="s">
+      <c r="G40" s="6" t="s">
         <v>398</v>
       </c>
-      <c r="H40" s="3" t="s">
+      <c r="H40" s="6" t="s">
         <v>333</v>
       </c>
-      <c r="I40" s="3" t="s">
+      <c r="I40" s="6" t="s">
         <v>68</v>
       </c>
-      <c r="J40" s="3" t="s">
+      <c r="J40" s="6" t="s">
         <v>457</v>
       </c>
-      <c r="K40" s="3" t="s">
+      <c r="K40" s="6" t="s">
         <v>402</v>
       </c>
-      <c r="L40" s="3" t="s">
+      <c r="L40" s="6" t="s">
         <v>449</v>
       </c>
-      <c r="M40" s="3" t="s">
+      <c r="M40" s="6" t="s">
         <v>439</v>
       </c>
-      <c r="N40" s="3" t="s">
+      <c r="N40" s="6" t="s">
         <v>427</v>
       </c>
-      <c r="O40" s="3" t="s">
+      <c r="O40" s="6" t="s">
         <v>458</v>
       </c>
-      <c r="P40" s="4" t="s">
+      <c r="P40" s="7" t="s">
         <v>459</v>
       </c>
     </row>
-    <row r="41" spans="1:16" s="4" customFormat="1" ht="145.19999999999999">
-      <c r="A41" s="3" t="s">
+    <row r="41" spans="1:16" s="7" customFormat="1" ht="145.19999999999999">
+      <c r="A41" s="6" t="s">
         <v>57</v>
       </c>
-      <c r="B41" s="3" t="s">
+      <c r="B41" s="6" t="s">
         <v>460</v>
       </c>
-      <c r="C41" s="3" t="s">
+      <c r="C41" s="6" t="s">
         <v>461</v>
       </c>
-      <c r="D41" s="3" t="s">
+      <c r="D41" s="6" t="s">
         <v>463</v>
       </c>
-      <c r="E41" s="3" t="s">
+      <c r="E41" s="6" t="s">
         <v>462</v>
       </c>
-      <c r="F41" s="3" t="s">
+      <c r="F41" s="6" t="s">
         <v>464</v>
       </c>
-      <c r="G41" s="3" t="s">
+      <c r="G41" s="6" t="s">
         <v>398</v>
       </c>
-      <c r="H41" s="3" t="s">
+      <c r="H41" s="6" t="s">
         <v>333</v>
       </c>
-      <c r="I41" s="3" t="s">
+      <c r="I41" s="6" t="s">
         <v>465</v>
       </c>
-      <c r="J41" s="3" t="s">
+      <c r="J41" s="6" t="s">
         <v>466</v>
       </c>
-      <c r="K41" s="3" t="s">
+      <c r="K41" s="6" t="s">
         <v>402</v>
       </c>
-      <c r="L41" s="3" t="s">
+      <c r="L41" s="6" t="s">
         <v>467</v>
       </c>
-      <c r="M41" s="3" t="s">
+      <c r="M41" s="6" t="s">
         <v>468</v>
       </c>
-      <c r="N41" s="3" t="s">
+      <c r="N41" s="6" t="s">
         <v>469</v>
       </c>
-      <c r="O41" s="3" t="s">
+      <c r="O41" s="6" t="s">
         <v>470</v>
       </c>
-      <c r="P41" s="4" t="s">
+      <c r="P41" s="7" t="s">
         <v>471</v>
       </c>
     </row>
-    <row r="42" spans="1:16" s="4" customFormat="1" ht="118.8">
-      <c r="A42" s="3" t="s">
+    <row r="42" spans="1:16" s="7" customFormat="1" ht="118.8">
+      <c r="A42" s="6" t="s">
         <v>58</v>
       </c>
-      <c r="B42" s="3" t="s">
+      <c r="B42" s="6" t="s">
         <v>472</v>
       </c>
-      <c r="C42" s="3" t="s">
+      <c r="C42" s="6" t="s">
         <v>473</v>
       </c>
-      <c r="D42" s="3" t="s">
+      <c r="D42" s="6" t="s">
         <v>474</v>
       </c>
-      <c r="E42" s="3" t="s">
+      <c r="E42" s="6" t="s">
         <v>456</v>
       </c>
-      <c r="F42" s="3" t="s">
+      <c r="F42" s="6" t="s">
         <v>447</v>
       </c>
-      <c r="G42" s="3" t="s">
+      <c r="G42" s="6" t="s">
         <v>398</v>
       </c>
-      <c r="H42" s="3" t="s">
+      <c r="H42" s="6" t="s">
         <v>448</v>
       </c>
-      <c r="I42" s="3" t="s">
+      <c r="I42" s="6" t="s">
         <v>475</v>
       </c>
-      <c r="J42" s="3" t="s">
+      <c r="J42" s="6" t="s">
         <v>373</v>
       </c>
-      <c r="K42" s="3" t="s">
+      <c r="K42" s="6" t="s">
         <v>402</v>
       </c>
-      <c r="L42" s="3" t="s">
+      <c r="L42" s="6" t="s">
         <v>449</v>
       </c>
-      <c r="M42" s="3" t="s">
+      <c r="M42" s="6" t="s">
         <v>476</v>
       </c>
-      <c r="N42" s="3" t="s">
+      <c r="N42" s="6" t="s">
         <v>477</v>
       </c>
-      <c r="O42" s="3" t="s">
+      <c r="O42" s="6" t="s">
         <v>478</v>
       </c>
-      <c r="P42" s="4" t="s">
+      <c r="P42" s="7" t="s">
         <v>479</v>
       </c>
     </row>
-    <row r="43" spans="1:16" s="4" customFormat="1" ht="145.19999999999999">
-      <c r="A43" s="3" t="s">
+    <row r="43" spans="1:16" s="7" customFormat="1" ht="145.19999999999999">
+      <c r="A43" s="6" t="s">
         <v>59</v>
       </c>
-      <c r="B43" s="3" t="s">
+      <c r="B43" s="6" t="s">
         <v>480</v>
       </c>
-      <c r="C43" s="3" t="s">
+      <c r="C43" s="6" t="s">
         <v>481</v>
       </c>
-      <c r="D43" s="3" t="s">
+      <c r="D43" s="6" t="s">
         <v>482</v>
       </c>
-      <c r="E43" s="3" t="s">
+      <c r="E43" s="6" t="s">
         <v>446</v>
       </c>
-      <c r="F43" s="3" t="s">
+      <c r="F43" s="6" t="s">
         <v>447</v>
       </c>
-      <c r="G43" s="3" t="s">
+      <c r="G43" s="6" t="s">
         <v>446</v>
       </c>
-      <c r="H43" s="3" t="s">
+      <c r="H43" s="6" t="s">
         <v>412</v>
       </c>
-      <c r="I43" s="3" t="s">
+      <c r="I43" s="6" t="s">
         <v>475</v>
       </c>
-      <c r="J43" s="3" t="s">
+      <c r="J43" s="6" t="s">
         <v>483</v>
       </c>
-      <c r="K43" s="3" t="s">
+      <c r="K43" s="6" t="s">
         <v>402</v>
       </c>
-      <c r="L43" s="3" t="s">
+      <c r="L43" s="6" t="s">
         <v>484</v>
       </c>
-      <c r="M43" s="3" t="s">
+      <c r="M43" s="6" t="s">
         <v>485</v>
       </c>
-      <c r="N43" s="3" t="s">
+      <c r="N43" s="6" t="s">
         <v>486</v>
       </c>
-      <c r="O43" s="3" t="s">
+      <c r="O43" s="6" t="s">
         <v>487</v>
       </c>
-      <c r="P43" s="4" t="s">
+      <c r="P43" s="7" t="s">
         <v>488</v>
       </c>
     </row>
-    <row r="44" spans="1:16" s="4" customFormat="1" ht="145.19999999999999">
-      <c r="A44" s="3" t="s">
+    <row r="44" spans="1:16" s="7" customFormat="1" ht="145.19999999999999">
+      <c r="A44" s="6" t="s">
         <v>60</v>
       </c>
-      <c r="B44" s="3" t="s">
+      <c r="B44" s="6" t="s">
         <v>489</v>
       </c>
-      <c r="C44" s="3" t="s">
+      <c r="C44" s="6" t="s">
         <v>490</v>
       </c>
-      <c r="D44" s="3" t="s">
+      <c r="D44" s="6" t="s">
         <v>491</v>
       </c>
-      <c r="E44" s="3" t="s">
+      <c r="E44" s="6" t="s">
         <v>369</v>
       </c>
-      <c r="F44" s="3" t="s">
+      <c r="F44" s="6" t="s">
         <v>447</v>
       </c>
-      <c r="G44" s="3" t="s">
+      <c r="G44" s="6" t="s">
         <v>369</v>
       </c>
-      <c r="H44" s="3" t="s">
+      <c r="H44" s="6" t="s">
         <v>412</v>
       </c>
-      <c r="I44" s="3" t="s">
+      <c r="I44" s="6" t="s">
         <v>475</v>
       </c>
-      <c r="J44" s="3" t="s">
+      <c r="J44" s="6" t="s">
         <v>492</v>
       </c>
-      <c r="K44" s="3" t="s">
+      <c r="K44" s="6" t="s">
         <v>402</v>
       </c>
-      <c r="L44" s="3" t="s">
+      <c r="L44" s="6" t="s">
         <v>493</v>
       </c>
-      <c r="M44" s="3" t="s">
+      <c r="M44" s="6" t="s">
         <v>494</v>
       </c>
-      <c r="N44" s="3" t="s">
+      <c r="N44" s="6" t="s">
         <v>495</v>
       </c>
-      <c r="O44" s="3" t="s">
+      <c r="O44" s="6" t="s">
         <v>496</v>
       </c>
-      <c r="P44" s="4" t="s">
+      <c r="P44" s="7" t="s">
         <v>497</v>
       </c>
     </row>
-    <row r="45" spans="1:16" s="4" customFormat="1" ht="171.6">
-      <c r="A45" s="3" t="s">
+    <row r="45" spans="1:16" s="7" customFormat="1" ht="171.6">
+      <c r="A45" s="6" t="s">
         <v>61</v>
       </c>
-      <c r="B45" s="3" t="s">
+      <c r="B45" s="6" t="s">
         <v>498</v>
       </c>
-      <c r="C45" s="3" t="s">
+      <c r="C45" s="6" t="s">
         <v>499</v>
       </c>
-      <c r="D45" s="3" t="s">
+      <c r="D45" s="6" t="s">
         <v>508</v>
       </c>
-      <c r="E45" s="3" t="s">
+      <c r="E45" s="6" t="s">
         <v>369</v>
       </c>
-      <c r="F45" s="3" t="s">
+      <c r="F45" s="6" t="s">
         <v>500</v>
       </c>
-      <c r="G45" s="3" t="s">
+      <c r="G45" s="6" t="s">
         <v>398</v>
       </c>
-      <c r="H45" s="3" t="s">
+      <c r="H45" s="6" t="s">
         <v>412</v>
       </c>
-      <c r="I45" s="3" t="s">
+      <c r="I45" s="6" t="s">
         <v>475</v>
       </c>
-      <c r="J45" s="3" t="s">
+      <c r="J45" s="6" t="s">
         <v>501</v>
       </c>
-      <c r="K45" s="3" t="s">
+      <c r="K45" s="6" t="s">
         <v>502</v>
       </c>
-      <c r="L45" s="3" t="s">
+      <c r="L45" s="6" t="s">
         <v>503</v>
       </c>
-      <c r="M45" s="3" t="s">
+      <c r="M45" s="6" t="s">
         <v>504</v>
       </c>
-      <c r="N45" s="3" t="s">
+      <c r="N45" s="6" t="s">
         <v>505</v>
       </c>
-      <c r="O45" s="3" t="s">
+      <c r="O45" s="6" t="s">
         <v>506</v>
       </c>
-      <c r="P45" s="4" t="s">
+      <c r="P45" s="7" t="s">
         <v>507</v>
       </c>
     </row>
-    <row r="46" spans="1:16">
+    <row r="46" spans="1:16" ht="145.19999999999999">
       <c r="A46" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="B46" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="C46" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="D46" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="E46" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="F46" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="G46" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="H46" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="I46" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="J46" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="K46" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="L46" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="M46" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="N46" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="O46" s="1" t="s">
-        <v>66</v>
+      <c r="B46" s="6" t="s">
+        <v>480</v>
+      </c>
+      <c r="C46" s="6" t="s">
+        <v>481</v>
+      </c>
+      <c r="D46" s="6" t="s">
+        <v>482</v>
+      </c>
+      <c r="E46" s="6" t="s">
+        <v>446</v>
+      </c>
+      <c r="F46" s="6" t="s">
+        <v>447</v>
+      </c>
+      <c r="G46" s="6" t="s">
+        <v>446</v>
+      </c>
+      <c r="H46" s="6" t="s">
+        <v>412</v>
+      </c>
+      <c r="I46" s="6" t="s">
+        <v>475</v>
+      </c>
+      <c r="J46" s="6" t="s">
+        <v>483</v>
+      </c>
+      <c r="K46" s="6" t="s">
+        <v>402</v>
+      </c>
+      <c r="L46" s="6" t="s">
+        <v>484</v>
+      </c>
+      <c r="M46" s="6" t="s">
+        <v>485</v>
+      </c>
+      <c r="N46" s="6" t="s">
+        <v>486</v>
+      </c>
+      <c r="O46" s="6" t="s">
+        <v>487</v>
+      </c>
+      <c r="P46" s="7" t="s">
+        <v>488</v>
       </c>
     </row>
   </sheetData>
@@ -4557,6 +4542,12 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x01010009048CEEA230F14796749F6DFD5F5263" ma:contentTypeVersion="4" ma:contentTypeDescription="Crear nuevo documento." ma:contentTypeScope="" ma:versionID="5105af4e7c1b0ed6cdb04338eaf51f7a">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="96457c7a-bdfc-427e-9d05-5faa5ab5244b" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="0baee1a300280ca08e7397f1756276d6" ns2:_="">
     <xsd:import namespace="96457c7a-bdfc-427e-9d05-5faa5ab5244b"/>
@@ -4700,12 +4691,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
@@ -4716,6 +4701,15 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1160EB8C-E200-4916-A3B3-9BF8115D37F8}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{75ADFBF6-8C74-4292-833E-68A026E87063}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -4733,15 +4727,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1160EB8C-E200-4916-A3B3-9BF8115D37F8}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{24F2579D-323E-48EA-8FED-D372AFFF0A04}">
   <ds:schemaRefs>

</xml_diff>